<commit_message>
todos los ataqes de armas y alguna modificación más
</commit_message>
<xml_diff>
--- a/arquetiposZ.xlsx
+++ b/arquetiposZ.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sergius\Desktop\Proyectos\hyperbole\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88D25541-0494-46D1-A64A-CE4D6CF4D7CF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95C91E45-437D-4B7A-91B7-13D0EEF7DBA6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="644" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="644" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RESUMEN" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1149" uniqueCount="794">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1151" uniqueCount="801">
   <si>
     <t>daños:</t>
   </si>
@@ -1143,15 +1143,6 @@
   </si>
   <si>
     <t>[katana 6]</t>
-  </si>
-  <si>
-    <t>[ballesta 3 back desesp]</t>
-  </si>
-  <si>
-    <t>[arco 5]</t>
-  </si>
-  <si>
-    <t>[ballesta 4]</t>
   </si>
   <si>
     <t>[arco+ballesta]</t>
@@ -1897,21 +1888,9 @@
     <t>[maza 5 + armaduras metálicas]</t>
   </si>
   <si>
-    <t>[maza 5 + plantas, volcanicos, abisales]</t>
-  </si>
-  <si>
     <t>objetos curativos x1'5</t>
   </si>
   <si>
-    <t>resistir quemadura</t>
-  </si>
-  <si>
-    <t>resistir congelacion</t>
-  </si>
-  <si>
-    <t>resistir parálisis</t>
-  </si>
-  <si>
     <t>elegant dancing</t>
   </si>
   <si>
@@ -2426,6 +2405,48 @@
   </si>
   <si>
     <t>life wall</t>
+  </si>
+  <si>
+    <t>[maza 5 + elems, animales, bestias]</t>
+  </si>
+  <si>
+    <t>[katana 7]</t>
+  </si>
+  <si>
+    <t>[espada 6]</t>
+  </si>
+  <si>
+    <t>[martillo 7]</t>
+  </si>
+  <si>
+    <t>[arco 6]</t>
+  </si>
+  <si>
+    <t>[ballesta 7]</t>
+  </si>
+  <si>
+    <t>resistir quemadura/congelacion</t>
+  </si>
+  <si>
+    <t>resistir paralisis/mareo</t>
+  </si>
+  <si>
+    <t>resistir veneno/amnesia</t>
+  </si>
+  <si>
+    <t>+10% precision</t>
+  </si>
+  <si>
+    <t>resistir sueño/furia</t>
+  </si>
+  <si>
+    <t>[ballesta 3 back confusión]</t>
+  </si>
+  <si>
+    <t>hex shot</t>
+  </si>
+  <si>
+    <t>wild salvo</t>
   </si>
 </sst>
 </file>
@@ -3529,7 +3550,7 @@
       <c r="J4" s="50"/>
       <c r="K4" s="50"/>
       <c r="L4" s="49" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="M4" s="50"/>
       <c r="N4" s="50"/>
@@ -3564,7 +3585,7 @@
     <row r="6" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B6" s="12"/>
       <c r="C6" s="52" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>1</v>
@@ -3678,7 +3699,7 @@
     <row r="10" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B10" s="12"/>
       <c r="C10" s="53" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>4</v>
@@ -3829,7 +3850,7 @@
     <row r="15" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B15" s="12"/>
       <c r="C15" s="53" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>300</v>
@@ -3980,7 +4001,7 @@
     <row r="20" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="12"/>
       <c r="C20" s="43" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="D20" s="45"/>
       <c r="E20" s="5"/>
@@ -4024,7 +4045,7 @@
         <v>34</v>
       </c>
       <c r="L21" s="5" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="M21" s="5"/>
       <c r="N21" s="5"/>
@@ -4067,7 +4088,7 @@
     <row r="23" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B23" s="12"/>
       <c r="C23" s="49" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="D23" s="50"/>
       <c r="E23" s="51"/>
@@ -4107,7 +4128,7 @@
         <v>48</v>
       </c>
       <c r="L24" s="5" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="M24" s="5"/>
       <c r="N24" s="5"/>
@@ -4121,7 +4142,7 @@
     <row r="25" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B25" s="12"/>
       <c r="C25" s="1" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="D25" s="5"/>
       <c r="E25" s="2"/>
@@ -4148,7 +4169,7 @@
     <row r="26" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B26" s="12"/>
       <c r="C26" s="1" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="D26" s="5"/>
       <c r="E26" s="2"/>
@@ -4165,7 +4186,7 @@
         <v>43</v>
       </c>
       <c r="L26" s="5" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="M26" s="5"/>
       <c r="N26" s="5"/>
@@ -4179,7 +4200,7 @@
     <row r="27" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B27" s="12"/>
       <c r="C27" s="1" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="D27" s="5"/>
       <c r="E27" s="2"/>
@@ -4206,7 +4227,7 @@
     <row r="28" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B28" s="12"/>
       <c r="C28" s="1" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="D28" s="5"/>
       <c r="E28" s="2"/>
@@ -4235,7 +4256,7 @@
     <row r="29" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B29" s="12"/>
       <c r="C29" s="1" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="D29" s="5"/>
       <c r="E29" s="2"/>
@@ -4262,7 +4283,7 @@
     <row r="30" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B30" s="12"/>
       <c r="C30" s="1" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="D30" s="5"/>
       <c r="E30" s="2"/>
@@ -4293,7 +4314,7 @@
     <row r="31" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B31" s="12"/>
       <c r="C31" s="1" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="D31" s="5"/>
       <c r="E31" s="2"/>
@@ -4310,7 +4331,7 @@
         <v>54</v>
       </c>
       <c r="L31" s="5" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
       <c r="M31" s="5"/>
       <c r="N31" s="5"/>
@@ -4324,7 +4345,7 @@
     <row r="32" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B32" s="12"/>
       <c r="C32" s="1" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="D32" s="5"/>
       <c r="E32" s="2"/>
@@ -4337,7 +4358,7 @@
         <v>55</v>
       </c>
       <c r="L32" s="5" t="s">
-        <v>593</v>
+        <v>590</v>
       </c>
       <c r="M32" s="5"/>
       <c r="N32" s="5"/>
@@ -4351,7 +4372,7 @@
     <row r="33" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B33" s="12"/>
       <c r="C33" s="1" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="D33" s="5"/>
       <c r="E33" s="2"/>
@@ -4360,13 +4381,13 @@
       <c r="H33" s="5"/>
       <c r="I33" s="1"/>
       <c r="J33" s="5" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="K33" s="5" t="s">
         <v>66</v>
       </c>
       <c r="L33" s="5" t="s">
-        <v>592</v>
+        <v>589</v>
       </c>
       <c r="M33" s="5"/>
       <c r="N33" s="5"/>
@@ -4380,7 +4401,7 @@
     <row r="34" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B34" s="12"/>
       <c r="C34" s="6" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="D34" s="7"/>
       <c r="E34" s="8"/>
@@ -4397,7 +4418,7 @@
         <v>58</v>
       </c>
       <c r="L34" s="5" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="M34" s="5"/>
       <c r="N34" s="5"/>
@@ -4422,7 +4443,7 @@
         <v>61</v>
       </c>
       <c r="L35" s="7" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="M35" s="7"/>
       <c r="N35" s="7"/>
@@ -4436,7 +4457,7 @@
     <row r="36" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B36" s="12"/>
       <c r="C36" s="40" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="D36" s="41"/>
       <c r="E36" s="42"/>
@@ -4505,7 +4526,7 @@
       <c r="E39" s="48"/>
       <c r="F39" s="5"/>
       <c r="G39" s="49" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="H39" s="50"/>
       <c r="I39" s="50"/>
@@ -4586,19 +4607,19 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="J7">
         <v>1</v>
       </c>
       <c r="K7" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.25">
@@ -4606,19 +4627,19 @@
         <v>4</v>
       </c>
       <c r="C8" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="F8">
         <v>2</v>
       </c>
       <c r="G8" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="J8">
         <v>5</v>
       </c>
       <c r="K8" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.25">
@@ -4626,19 +4647,19 @@
         <v>5</v>
       </c>
       <c r="C9" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="F9">
         <v>3</v>
       </c>
       <c r="G9" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="J9">
         <v>6</v>
       </c>
       <c r="K9" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.25">
@@ -4646,19 +4667,19 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="F10">
         <v>5</v>
       </c>
       <c r="G10" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="J10">
         <v>7</v>
       </c>
       <c r="K10" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.25">
@@ -4666,19 +4687,19 @@
         <v>7</v>
       </c>
       <c r="C11" s="39" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="F11">
         <v>6</v>
       </c>
       <c r="G11" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="J11">
         <v>8</v>
       </c>
       <c r="K11" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.25">
@@ -4686,19 +4707,19 @@
         <v>8</v>
       </c>
       <c r="C12" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="F12">
         <v>8</v>
       </c>
       <c r="G12" t="s">
-        <v>791</v>
+        <v>784</v>
       </c>
       <c r="J12">
         <v>10</v>
       </c>
       <c r="K12" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.25">
@@ -4706,19 +4727,19 @@
         <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="F13">
         <v>12</v>
       </c>
       <c r="G13" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="J13">
         <v>12</v>
       </c>
       <c r="K13" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
     </row>
     <row r="14" spans="2:11" x14ac:dyDescent="0.25">
@@ -4726,19 +4747,19 @@
         <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="F14">
         <v>14</v>
       </c>
       <c r="G14" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="J14">
         <v>15</v>
       </c>
       <c r="K14" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.25">
@@ -4746,19 +4767,19 @@
         <v>13</v>
       </c>
       <c r="C15" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="F15">
         <v>16</v>
       </c>
       <c r="G15" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="J15">
         <v>17</v>
       </c>
       <c r="K15" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.25">
@@ -4766,19 +4787,19 @@
         <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="F16">
         <v>20</v>
       </c>
       <c r="G16" t="s">
-        <v>777</v>
+        <v>770</v>
       </c>
       <c r="J16">
         <v>20</v>
       </c>
       <c r="K16" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
     </row>
     <row r="17" spans="8:11" x14ac:dyDescent="0.25">
@@ -4786,7 +4807,7 @@
         <v>24</v>
       </c>
       <c r="K17" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
     </row>
     <row r="18" spans="8:11" x14ac:dyDescent="0.25">
@@ -4794,57 +4815,57 @@
         <v>25</v>
       </c>
       <c r="K18" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
     </row>
     <row r="24" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H24" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
     </row>
     <row r="25" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H25" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
     </row>
     <row r="26" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H26" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
     </row>
     <row r="27" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H27" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
     </row>
     <row r="28" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H28" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
     </row>
     <row r="29" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H29" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="30" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H30" t="s">
-        <v>792</v>
+        <v>785</v>
       </c>
     </row>
     <row r="31" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H31" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
     </row>
     <row r="32" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H32" t="s">
-        <v>780</v>
+        <v>773</v>
       </c>
     </row>
     <row r="33" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H33" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
     </row>
   </sheetData>
@@ -4886,7 +4907,7 @@
         <v>48</v>
       </c>
       <c r="U6" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
     </row>
     <row r="7" spans="2:21" x14ac:dyDescent="0.25">
@@ -4894,43 +4915,43 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="E7">
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="H7">
         <v>1</v>
       </c>
       <c r="I7" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="K7">
         <v>1</v>
       </c>
       <c r="L7" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="N7">
         <v>1</v>
       </c>
       <c r="O7" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="Q7">
         <v>1</v>
       </c>
       <c r="R7" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="T7">
         <v>1</v>
       </c>
       <c r="U7" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
     </row>
     <row r="8" spans="2:21" x14ac:dyDescent="0.25">
@@ -4938,31 +4959,31 @@
         <v>3</v>
       </c>
       <c r="C8" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="E8">
         <v>2</v>
       </c>
       <c r="F8" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
       <c r="H8">
         <v>2</v>
       </c>
       <c r="I8" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
       <c r="K8">
         <v>2</v>
       </c>
       <c r="L8" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="N8">
         <v>3</v>
       </c>
       <c r="O8" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="Q8">
         <v>2</v>
@@ -4974,7 +4995,7 @@
         <v>1</v>
       </c>
       <c r="U8" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
     </row>
     <row r="9" spans="2:21" x14ac:dyDescent="0.25">
@@ -4982,43 +5003,43 @@
         <v>5</v>
       </c>
       <c r="C9" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="E9">
         <v>4</v>
       </c>
       <c r="F9" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="H9">
         <v>4</v>
       </c>
       <c r="I9" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
       <c r="K9">
         <v>5</v>
       </c>
       <c r="L9" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
       <c r="N9">
         <v>5</v>
       </c>
       <c r="O9" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="Q9">
         <v>5</v>
       </c>
       <c r="R9" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="T9">
         <v>3</v>
       </c>
       <c r="U9" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
     </row>
     <row r="10" spans="2:21" x14ac:dyDescent="0.25">
@@ -5026,43 +5047,43 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
       <c r="E10">
         <v>6</v>
       </c>
       <c r="F10" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="H10">
         <v>5</v>
       </c>
       <c r="I10" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="K10">
         <v>8</v>
       </c>
       <c r="L10" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="N10">
         <v>8</v>
       </c>
       <c r="O10" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
       <c r="Q10">
         <v>8</v>
       </c>
       <c r="R10" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="T10">
         <v>3</v>
       </c>
       <c r="U10" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
     </row>
     <row r="11" spans="2:21" x14ac:dyDescent="0.25">
@@ -5070,37 +5091,37 @@
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="E11">
         <v>8</v>
       </c>
       <c r="F11" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
       <c r="H11">
         <v>7</v>
       </c>
       <c r="I11" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="K11">
         <v>10</v>
       </c>
       <c r="L11" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="N11">
         <v>12</v>
       </c>
       <c r="O11" t="s">
-        <v>789</v>
+        <v>782</v>
       </c>
       <c r="Q11">
         <v>10</v>
       </c>
       <c r="R11" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="T11">
         <v>6</v>
@@ -5114,31 +5135,31 @@
         <v>10</v>
       </c>
       <c r="C12" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="E12">
         <v>11</v>
       </c>
       <c r="F12" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="H12">
         <v>8</v>
       </c>
       <c r="I12" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="K12">
         <v>12</v>
       </c>
       <c r="L12" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="N12">
         <v>13</v>
       </c>
       <c r="O12" t="s">
-        <v>787</v>
+        <v>780</v>
       </c>
       <c r="Q12">
         <v>12</v>
@@ -5150,7 +5171,7 @@
         <v>9</v>
       </c>
       <c r="U12" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
     </row>
     <row r="13" spans="2:21" x14ac:dyDescent="0.25">
@@ -5158,13 +5179,13 @@
         <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="E13">
         <v>15</v>
       </c>
       <c r="F13" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="H13">
         <v>13</v>
@@ -5176,25 +5197,25 @@
         <v>14</v>
       </c>
       <c r="L13" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="N13">
         <v>14</v>
       </c>
       <c r="O13" t="s">
-        <v>786</v>
+        <v>779</v>
       </c>
       <c r="Q13">
         <v>14</v>
       </c>
       <c r="R13" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="T13">
         <v>12</v>
       </c>
       <c r="U13" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
     </row>
     <row r="14" spans="2:21" x14ac:dyDescent="0.25">
@@ -5202,43 +5223,43 @@
         <v>11</v>
       </c>
       <c r="C14" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="E14">
         <v>16</v>
       </c>
       <c r="F14" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="H14">
         <v>16</v>
       </c>
       <c r="I14" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="K14">
         <v>15</v>
       </c>
       <c r="L14" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="N14">
         <v>15</v>
       </c>
       <c r="O14" t="s">
-        <v>788</v>
+        <v>781</v>
       </c>
       <c r="Q14">
         <v>15</v>
       </c>
       <c r="R14" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="T14">
         <v>15</v>
       </c>
       <c r="U14" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
     </row>
     <row r="15" spans="2:21" x14ac:dyDescent="0.25">
@@ -5246,43 +5267,43 @@
         <v>13</v>
       </c>
       <c r="C15" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="E15">
         <v>18</v>
       </c>
       <c r="F15" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="H15">
         <v>17</v>
       </c>
       <c r="I15" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="K15">
         <v>16</v>
       </c>
       <c r="L15" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="N15">
         <v>16</v>
       </c>
       <c r="O15" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="Q15">
         <v>16</v>
       </c>
       <c r="R15" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="T15">
         <v>17</v>
       </c>
       <c r="U15" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
     </row>
     <row r="16" spans="2:21" x14ac:dyDescent="0.25">
@@ -5290,43 +5311,43 @@
         <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="E16">
         <v>20</v>
       </c>
       <c r="F16" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="H16">
         <v>20</v>
       </c>
       <c r="I16" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="K16">
         <v>20</v>
       </c>
       <c r="L16" t="s">
-        <v>793</v>
+        <v>786</v>
       </c>
       <c r="N16">
         <v>20</v>
       </c>
       <c r="O16" t="s">
-        <v>594</v>
+        <v>591</v>
       </c>
       <c r="Q16">
         <v>20</v>
       </c>
       <c r="R16" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="T16">
         <v>19</v>
       </c>
       <c r="U16" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
     </row>
     <row r="17" spans="9:21" x14ac:dyDescent="0.25">
@@ -5334,25 +5355,25 @@
         <v>23</v>
       </c>
       <c r="L17" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="N17">
         <v>23</v>
       </c>
       <c r="O17" t="s">
-        <v>782</v>
+        <v>775</v>
       </c>
       <c r="Q17">
         <v>23</v>
       </c>
       <c r="R17" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="T17">
         <v>23</v>
       </c>
       <c r="U17" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
     </row>
     <row r="18" spans="9:21" x14ac:dyDescent="0.25">
@@ -5360,110 +5381,110 @@
         <v>25</v>
       </c>
       <c r="L18" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="N18">
         <v>25</v>
       </c>
       <c r="O18" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="Q18">
         <v>25</v>
       </c>
       <c r="R18" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="T18">
         <v>25</v>
       </c>
       <c r="U18" t="s">
-        <v>740</v>
+        <v>733</v>
       </c>
     </row>
     <row r="21" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I21" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
     </row>
     <row r="22" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I22" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
     </row>
     <row r="23" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I23" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
     </row>
     <row r="24" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I24" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
     </row>
     <row r="25" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I25" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
     </row>
     <row r="26" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I26" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
     </row>
     <row r="27" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I27" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
     </row>
     <row r="28" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I28" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
     </row>
     <row r="29" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I29" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
     </row>
     <row r="30" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I30" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
     </row>
     <row r="31" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I31" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
     </row>
     <row r="32" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I32" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
     </row>
     <row r="33" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I33" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
     </row>
     <row r="34" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I34" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
     </row>
     <row r="35" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I35" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
     </row>
     <row r="36" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I36" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
     </row>
     <row r="37" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I37" t="s">
-        <v>741</v>
+        <v>734</v>
       </c>
     </row>
   </sheetData>
@@ -5528,7 +5549,7 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="H7">
         <v>1</v>
@@ -5540,7 +5561,7 @@
         <v>1</v>
       </c>
       <c r="L7" t="s">
-        <v>731</v>
+        <v>724</v>
       </c>
       <c r="N7">
         <v>1</v>
@@ -5584,13 +5605,13 @@
         <v>1</v>
       </c>
       <c r="L8" t="s">
-        <v>732</v>
+        <v>725</v>
       </c>
       <c r="N8">
         <v>1</v>
       </c>
       <c r="O8" t="s">
-        <v>692</v>
+        <v>685</v>
       </c>
       <c r="Q8">
         <v>1</v>
@@ -5610,7 +5631,7 @@
         <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>733</v>
+        <v>726</v>
       </c>
       <c r="E9">
         <v>2</v>
@@ -5628,7 +5649,7 @@
         <v>1</v>
       </c>
       <c r="L9" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
       <c r="N9">
         <v>1</v>
@@ -5654,13 +5675,13 @@
         <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>734</v>
+        <v>727</v>
       </c>
       <c r="E10">
         <v>5</v>
       </c>
       <c r="F10" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="H10">
         <v>7</v>
@@ -5672,7 +5693,7 @@
         <v>5</v>
       </c>
       <c r="L10" t="s">
-        <v>730</v>
+        <v>723</v>
       </c>
       <c r="N10">
         <v>5</v>
@@ -5684,7 +5705,7 @@
         <v>2</v>
       </c>
       <c r="R10" t="s">
-        <v>765</v>
+        <v>758</v>
       </c>
       <c r="T10">
         <v>4</v>
@@ -5698,13 +5719,13 @@
         <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>735</v>
+        <v>728</v>
       </c>
       <c r="E11">
         <v>10</v>
       </c>
       <c r="F11" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="H11">
         <v>10</v>
@@ -5716,7 +5737,7 @@
         <v>8</v>
       </c>
       <c r="L11" t="s">
-        <v>724</v>
+        <v>717</v>
       </c>
       <c r="N11">
         <v>10</v>
@@ -5734,7 +5755,7 @@
         <v>7</v>
       </c>
       <c r="U11" t="s">
-        <v>689</v>
+        <v>682</v>
       </c>
     </row>
     <row r="12" spans="2:21" x14ac:dyDescent="0.25">
@@ -5760,7 +5781,7 @@
         <v>13</v>
       </c>
       <c r="L12" t="s">
-        <v>728</v>
+        <v>721</v>
       </c>
       <c r="N12">
         <v>12</v>
@@ -5772,7 +5793,7 @@
         <v>7</v>
       </c>
       <c r="R12" t="s">
-        <v>688</v>
+        <v>681</v>
       </c>
       <c r="T12">
         <v>10</v>
@@ -5792,7 +5813,7 @@
         <v>17</v>
       </c>
       <c r="F13" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="H13">
         <v>15</v>
@@ -5804,7 +5825,7 @@
         <v>16</v>
       </c>
       <c r="L13" t="s">
-        <v>736</v>
+        <v>729</v>
       </c>
       <c r="N13">
         <v>12</v>
@@ -5830,13 +5851,13 @@
         <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="E14">
         <v>18</v>
       </c>
       <c r="F14" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="H14">
         <v>20</v>
@@ -5848,13 +5869,13 @@
         <v>18</v>
       </c>
       <c r="L14" t="s">
-        <v>737</v>
+        <v>730</v>
       </c>
       <c r="N14">
         <v>15</v>
       </c>
       <c r="O14" t="s">
-        <v>573</v>
+        <v>570</v>
       </c>
       <c r="Q14">
         <v>12</v>
@@ -5874,7 +5895,7 @@
         <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>764</v>
+        <v>757</v>
       </c>
       <c r="E15">
         <v>19</v>
@@ -5892,7 +5913,7 @@
         <v>20</v>
       </c>
       <c r="L15" t="s">
-        <v>725</v>
+        <v>718</v>
       </c>
       <c r="N15">
         <v>18</v>
@@ -5918,13 +5939,13 @@
         <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
       <c r="E16">
         <v>20</v>
       </c>
       <c r="F16" t="s">
-        <v>546</v>
+        <v>543</v>
       </c>
       <c r="H16">
         <v>20</v>
@@ -5936,7 +5957,7 @@
         <v>21</v>
       </c>
       <c r="L16" t="s">
-        <v>729</v>
+        <v>722</v>
       </c>
       <c r="N16">
         <v>20</v>
@@ -5954,7 +5975,7 @@
         <v>19</v>
       </c>
       <c r="U16" t="s">
-        <v>693</v>
+        <v>686</v>
       </c>
     </row>
     <row r="17" spans="10:21" x14ac:dyDescent="0.25">
@@ -5962,7 +5983,7 @@
         <v>22</v>
       </c>
       <c r="L17" t="s">
-        <v>738</v>
+        <v>731</v>
       </c>
       <c r="N17">
         <v>20</v>
@@ -5988,7 +6009,7 @@
         <v>25</v>
       </c>
       <c r="L18" t="s">
-        <v>739</v>
+        <v>732</v>
       </c>
       <c r="N18">
         <v>25</v>
@@ -6026,22 +6047,22 @@
     </row>
     <row r="25" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J25" t="s">
-        <v>690</v>
+        <v>683</v>
       </c>
     </row>
     <row r="26" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J26" t="s">
-        <v>685</v>
+        <v>678</v>
       </c>
     </row>
     <row r="27" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J27" t="s">
-        <v>686</v>
+        <v>679</v>
       </c>
     </row>
     <row r="28" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J28" t="s">
-        <v>773</v>
+        <v>766</v>
       </c>
     </row>
     <row r="29" spans="10:21" x14ac:dyDescent="0.25">
@@ -6056,27 +6077,27 @@
     </row>
     <row r="31" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J31" t="s">
-        <v>687</v>
+        <v>680</v>
       </c>
     </row>
     <row r="32" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J32" t="s">
-        <v>691</v>
+        <v>684</v>
       </c>
     </row>
     <row r="33" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J33" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
     </row>
     <row r="34" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J34" t="s">
-        <v>694</v>
+        <v>687</v>
       </c>
     </row>
     <row r="35" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J35" t="s">
-        <v>695</v>
+        <v>688</v>
       </c>
     </row>
   </sheetData>
@@ -6111,19 +6132,19 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>673</v>
+        <v>666</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>675</v>
+        <v>668</v>
       </c>
       <c r="J7">
         <v>1</v>
       </c>
       <c r="K7" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.25">
@@ -6131,7 +6152,7 @@
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>661</v>
+        <v>654</v>
       </c>
       <c r="F8">
         <v>1</v>
@@ -6143,7 +6164,7 @@
         <v>5</v>
       </c>
       <c r="K8" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.25">
@@ -6151,19 +6172,19 @@
         <v>5</v>
       </c>
       <c r="C9" t="s">
-        <v>674</v>
+        <v>667</v>
       </c>
       <c r="F9">
         <v>3</v>
       </c>
       <c r="G9" t="s">
-        <v>678</v>
+        <v>671</v>
       </c>
       <c r="J9">
         <v>7</v>
       </c>
       <c r="K9" t="s">
-        <v>594</v>
+        <v>591</v>
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.25">
@@ -6177,13 +6198,13 @@
         <v>6</v>
       </c>
       <c r="G10" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="J10">
         <v>8</v>
       </c>
       <c r="K10" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.25">
@@ -6191,19 +6212,19 @@
         <v>7</v>
       </c>
       <c r="C11" t="s">
-        <v>667</v>
+        <v>660</v>
       </c>
       <c r="F11">
         <v>7</v>
       </c>
       <c r="G11" t="s">
-        <v>726</v>
+        <v>719</v>
       </c>
       <c r="J11">
         <v>11</v>
       </c>
       <c r="K11" t="s">
-        <v>681</v>
+        <v>674</v>
       </c>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.25">
@@ -6211,19 +6232,19 @@
         <v>8</v>
       </c>
       <c r="C12" t="s">
-        <v>668</v>
+        <v>661</v>
       </c>
       <c r="F12">
         <v>8</v>
       </c>
       <c r="G12" t="s">
-        <v>669</v>
+        <v>662</v>
       </c>
       <c r="J12">
         <v>11</v>
       </c>
       <c r="K12" t="s">
-        <v>680</v>
+        <v>673</v>
       </c>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.25">
@@ -6231,19 +6252,19 @@
         <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>675</v>
+        <v>668</v>
       </c>
       <c r="F13">
         <v>12</v>
       </c>
       <c r="G13" t="s">
-        <v>670</v>
+        <v>663</v>
       </c>
       <c r="J13">
         <v>13</v>
       </c>
       <c r="K13" t="s">
-        <v>723</v>
+        <v>716</v>
       </c>
     </row>
     <row r="14" spans="2:11" x14ac:dyDescent="0.25">
@@ -6257,13 +6278,13 @@
         <v>16</v>
       </c>
       <c r="G14" t="s">
-        <v>683</v>
+        <v>676</v>
       </c>
       <c r="J14">
         <v>15</v>
       </c>
       <c r="K14" t="s">
-        <v>781</v>
+        <v>774</v>
       </c>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.25">
@@ -6271,19 +6292,19 @@
         <v>13</v>
       </c>
       <c r="C15" t="s">
-        <v>676</v>
+        <v>669</v>
       </c>
       <c r="F15">
         <v>19</v>
       </c>
       <c r="G15" t="s">
-        <v>684</v>
+        <v>677</v>
       </c>
       <c r="J15">
         <v>18</v>
       </c>
       <c r="K15" t="s">
-        <v>679</v>
+        <v>672</v>
       </c>
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.25">
@@ -6291,19 +6312,19 @@
         <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>677</v>
+        <v>670</v>
       </c>
       <c r="F16">
         <v>20</v>
       </c>
       <c r="G16" t="s">
-        <v>594</v>
+        <v>591</v>
       </c>
       <c r="J16">
         <v>20</v>
       </c>
       <c r="K16" t="s">
-        <v>671</v>
+        <v>664</v>
       </c>
     </row>
     <row r="17" spans="10:11" x14ac:dyDescent="0.25">
@@ -6311,7 +6332,7 @@
         <v>20</v>
       </c>
       <c r="K17" t="s">
-        <v>672</v>
+        <v>665</v>
       </c>
     </row>
     <row r="18" spans="10:11" x14ac:dyDescent="0.25">
@@ -6319,27 +6340,27 @@
         <v>25</v>
       </c>
       <c r="K18" t="s">
-        <v>660</v>
+        <v>653</v>
       </c>
     </row>
     <row r="27" spans="10:11" x14ac:dyDescent="0.25">
       <c r="K27" t="s">
-        <v>662</v>
+        <v>655</v>
       </c>
     </row>
     <row r="28" spans="10:11" x14ac:dyDescent="0.25">
       <c r="K28" t="s">
-        <v>664</v>
+        <v>657</v>
       </c>
     </row>
     <row r="29" spans="10:11" x14ac:dyDescent="0.25">
       <c r="K29" t="s">
-        <v>663</v>
+        <v>656</v>
       </c>
     </row>
     <row r="30" spans="10:11" x14ac:dyDescent="0.25">
       <c r="K30" t="s">
-        <v>682</v>
+        <v>675</v>
       </c>
     </row>
   </sheetData>
@@ -6372,7 +6393,7 @@
         <v>63</v>
       </c>
       <c r="I6" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="L6" t="s">
         <v>54</v>
@@ -6381,7 +6402,7 @@
         <v>55</v>
       </c>
       <c r="R6" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="V6" t="s">
         <v>66</v>
@@ -6392,7 +6413,7 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -6404,7 +6425,7 @@
         <v>1</v>
       </c>
       <c r="I7" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="K7">
         <v>1</v>
@@ -6416,19 +6437,19 @@
         <v>1</v>
       </c>
       <c r="O7" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="Q7">
         <v>1</v>
       </c>
       <c r="R7" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
       <c r="U7">
         <v>1</v>
       </c>
       <c r="V7" t="s">
-        <v>760</v>
+        <v>753</v>
       </c>
     </row>
     <row r="8" spans="2:22" x14ac:dyDescent="0.25">
@@ -6436,7 +6457,7 @@
         <v>3</v>
       </c>
       <c r="C8" t="s">
-        <v>622</v>
+        <v>615</v>
       </c>
       <c r="E8">
         <v>4</v>
@@ -6448,13 +6469,13 @@
         <v>1</v>
       </c>
       <c r="I8" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
       <c r="K8">
         <v>2</v>
       </c>
       <c r="L8" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="N8">
         <v>2</v>
@@ -6466,13 +6487,13 @@
         <v>3</v>
       </c>
       <c r="R8" t="s">
-        <v>756</v>
+        <v>749</v>
       </c>
       <c r="U8">
         <v>2</v>
       </c>
       <c r="V8" t="s">
-        <v>751</v>
+        <v>744</v>
       </c>
     </row>
     <row r="9" spans="2:22" x14ac:dyDescent="0.25">
@@ -6480,13 +6501,13 @@
         <v>5</v>
       </c>
       <c r="C9" t="s">
-        <v>746</v>
+        <v>739</v>
       </c>
       <c r="E9">
         <v>4</v>
       </c>
       <c r="F9" t="s">
-        <v>632</v>
+        <v>625</v>
       </c>
       <c r="H9">
         <v>4</v>
@@ -6498,7 +6519,7 @@
         <v>2</v>
       </c>
       <c r="L9" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="N9">
         <v>5</v>
@@ -6510,13 +6531,13 @@
         <v>5</v>
       </c>
       <c r="R9" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="U9">
         <v>2</v>
       </c>
       <c r="V9" t="s">
-        <v>747</v>
+        <v>740</v>
       </c>
     </row>
     <row r="10" spans="2:22" x14ac:dyDescent="0.25">
@@ -6524,43 +6545,43 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
       <c r="E10">
         <v>6</v>
       </c>
       <c r="F10" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="H10">
         <v>5</v>
       </c>
       <c r="I10" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
       <c r="K10">
         <v>8</v>
       </c>
       <c r="L10" t="s">
-        <v>634</v>
+        <v>627</v>
       </c>
       <c r="N10">
         <v>8</v>
       </c>
       <c r="O10" t="s">
-        <v>591</v>
+        <v>588</v>
       </c>
       <c r="Q10">
         <v>8</v>
       </c>
       <c r="R10" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="U10">
         <v>6</v>
       </c>
       <c r="V10" t="s">
-        <v>757</v>
+        <v>750</v>
       </c>
     </row>
     <row r="11" spans="2:22" x14ac:dyDescent="0.25">
@@ -6568,19 +6589,19 @@
         <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="E11">
         <v>8</v>
       </c>
       <c r="F11" t="s">
-        <v>624</v>
+        <v>617</v>
       </c>
       <c r="H11">
         <v>7</v>
       </c>
       <c r="I11" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="K11">
         <v>10</v>
@@ -6592,19 +6613,19 @@
         <v>10</v>
       </c>
       <c r="O11" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="Q11">
         <v>10</v>
       </c>
       <c r="R11" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="U11">
         <v>7</v>
       </c>
       <c r="V11" t="s">
-        <v>767</v>
+        <v>760</v>
       </c>
     </row>
     <row r="12" spans="2:22" x14ac:dyDescent="0.25">
@@ -6612,25 +6633,25 @@
         <v>10</v>
       </c>
       <c r="C12" t="s">
-        <v>752</v>
+        <v>745</v>
       </c>
       <c r="E12">
         <v>11</v>
       </c>
       <c r="F12" t="s">
-        <v>607</v>
+        <v>604</v>
       </c>
       <c r="H12">
         <v>8</v>
       </c>
       <c r="I12" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="K12">
         <v>12</v>
       </c>
       <c r="L12" t="s">
-        <v>552</v>
+        <v>549</v>
       </c>
       <c r="N12">
         <v>12</v>
@@ -6642,13 +6663,13 @@
         <v>12</v>
       </c>
       <c r="R12" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
       <c r="U12">
         <v>8</v>
       </c>
       <c r="V12" t="s">
-        <v>758</v>
+        <v>751</v>
       </c>
     </row>
     <row r="13" spans="2:22" x14ac:dyDescent="0.25">
@@ -6656,25 +6677,25 @@
         <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>626</v>
+        <v>619</v>
       </c>
       <c r="E13">
         <v>14</v>
       </c>
       <c r="F13" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="H13">
         <v>9</v>
       </c>
       <c r="I13" t="s">
-        <v>771</v>
+        <v>764</v>
       </c>
       <c r="K13">
         <v>14</v>
       </c>
       <c r="L13" t="s">
-        <v>627</v>
+        <v>620</v>
       </c>
       <c r="N13">
         <v>14</v>
@@ -6686,13 +6707,13 @@
         <v>14</v>
       </c>
       <c r="R13" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="U13">
         <v>9</v>
       </c>
       <c r="V13" t="s">
-        <v>748</v>
+        <v>741</v>
       </c>
     </row>
     <row r="14" spans="2:22" x14ac:dyDescent="0.25">
@@ -6700,7 +6721,7 @@
         <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="E14">
         <v>16</v>
@@ -6712,7 +6733,7 @@
         <v>11</v>
       </c>
       <c r="I14" t="s">
-        <v>750</v>
+        <v>743</v>
       </c>
       <c r="K14">
         <v>15</v>
@@ -6724,19 +6745,19 @@
         <v>15</v>
       </c>
       <c r="O14" t="s">
-        <v>590</v>
+        <v>587</v>
       </c>
       <c r="Q14">
         <v>15</v>
       </c>
       <c r="R14" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="U14">
         <v>14</v>
       </c>
       <c r="V14" t="s">
-        <v>762</v>
+        <v>755</v>
       </c>
     </row>
     <row r="15" spans="2:22" x14ac:dyDescent="0.25">
@@ -6744,25 +6765,25 @@
         <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>769</v>
+        <v>762</v>
       </c>
       <c r="E15">
         <v>18</v>
       </c>
       <c r="F15" t="s">
-        <v>753</v>
+        <v>746</v>
       </c>
       <c r="H15">
         <v>16</v>
       </c>
       <c r="I15" t="s">
-        <v>597</v>
+        <v>594</v>
       </c>
       <c r="K15">
         <v>20</v>
       </c>
       <c r="L15" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
       <c r="N15">
         <v>16</v>
@@ -6774,13 +6795,13 @@
         <v>16</v>
       </c>
       <c r="R15" t="s">
-        <v>761</v>
+        <v>754</v>
       </c>
       <c r="U15">
         <v>17</v>
       </c>
       <c r="V15" t="s">
-        <v>633</v>
+        <v>626</v>
       </c>
     </row>
     <row r="16" spans="2:22" x14ac:dyDescent="0.25">
@@ -6788,43 +6809,43 @@
         <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>628</v>
+        <v>621</v>
       </c>
       <c r="E16">
         <v>20</v>
       </c>
       <c r="F16" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="H16">
         <v>20</v>
       </c>
       <c r="I16" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
       <c r="K16">
         <v>20</v>
       </c>
       <c r="L16" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="N16">
         <v>20</v>
       </c>
       <c r="O16" t="s">
-        <v>658</v>
+        <v>651</v>
       </c>
       <c r="Q16">
         <v>20</v>
       </c>
       <c r="R16" t="s">
-        <v>631</v>
+        <v>624</v>
       </c>
       <c r="U16">
         <v>20</v>
       </c>
       <c r="V16" t="s">
-        <v>749</v>
+        <v>742</v>
       </c>
     </row>
     <row r="17" spans="11:22" x14ac:dyDescent="0.25">
@@ -6832,25 +6853,25 @@
         <v>24</v>
       </c>
       <c r="L17" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="N17">
         <v>23</v>
       </c>
       <c r="O17" t="s">
-        <v>604</v>
+        <v>601</v>
       </c>
       <c r="Q17">
         <v>23</v>
       </c>
       <c r="R17" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
       <c r="U17">
         <v>24</v>
       </c>
       <c r="V17" t="s">
-        <v>759</v>
+        <v>752</v>
       </c>
     </row>
     <row r="18" spans="11:22" x14ac:dyDescent="0.25">
@@ -6858,75 +6879,75 @@
         <v>25</v>
       </c>
       <c r="L18" t="s">
-        <v>629</v>
+        <v>622</v>
       </c>
       <c r="N18">
         <v>25</v>
       </c>
       <c r="O18" t="s">
-        <v>784</v>
+        <v>777</v>
       </c>
       <c r="Q18">
         <v>25</v>
       </c>
       <c r="R18" t="s">
-        <v>635</v>
+        <v>628</v>
       </c>
       <c r="U18">
         <v>25</v>
       </c>
       <c r="V18" t="s">
-        <v>768</v>
+        <v>761</v>
       </c>
     </row>
     <row r="22" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L22" t="s">
-        <v>785</v>
+        <v>778</v>
       </c>
     </row>
     <row r="23" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L23" t="s">
-        <v>770</v>
+        <v>763</v>
       </c>
     </row>
     <row r="24" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L24" t="s">
-        <v>772</v>
+        <v>765</v>
       </c>
     </row>
     <row r="25" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L25" t="s">
-        <v>623</v>
+        <v>616</v>
       </c>
     </row>
     <row r="26" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L26" t="s">
-        <v>625</v>
+        <v>618</v>
       </c>
     </row>
     <row r="27" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L27" t="s">
-        <v>659</v>
+        <v>652</v>
       </c>
     </row>
     <row r="28" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L28" t="s">
-        <v>630</v>
+        <v>623</v>
       </c>
     </row>
     <row r="29" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L29" t="s">
-        <v>666</v>
+        <v>659</v>
       </c>
     </row>
     <row r="30" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L30" t="s">
-        <v>665</v>
+        <v>658</v>
       </c>
     </row>
     <row r="33" spans="13:13" x14ac:dyDescent="0.25">
       <c r="M33" t="s">
-        <v>763</v>
+        <v>756</v>
       </c>
     </row>
   </sheetData>
@@ -6974,19 +6995,19 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
+        <v>575</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7" t="s">
+        <v>609</v>
+      </c>
+      <c r="K7">
+        <v>1</v>
+      </c>
+      <c r="L7" t="s">
         <v>578</v>
-      </c>
-      <c r="H7">
-        <v>1</v>
-      </c>
-      <c r="I7" t="s">
-        <v>612</v>
-      </c>
-      <c r="K7">
-        <v>1</v>
-      </c>
-      <c r="L7" t="s">
-        <v>581</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
@@ -6997,36 +7018,36 @@
         <v>279</v>
       </c>
       <c r="E8">
-        <v>1</v>
-      </c>
-      <c r="F8" t="s">
-        <v>337</v>
+        <v>2</v>
+      </c>
+      <c r="F8" s="39" t="s">
+        <v>796</v>
       </c>
       <c r="H8">
         <v>2</v>
       </c>
       <c r="I8" t="s">
-        <v>700</v>
+        <v>693</v>
       </c>
       <c r="K8">
         <v>1</v>
       </c>
       <c r="L8" t="s">
-        <v>617</v>
+        <v>613</v>
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="E9">
         <v>3</v>
       </c>
       <c r="F9" t="s">
-        <v>696</v>
+        <v>689</v>
       </c>
       <c r="H9">
         <v>5</v>
@@ -7038,59 +7059,59 @@
         <v>3</v>
       </c>
       <c r="L9" t="s">
-        <v>709</v>
+        <v>702</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>619</v>
+        <v>328</v>
       </c>
       <c r="E10">
         <v>4</v>
       </c>
       <c r="F10" t="s">
-        <v>618</v>
+        <v>691</v>
       </c>
       <c r="H10">
         <v>8</v>
       </c>
       <c r="I10" t="s">
-        <v>697</v>
+        <v>690</v>
       </c>
       <c r="K10">
         <v>4</v>
       </c>
       <c r="L10" t="s">
-        <v>616</v>
+        <v>698</v>
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C11" t="s">
-        <v>328</v>
+        <v>793</v>
       </c>
       <c r="E11">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F11" t="s">
-        <v>698</v>
+        <v>338</v>
       </c>
       <c r="H11">
         <v>10</v>
       </c>
       <c r="I11" t="s">
-        <v>702</v>
+        <v>695</v>
       </c>
       <c r="K11">
         <v>5</v>
       </c>
       <c r="L11" t="s">
-        <v>705</v>
+        <v>787</v>
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
@@ -7098,13 +7119,13 @@
         <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>620</v>
+        <v>794</v>
       </c>
       <c r="E12">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F12" t="s">
-        <v>338</v>
+        <v>614</v>
       </c>
       <c r="H12">
         <v>12</v>
@@ -7116,7 +7137,7 @@
         <v>8</v>
       </c>
       <c r="L12" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
@@ -7130,19 +7151,19 @@
         <v>13</v>
       </c>
       <c r="F13" t="s">
-        <v>699</v>
+        <v>371</v>
       </c>
       <c r="H13">
         <v>14</v>
       </c>
       <c r="I13" t="s">
-        <v>701</v>
+        <v>694</v>
       </c>
       <c r="K13">
         <v>10</v>
       </c>
       <c r="L13" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
@@ -7150,13 +7171,13 @@
         <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>621</v>
+        <v>795</v>
       </c>
       <c r="E14">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F14" t="s">
-        <v>241</v>
+        <v>692</v>
       </c>
       <c r="H14">
         <v>15</v>
@@ -7168,7 +7189,7 @@
         <v>15</v>
       </c>
       <c r="L14" t="s">
-        <v>779</v>
+        <v>772</v>
       </c>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.25">
@@ -7182,19 +7203,19 @@
         <v>17</v>
       </c>
       <c r="F15" t="s">
-        <v>374</v>
+        <v>241</v>
       </c>
       <c r="H15">
         <v>16</v>
       </c>
       <c r="I15" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="K15">
         <v>18</v>
       </c>
       <c r="L15" t="s">
-        <v>707</v>
+        <v>700</v>
       </c>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
@@ -7202,25 +7223,25 @@
         <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>578</v>
+        <v>797</v>
       </c>
       <c r="E16">
         <v>20</v>
       </c>
       <c r="F16" t="s">
-        <v>704</v>
+        <v>697</v>
       </c>
       <c r="H16">
         <v>20</v>
       </c>
       <c r="I16" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
       <c r="K16">
         <v>20</v>
       </c>
       <c r="L16" t="s">
-        <v>706</v>
+        <v>699</v>
       </c>
     </row>
     <row r="17" spans="8:12" x14ac:dyDescent="0.25">
@@ -7228,13 +7249,13 @@
         <v>23</v>
       </c>
       <c r="I17" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="K17">
         <v>21</v>
       </c>
       <c r="L17" t="s">
-        <v>576</v>
+        <v>573</v>
       </c>
     </row>
     <row r="18" spans="8:12" x14ac:dyDescent="0.25">
@@ -7242,38 +7263,38 @@
         <v>25</v>
       </c>
       <c r="I18" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
       <c r="K18">
         <v>25</v>
       </c>
       <c r="L18" t="s">
-        <v>708</v>
+        <v>701</v>
       </c>
     </row>
     <row r="22" spans="8:12" x14ac:dyDescent="0.25">
       <c r="I22" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
     </row>
     <row r="23" spans="8:12" x14ac:dyDescent="0.25">
       <c r="I23" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
     </row>
     <row r="24" spans="8:12" x14ac:dyDescent="0.25">
       <c r="I24" t="s">
-        <v>703</v>
+        <v>696</v>
       </c>
     </row>
     <row r="25" spans="8:12" x14ac:dyDescent="0.25">
       <c r="I25" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
     </row>
     <row r="26" spans="8:12" x14ac:dyDescent="0.25">
       <c r="I26" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
     </row>
   </sheetData>
@@ -7297,55 +7318,55 @@
         <v>11</v>
       </c>
       <c r="D4" s="17" t="s">
+        <v>435</v>
+      </c>
+      <c r="E4" s="17" t="s">
+        <v>436</v>
+      </c>
+      <c r="F4" s="17" t="s">
+        <v>437</v>
+      </c>
+      <c r="G4" s="17" t="s">
+        <v>440</v>
+      </c>
+      <c r="H4" s="17" t="s">
         <v>438</v>
       </c>
-      <c r="E4" s="17" t="s">
+      <c r="I4" s="17" t="s">
         <v>439</v>
       </c>
-      <c r="F4" s="17" t="s">
-        <v>440</v>
-      </c>
-      <c r="G4" s="17" t="s">
-        <v>443</v>
-      </c>
-      <c r="H4" s="17" t="s">
+      <c r="J4" s="17" t="s">
         <v>441</v>
       </c>
-      <c r="I4" s="17" t="s">
+      <c r="K4" s="17" t="s">
         <v>442</v>
-      </c>
-      <c r="J4" s="17" t="s">
-        <v>444</v>
-      </c>
-      <c r="K4" s="17" t="s">
-        <v>445</v>
       </c>
       <c r="L4" s="17" t="s">
         <v>11</v>
       </c>
       <c r="M4" s="17" t="s">
+        <v>435</v>
+      </c>
+      <c r="N4" s="17" t="s">
+        <v>436</v>
+      </c>
+      <c r="O4" s="17" t="s">
+        <v>437</v>
+      </c>
+      <c r="P4" s="17" t="s">
+        <v>440</v>
+      </c>
+      <c r="Q4" s="17" t="s">
         <v>438</v>
       </c>
-      <c r="N4" s="17" t="s">
+      <c r="R4" s="17" t="s">
         <v>439</v>
       </c>
-      <c r="O4" s="17" t="s">
-        <v>440</v>
-      </c>
-      <c r="P4" s="17" t="s">
-        <v>443</v>
-      </c>
-      <c r="Q4" s="17" t="s">
+      <c r="S4" s="17" t="s">
         <v>441</v>
       </c>
-      <c r="R4" s="17" t="s">
+      <c r="T4" s="17" t="s">
         <v>442</v>
-      </c>
-      <c r="S4" s="17" t="s">
-        <v>444</v>
-      </c>
-      <c r="T4" s="17" t="s">
-        <v>445</v>
       </c>
     </row>
     <row r="5" spans="3:20" x14ac:dyDescent="0.25">
@@ -7623,7 +7644,7 @@
         <v>2</v>
       </c>
       <c r="L11" s="25" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="M11" s="28"/>
       <c r="N11" s="20">
@@ -8611,17 +8632,17 @@
     </row>
     <row r="36" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C36" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
     </row>
     <row r="37" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C37" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
     </row>
     <row r="38" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C38" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
     </row>
   </sheetData>
@@ -8644,10 +8665,10 @@
     <row r="7" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B8" s="35" t="s">
-        <v>711</v>
+        <v>704</v>
       </c>
       <c r="C8" s="36" t="s">
-        <v>710</v>
+        <v>703</v>
       </c>
       <c r="H8" t="s">
         <v>12</v>
@@ -8768,7 +8789,7 @@
         <v>130</v>
       </c>
       <c r="L14" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="M14" t="s">
         <v>148</v>
@@ -8827,7 +8848,7 @@
         <v>253</v>
       </c>
       <c r="M17" t="s">
-        <v>712</v>
+        <v>705</v>
       </c>
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.25">
@@ -8957,13 +8978,13 @@
         <v>39</v>
       </c>
       <c r="I24" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="L24" t="s">
         <v>41</v>
       </c>
       <c r="M24" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
     </row>
     <row r="25" spans="2:13" x14ac:dyDescent="0.25">
@@ -9017,7 +9038,7 @@
         <v>49</v>
       </c>
       <c r="M27" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
     </row>
     <row r="28" spans="2:13" x14ac:dyDescent="0.25">
@@ -9025,7 +9046,7 @@
         <v>45</v>
       </c>
       <c r="I28" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="L28" t="s">
         <v>43</v>
@@ -9081,7 +9102,7 @@
         <v>63</v>
       </c>
       <c r="I32" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="L32" t="s">
         <v>51</v>
@@ -9092,16 +9113,16 @@
     </row>
     <row r="33" spans="8:13" x14ac:dyDescent="0.25">
       <c r="H33" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="I33" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
       <c r="L33" t="s">
         <v>54</v>
       </c>
       <c r="M33" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
     </row>
     <row r="34" spans="8:13" x14ac:dyDescent="0.25">
@@ -9109,7 +9130,7 @@
         <v>64</v>
       </c>
       <c r="I34" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
       <c r="L34" t="s">
         <v>55</v>
@@ -9123,13 +9144,13 @@
         <v>59</v>
       </c>
       <c r="I35" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
       <c r="L35" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="M35" t="s">
-        <v>606</v>
+        <v>603</v>
       </c>
     </row>
     <row r="36" spans="8:13" x14ac:dyDescent="0.25">
@@ -9137,7 +9158,7 @@
         <v>58</v>
       </c>
       <c r="M36" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
     </row>
     <row r="37" spans="8:13" x14ac:dyDescent="0.25">
@@ -9145,7 +9166,7 @@
         <v>61</v>
       </c>
       <c r="M37" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
     </row>
   </sheetData>
@@ -9163,7 +9184,7 @@
   <sheetData>
     <row r="5" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>713</v>
+        <v>706</v>
       </c>
     </row>
     <row r="6" spans="2:2" x14ac:dyDescent="0.25">
@@ -9173,7 +9194,7 @@
     </row>
     <row r="8" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>585</v>
+        <v>582</v>
       </c>
     </row>
     <row r="9" spans="2:2" x14ac:dyDescent="0.25">
@@ -9193,7 +9214,7 @@
     </row>
     <row r="13" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
     </row>
     <row r="14" spans="2:2" x14ac:dyDescent="0.25">
@@ -9203,7 +9224,7 @@
     </row>
     <row r="16" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>584</v>
+        <v>581</v>
       </c>
     </row>
   </sheetData>
@@ -9320,13 +9341,13 @@
         <v>1</v>
       </c>
       <c r="L8" t="s">
-        <v>636</v>
+        <v>629</v>
       </c>
       <c r="N8">
         <v>2</v>
       </c>
       <c r="O8" t="s">
-        <v>650</v>
+        <v>643</v>
       </c>
       <c r="Q8">
         <v>2</v>
@@ -9338,7 +9359,7 @@
         <v>2</v>
       </c>
       <c r="U8" t="s">
-        <v>641</v>
+        <v>634</v>
       </c>
     </row>
     <row r="9" spans="2:21" x14ac:dyDescent="0.25">
@@ -9434,13 +9455,13 @@
         <v>8</v>
       </c>
       <c r="C11" s="39" t="s">
-        <v>775</v>
+        <v>768</v>
       </c>
       <c r="E11">
         <v>10</v>
       </c>
       <c r="F11" t="s">
-        <v>714</v>
+        <v>707</v>
       </c>
       <c r="H11">
         <v>10</v>
@@ -9540,25 +9561,25 @@
         <v>14</v>
       </c>
       <c r="L13" t="s">
-        <v>776</v>
+        <v>769</v>
       </c>
       <c r="N13">
         <v>14</v>
       </c>
       <c r="O13" t="s">
-        <v>776</v>
+        <v>769</v>
       </c>
       <c r="Q13">
         <v>14</v>
       </c>
       <c r="R13" t="s">
-        <v>776</v>
+        <v>769</v>
       </c>
       <c r="T13">
         <v>14</v>
       </c>
       <c r="U13" t="s">
-        <v>776</v>
+        <v>769</v>
       </c>
     </row>
     <row r="14" spans="2:21" x14ac:dyDescent="0.25">
@@ -9654,25 +9675,25 @@
         <v>20</v>
       </c>
       <c r="L16" t="s">
-        <v>653</v>
+        <v>646</v>
       </c>
       <c r="N16">
         <v>20</v>
       </c>
       <c r="O16" t="s">
-        <v>652</v>
+        <v>645</v>
       </c>
       <c r="Q16">
         <v>20</v>
       </c>
       <c r="R16" t="s">
-        <v>651</v>
+        <v>644</v>
       </c>
       <c r="T16">
         <v>20</v>
       </c>
       <c r="U16" t="s">
-        <v>640</v>
+        <v>633</v>
       </c>
     </row>
     <row r="17" spans="9:21" x14ac:dyDescent="0.25">
@@ -9729,42 +9750,42 @@
     </row>
     <row r="22" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I22" t="s">
-        <v>645</v>
+        <v>638</v>
       </c>
     </row>
     <row r="23" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I23" t="s">
-        <v>646</v>
+        <v>639</v>
       </c>
     </row>
     <row r="24" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I24" t="s">
-        <v>644</v>
+        <v>637</v>
       </c>
     </row>
     <row r="25" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I25" t="s">
-        <v>647</v>
+        <v>640</v>
       </c>
     </row>
     <row r="26" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I26" t="s">
-        <v>649</v>
+        <v>642</v>
       </c>
     </row>
     <row r="27" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I27" t="s">
-        <v>648</v>
+        <v>641</v>
       </c>
     </row>
     <row r="28" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I28" t="s">
-        <v>642</v>
+        <v>635</v>
       </c>
     </row>
     <row r="29" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I29" t="s">
-        <v>643</v>
+        <v>636</v>
       </c>
     </row>
     <row r="36" spans="11:11" x14ac:dyDescent="0.25">
@@ -9855,7 +9876,7 @@
         <v>3</v>
       </c>
       <c r="I8" t="s">
-        <v>638</v>
+        <v>631</v>
       </c>
       <c r="K8">
         <v>2</v>
@@ -9875,7 +9896,7 @@
         <v>5</v>
       </c>
       <c r="C9" s="39" t="s">
-        <v>774</v>
+        <v>767</v>
       </c>
       <c r="E9">
         <v>5</v>
@@ -9887,13 +9908,13 @@
         <v>5</v>
       </c>
       <c r="I9" t="s">
-        <v>654</v>
+        <v>647</v>
       </c>
       <c r="K9">
         <v>5</v>
       </c>
       <c r="L9" t="s">
-        <v>655</v>
+        <v>648</v>
       </c>
       <c r="N9">
         <v>5</v>
@@ -9919,13 +9940,13 @@
         <v>8</v>
       </c>
       <c r="I10" t="s">
-        <v>715</v>
+        <v>708</v>
       </c>
       <c r="K10">
         <v>8</v>
       </c>
       <c r="L10" t="s">
-        <v>716</v>
+        <v>709</v>
       </c>
       <c r="N10">
         <v>6</v>
@@ -10003,7 +10024,7 @@
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="E13">
         <v>14</v>
@@ -10015,19 +10036,19 @@
         <v>14</v>
       </c>
       <c r="I13" t="s">
-        <v>776</v>
+        <v>769</v>
       </c>
       <c r="K13">
         <v>14</v>
       </c>
       <c r="L13" t="s">
-        <v>776</v>
+        <v>769</v>
       </c>
       <c r="N13">
         <v>15</v>
       </c>
       <c r="O13" t="s">
-        <v>778</v>
+        <v>771</v>
       </c>
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.25">
@@ -10059,7 +10080,7 @@
         <v>17</v>
       </c>
       <c r="O14" t="s">
-        <v>783</v>
+        <v>776</v>
       </c>
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.25">
@@ -10111,19 +10132,19 @@
         <v>20</v>
       </c>
       <c r="I16" t="s">
-        <v>639</v>
+        <v>632</v>
       </c>
       <c r="K16">
         <v>20</v>
       </c>
       <c r="L16" t="s">
-        <v>637</v>
+        <v>630</v>
       </c>
       <c r="N16">
         <v>19</v>
       </c>
       <c r="O16" t="s">
-        <v>656</v>
+        <v>649</v>
       </c>
     </row>
     <row r="17" spans="8:15" x14ac:dyDescent="0.25">
@@ -10151,13 +10172,13 @@
         <v>25</v>
       </c>
       <c r="I18" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="K18">
         <v>25</v>
       </c>
       <c r="L18" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="N18">
         <v>25</v>
@@ -10168,27 +10189,27 @@
     </row>
     <row r="22" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I22" t="s">
-        <v>742</v>
+        <v>735</v>
       </c>
     </row>
     <row r="23" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I23" t="s">
-        <v>744</v>
+        <v>737</v>
       </c>
     </row>
     <row r="24" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I24" t="s">
-        <v>745</v>
+        <v>738</v>
       </c>
     </row>
     <row r="25" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I25" t="s">
-        <v>743</v>
+        <v>736</v>
       </c>
     </row>
     <row r="26" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I26" t="s">
-        <v>657</v>
+        <v>650</v>
       </c>
     </row>
   </sheetData>
@@ -10398,7 +10419,7 @@
         <v>10</v>
       </c>
       <c r="F12" t="s">
-        <v>765</v>
+        <v>758</v>
       </c>
       <c r="H12">
         <v>12</v>
@@ -10430,7 +10451,7 @@
         <v>15</v>
       </c>
       <c r="F13" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="H13">
         <v>14</v>
@@ -10456,7 +10477,7 @@
         <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>764</v>
+        <v>757</v>
       </c>
       <c r="E14">
         <v>16</v>
@@ -10506,7 +10527,7 @@
         <v>16</v>
       </c>
       <c r="L15" t="s">
-        <v>766</v>
+        <v>759</v>
       </c>
       <c r="N15">
         <v>20</v>
@@ -10584,7 +10605,7 @@
         <v>25</v>
       </c>
       <c r="O18" t="s">
-        <v>727</v>
+        <v>720</v>
       </c>
     </row>
   </sheetData>
@@ -10693,7 +10714,7 @@
         <v>1</v>
       </c>
       <c r="L9" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
@@ -10745,7 +10766,7 @@
         <v>5</v>
       </c>
       <c r="L11" t="s">
-        <v>589</v>
+        <v>586</v>
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
@@ -10753,13 +10774,13 @@
         <v>10</v>
       </c>
       <c r="C12" t="s">
-        <v>754</v>
+        <v>747</v>
       </c>
       <c r="E12">
         <v>12</v>
       </c>
       <c r="F12" t="s">
-        <v>755</v>
+        <v>748</v>
       </c>
       <c r="H12">
         <v>12</v>
@@ -10771,7 +10792,7 @@
         <v>8</v>
       </c>
       <c r="L12" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
@@ -10797,7 +10818,7 @@
         <v>10</v>
       </c>
       <c r="L13" t="s">
-        <v>587</v>
+        <v>584</v>
       </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
@@ -10811,13 +10832,13 @@
         <v>17</v>
       </c>
       <c r="F14" s="39" t="s">
-        <v>790</v>
+        <v>783</v>
       </c>
       <c r="H14">
         <v>15</v>
       </c>
       <c r="I14" t="s">
-        <v>692</v>
+        <v>685</v>
       </c>
       <c r="K14">
         <v>15</v>
@@ -10863,7 +10884,7 @@
         <v>20</v>
       </c>
       <c r="F16" t="s">
-        <v>292</v>
+        <v>340</v>
       </c>
       <c r="H16">
         <v>20</v>
@@ -11125,13 +11146,13 @@
         <v>8</v>
       </c>
       <c r="R10" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="T10">
         <v>8</v>
       </c>
       <c r="U10" t="s">
-        <v>368</v>
+        <v>798</v>
       </c>
     </row>
     <row r="11" spans="2:21" x14ac:dyDescent="0.25">
@@ -11157,25 +11178,25 @@
         <v>10</v>
       </c>
       <c r="L11" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
       <c r="N11">
         <v>9</v>
       </c>
       <c r="O11" t="s">
-        <v>777</v>
+        <v>770</v>
       </c>
       <c r="Q11">
         <v>9</v>
       </c>
       <c r="R11" t="s">
-        <v>777</v>
+        <v>770</v>
       </c>
       <c r="T11">
         <v>9</v>
       </c>
       <c r="U11" t="s">
-        <v>777</v>
+        <v>770</v>
       </c>
     </row>
     <row r="12" spans="2:21" x14ac:dyDescent="0.25">
@@ -11213,13 +11234,13 @@
         <v>12</v>
       </c>
       <c r="R12" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="T12">
         <v>12</v>
       </c>
       <c r="U12" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
     </row>
     <row r="13" spans="2:21" x14ac:dyDescent="0.25">
@@ -11251,19 +11272,19 @@
         <v>14</v>
       </c>
       <c r="O13" t="s">
-        <v>366</v>
+        <v>788</v>
       </c>
       <c r="Q13">
         <v>14</v>
       </c>
       <c r="R13" t="s">
-        <v>375</v>
+        <v>790</v>
       </c>
       <c r="T13">
         <v>14</v>
       </c>
       <c r="U13" t="s">
-        <v>369</v>
+        <v>792</v>
       </c>
     </row>
     <row r="14" spans="2:21" x14ac:dyDescent="0.25">
@@ -11301,13 +11322,13 @@
         <v>15</v>
       </c>
       <c r="R14" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="T14">
         <v>15</v>
       </c>
       <c r="U14" t="s">
-        <v>370</v>
+        <v>791</v>
       </c>
     </row>
     <row r="15" spans="2:21" x14ac:dyDescent="0.25">
@@ -11321,7 +11342,7 @@
         <v>19</v>
       </c>
       <c r="F15" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="H15">
         <v>19</v>
@@ -11339,19 +11360,19 @@
         <v>17</v>
       </c>
       <c r="O15" t="s">
-        <v>721</v>
+        <v>714</v>
       </c>
       <c r="Q15">
         <v>17</v>
       </c>
       <c r="R15" t="s">
-        <v>720</v>
+        <v>713</v>
       </c>
       <c r="T15">
         <v>17</v>
       </c>
       <c r="U15" t="s">
-        <v>722</v>
+        <v>715</v>
       </c>
     </row>
     <row r="16" spans="2:21" x14ac:dyDescent="0.25">
@@ -11359,7 +11380,7 @@
         <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="E16">
         <v>20</v>
@@ -11383,19 +11404,19 @@
         <v>21</v>
       </c>
       <c r="O16" t="s">
-        <v>367</v>
+        <v>789</v>
       </c>
       <c r="Q16">
         <v>21</v>
       </c>
       <c r="R16" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="T16">
         <v>21</v>
       </c>
       <c r="U16" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
     </row>
     <row r="17" spans="9:21" x14ac:dyDescent="0.25">
@@ -11403,19 +11424,19 @@
         <v>22</v>
       </c>
       <c r="O17" t="s">
-        <v>717</v>
+        <v>710</v>
       </c>
       <c r="Q17">
         <v>22</v>
       </c>
       <c r="R17" t="s">
-        <v>718</v>
+        <v>711</v>
       </c>
       <c r="T17">
         <v>22</v>
       </c>
       <c r="U17" t="s">
-        <v>719</v>
+        <v>712</v>
       </c>
     </row>
     <row r="18" spans="9:21" x14ac:dyDescent="0.25">
@@ -11423,19 +11444,29 @@
         <v>25</v>
       </c>
       <c r="O18" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="Q18">
         <v>25</v>
       </c>
       <c r="R18" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="T18">
         <v>25</v>
       </c>
       <c r="U18" t="s">
-        <v>371</v>
+        <v>368</v>
+      </c>
+    </row>
+    <row r="20" spans="9:21" x14ac:dyDescent="0.25">
+      <c r="R20" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="21" spans="9:21" x14ac:dyDescent="0.25">
+      <c r="R21" t="s">
+        <v>800</v>
       </c>
     </row>
     <row r="24" spans="9:21" x14ac:dyDescent="0.25">
@@ -11465,12 +11496,12 @@
     </row>
     <row r="29" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I29" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
     </row>
     <row r="30" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I30" t="s">
-        <v>595</v>
+        <v>592</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
invocación y ultmos pulidos excel
</commit_message>
<xml_diff>
--- a/arquetiposZ.xlsx
+++ b/arquetiposZ.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sergius\Desktop\Proyectos\hyperbole\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CEB77C5-2DEA-496F-9AEE-C3E0889762C1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1353EF6-C2CB-4A48-AF6E-B8D962E7D4D1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="644" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="644" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RESUMEN" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1145" uniqueCount="811">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1145" uniqueCount="812">
   <si>
     <t>daños:</t>
   </si>
@@ -1612,15 +1612,6 @@
     <t>mas daño invocs</t>
   </si>
   <si>
-    <t>invoc hielo medium todos IR</t>
-  </si>
-  <si>
-    <t>invoc frei grave uno IR</t>
-  </si>
-  <si>
-    <t>invoc viento medium x2-3 uno IR</t>
-  </si>
-  <si>
     <t>invoc mediarahan + lluvia amrita</t>
   </si>
   <si>
@@ -2116,18 +2107,9 @@
     <t>invoc psio grave todos IR</t>
   </si>
   <si>
-    <t>invoc fuego grave uno x2-3 IR miedo</t>
-  </si>
-  <si>
     <t>masamarecarm</t>
   </si>
   <si>
-    <t>invoc eiga medio x3 uno IR desesp</t>
-  </si>
-  <si>
-    <t>invoc hielo leve x4-5 todos IR</t>
-  </si>
-  <si>
     <t>invoc viento leve x10-15 uno IR</t>
   </si>
   <si>
@@ -2146,12 +2128,6 @@
     <t>invoc cort mag light uno IR</t>
   </si>
   <si>
-    <t>invoc trueno grave todos IR amnesia</t>
-  </si>
-  <si>
-    <t>invoc kouga sever uno IR mareo</t>
-  </si>
-  <si>
     <t>invoc frei sever uno IR quem</t>
   </si>
   <si>
@@ -2477,6 +2453,33 @@
   </si>
   <si>
     <t>usar dos objetos</t>
+  </si>
+  <si>
+    <t>drain boost</t>
+  </si>
+  <si>
+    <t>invoc trueno osc medium todos IR</t>
+  </si>
+  <si>
+    <t>invoc hielo nuc medium x2 uno IR</t>
+  </si>
+  <si>
+    <t>invoc fuego sever uno IR miedo</t>
+  </si>
+  <si>
+    <t>invoc trueno grave todos IR brainw</t>
+  </si>
+  <si>
+    <t>invoc eiga grave todos x2-3 IR desesp</t>
+  </si>
+  <si>
+    <t>invocar noctiluca</t>
+  </si>
+  <si>
+    <t>invoc kouga medio x3 uno IR sleep</t>
+  </si>
+  <si>
+    <t>invoc hielo leve x4-5 todos IR mareo</t>
   </si>
 </sst>
 </file>
@@ -4361,7 +4364,7 @@
         <v>54</v>
       </c>
       <c r="L31" s="5" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="M31" s="5"/>
       <c r="N31" s="5"/>
@@ -4388,7 +4391,7 @@
         <v>55</v>
       </c>
       <c r="L32" s="5" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="M32" s="5"/>
       <c r="N32" s="5"/>
@@ -4417,7 +4420,7 @@
         <v>66</v>
       </c>
       <c r="L33" s="5" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="M33" s="5"/>
       <c r="N33" s="5"/>
@@ -4743,7 +4746,7 @@
         <v>15</v>
       </c>
       <c r="G12" t="s">
-        <v>751</v>
+        <v>743</v>
       </c>
       <c r="J12">
         <v>10</v>
@@ -4825,7 +4828,7 @@
         <v>24</v>
       </c>
       <c r="K17" t="s">
-        <v>795</v>
+        <v>787</v>
       </c>
     </row>
     <row r="18" spans="8:11" x14ac:dyDescent="0.25">
@@ -4868,7 +4871,7 @@
     </row>
     <row r="30" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H30" t="s">
-        <v>752</v>
+        <v>744</v>
       </c>
     </row>
     <row r="31" spans="8:11" x14ac:dyDescent="0.25">
@@ -4878,7 +4881,7 @@
     </row>
     <row r="32" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H32" t="s">
-        <v>740</v>
+        <v>732</v>
       </c>
     </row>
     <row r="33" spans="8:8" x14ac:dyDescent="0.25">
@@ -4957,7 +4960,7 @@
         <v>1</v>
       </c>
       <c r="O7" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="Q7">
         <v>1</v>
@@ -5133,13 +5136,13 @@
         <v>9</v>
       </c>
       <c r="O11" t="s">
-        <v>749</v>
+        <v>741</v>
       </c>
       <c r="Q11">
         <v>10</v>
       </c>
       <c r="R11" t="s">
-        <v>679</v>
+        <v>676</v>
       </c>
       <c r="T11">
         <v>6</v>
@@ -5165,7 +5168,7 @@
         <v>10</v>
       </c>
       <c r="I12" t="s">
-        <v>781</v>
+        <v>773</v>
       </c>
       <c r="K12">
         <v>12</v>
@@ -5177,7 +5180,7 @@
         <v>10</v>
       </c>
       <c r="O12" t="s">
-        <v>747</v>
+        <v>739</v>
       </c>
       <c r="Q12">
         <v>12</v>
@@ -5209,7 +5212,7 @@
         <v>10</v>
       </c>
       <c r="I13" t="s">
-        <v>782</v>
+        <v>774</v>
       </c>
       <c r="K13">
         <v>14</v>
@@ -5221,7 +5224,7 @@
         <v>11</v>
       </c>
       <c r="O13" t="s">
-        <v>746</v>
+        <v>738</v>
       </c>
       <c r="Q13">
         <v>14</v>
@@ -5241,7 +5244,7 @@
         <v>13</v>
       </c>
       <c r="C14" s="39" t="s">
-        <v>766</v>
+        <v>758</v>
       </c>
       <c r="E14">
         <v>16</v>
@@ -5259,13 +5262,13 @@
         <v>15</v>
       </c>
       <c r="L14" t="s">
-        <v>804</v>
+        <v>796</v>
       </c>
       <c r="N14">
         <v>12</v>
       </c>
       <c r="O14" t="s">
-        <v>748</v>
+        <v>740</v>
       </c>
       <c r="Q14">
         <v>15</v>
@@ -5291,7 +5294,7 @@
         <v>18</v>
       </c>
       <c r="F15" t="s">
-        <v>803</v>
+        <v>795</v>
       </c>
       <c r="H15">
         <v>16</v>
@@ -5303,7 +5306,7 @@
         <v>16</v>
       </c>
       <c r="L15" t="s">
-        <v>796</v>
+        <v>788</v>
       </c>
       <c r="N15">
         <v>13</v>
@@ -5341,13 +5344,13 @@
         <v>20</v>
       </c>
       <c r="L16" t="s">
-        <v>753</v>
+        <v>745</v>
       </c>
       <c r="N16">
         <v>15</v>
       </c>
       <c r="O16" t="s">
-        <v>742</v>
+        <v>734</v>
       </c>
       <c r="Q16">
         <v>20</v>
@@ -5373,7 +5376,7 @@
         <v>20</v>
       </c>
       <c r="O17" t="s">
-        <v>802</v>
+        <v>794</v>
       </c>
       <c r="Q17">
         <v>23</v>
@@ -5411,7 +5414,7 @@
         <v>25</v>
       </c>
       <c r="U18" t="s">
-        <v>704</v>
+        <v>696</v>
       </c>
     </row>
     <row r="21" spans="9:21" x14ac:dyDescent="0.25">
@@ -5496,7 +5499,7 @@
     </row>
     <row r="37" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I37" t="s">
-        <v>705</v>
+        <v>697</v>
       </c>
     </row>
   </sheetData>
@@ -5561,7 +5564,7 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>524</v>
+        <v>805</v>
       </c>
       <c r="H7">
         <v>1</v>
@@ -5573,7 +5576,7 @@
         <v>1</v>
       </c>
       <c r="L7" t="s">
-        <v>695</v>
+        <v>689</v>
       </c>
       <c r="N7">
         <v>1</v>
@@ -5585,13 +5588,13 @@
         <v>1</v>
       </c>
       <c r="R7" t="s">
-        <v>772</v>
+        <v>764</v>
       </c>
       <c r="T7">
         <v>1</v>
       </c>
       <c r="U7" s="39" t="s">
-        <v>779</v>
+        <v>771</v>
       </c>
     </row>
     <row r="8" spans="2:21" x14ac:dyDescent="0.25">
@@ -5602,7 +5605,7 @@
         <v>275</v>
       </c>
       <c r="E8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F8" t="s">
         <v>239</v>
@@ -5617,36 +5620,36 @@
         <v>1</v>
       </c>
       <c r="L8" t="s">
-        <v>696</v>
+        <v>690</v>
       </c>
       <c r="N8">
         <v>1</v>
       </c>
       <c r="O8" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
       <c r="Q8">
         <v>1</v>
       </c>
       <c r="R8" t="s">
-        <v>773</v>
+        <v>765</v>
       </c>
       <c r="T8">
         <v>1</v>
       </c>
       <c r="U8" t="s">
-        <v>777</v>
+        <v>769</v>
       </c>
     </row>
     <row r="9" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C9" t="s">
-        <v>697</v>
+        <v>691</v>
       </c>
       <c r="E9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F9" t="s">
         <v>282</v>
@@ -5673,27 +5676,27 @@
         <v>1</v>
       </c>
       <c r="R9" t="s">
-        <v>774</v>
+        <v>766</v>
       </c>
       <c r="T9">
         <v>1</v>
       </c>
       <c r="U9" t="s">
-        <v>778</v>
+        <v>770</v>
       </c>
     </row>
     <row r="10" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B10">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>698</v>
+        <v>692</v>
       </c>
       <c r="E10">
         <v>5</v>
       </c>
       <c r="F10" t="s">
-        <v>523</v>
+        <v>809</v>
       </c>
       <c r="H10">
         <v>7</v>
@@ -5705,22 +5708,22 @@
         <v>5</v>
       </c>
       <c r="L10" t="s">
-        <v>694</v>
+        <v>686</v>
       </c>
       <c r="N10">
         <v>5</v>
       </c>
       <c r="O10" t="s">
-        <v>296</v>
+        <v>803</v>
       </c>
       <c r="Q10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R10" t="s">
         <v>176</v>
       </c>
       <c r="T10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U10" t="s">
         <v>177</v>
@@ -5731,13 +5734,13 @@
         <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>699</v>
+        <v>693</v>
       </c>
       <c r="E11">
         <v>10</v>
       </c>
       <c r="F11" t="s">
-        <v>522</v>
+        <v>804</v>
       </c>
       <c r="H11">
         <v>10</v>
@@ -5746,10 +5749,10 @@
         <v>298</v>
       </c>
       <c r="K11">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L11" t="s">
-        <v>689</v>
+        <v>522</v>
       </c>
       <c r="N11">
         <v>10</v>
@@ -5761,13 +5764,13 @@
         <v>7</v>
       </c>
       <c r="R11" t="s">
-        <v>654</v>
+        <v>651</v>
       </c>
       <c r="T11">
         <v>7</v>
       </c>
       <c r="U11" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
     </row>
     <row r="12" spans="2:21" x14ac:dyDescent="0.25">
@@ -5778,10 +5781,10 @@
         <v>168</v>
       </c>
       <c r="E12">
-        <v>13</v>
-      </c>
-      <c r="F12" t="s">
-        <v>727</v>
+        <v>12</v>
+      </c>
+      <c r="F12" s="39" t="s">
+        <v>759</v>
       </c>
       <c r="H12">
         <v>15</v>
@@ -5790,10 +5793,10 @@
         <v>172</v>
       </c>
       <c r="K12">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="L12" t="s">
-        <v>692</v>
+        <v>810</v>
       </c>
       <c r="N12">
         <v>12</v>
@@ -5825,7 +5828,7 @@
         <v>17</v>
       </c>
       <c r="F13" t="s">
-        <v>525</v>
+        <v>521</v>
       </c>
       <c r="H13">
         <v>15</v>
@@ -5834,10 +5837,10 @@
         <v>173</v>
       </c>
       <c r="K13">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="L13" t="s">
-        <v>700</v>
+        <v>807</v>
       </c>
       <c r="N13">
         <v>12</v>
@@ -5849,7 +5852,7 @@
         <v>11</v>
       </c>
       <c r="R13" t="s">
-        <v>728</v>
+        <v>720</v>
       </c>
       <c r="T13">
         <v>11</v>
@@ -5863,31 +5866,31 @@
         <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
       <c r="E14">
         <v>18</v>
       </c>
       <c r="F14" t="s">
-        <v>521</v>
+        <v>293</v>
       </c>
       <c r="H14">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I14" t="s">
-        <v>769</v>
+        <v>761</v>
       </c>
       <c r="K14">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="L14" t="s">
-        <v>701</v>
+        <v>806</v>
       </c>
       <c r="N14">
         <v>15</v>
       </c>
       <c r="O14" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="Q14">
         <v>12</v>
@@ -5907,25 +5910,25 @@
         <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>546</v>
+        <v>543</v>
       </c>
       <c r="E15">
         <v>19</v>
       </c>
       <c r="F15" t="s">
-        <v>293</v>
+        <v>520</v>
       </c>
       <c r="H15">
         <v>20</v>
       </c>
       <c r="I15" t="s">
-        <v>770</v>
+        <v>762</v>
       </c>
       <c r="K15">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="L15" t="s">
-        <v>690</v>
+        <v>808</v>
       </c>
       <c r="N15">
         <v>18</v>
@@ -5950,26 +5953,26 @@
       <c r="B16">
         <v>15</v>
       </c>
-      <c r="C16" s="39" t="s">
-        <v>767</v>
+      <c r="C16" t="s">
+        <v>719</v>
       </c>
       <c r="E16">
         <v>20</v>
       </c>
       <c r="F16" t="s">
-        <v>520</v>
+        <v>688</v>
       </c>
       <c r="H16">
         <v>20</v>
       </c>
       <c r="I16" t="s">
-        <v>771</v>
+        <v>763</v>
       </c>
       <c r="K16">
         <v>21</v>
       </c>
       <c r="L16" t="s">
-        <v>693</v>
+        <v>811</v>
       </c>
       <c r="N16">
         <v>20</v>
@@ -5987,7 +5990,7 @@
         <v>19</v>
       </c>
       <c r="U16" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
     </row>
     <row r="17" spans="10:21" x14ac:dyDescent="0.25">
@@ -5995,7 +5998,7 @@
         <v>22</v>
       </c>
       <c r="L17" t="s">
-        <v>702</v>
+        <v>694</v>
       </c>
       <c r="N17">
         <v>20</v>
@@ -6021,7 +6024,7 @@
         <v>25</v>
       </c>
       <c r="L18" t="s">
-        <v>703</v>
+        <v>695</v>
       </c>
       <c r="N18">
         <v>25</v>
@@ -6059,22 +6062,22 @@
     </row>
     <row r="25" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J25" t="s">
-        <v>775</v>
+        <v>767</v>
       </c>
     </row>
     <row r="26" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J26" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
     </row>
     <row r="27" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J27" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
     </row>
     <row r="28" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J28" t="s">
-        <v>776</v>
+        <v>768</v>
       </c>
     </row>
     <row r="29" spans="10:21" x14ac:dyDescent="0.25">
@@ -6089,27 +6092,27 @@
     </row>
     <row r="31" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J31" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
     </row>
     <row r="32" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J32" t="s">
-        <v>656</v>
+        <v>653</v>
       </c>
     </row>
     <row r="33" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J33" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
     </row>
     <row r="34" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J34" t="s">
-        <v>659</v>
+        <v>656</v>
       </c>
     </row>
     <row r="35" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J35" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
     </row>
   </sheetData>
@@ -6144,13 +6147,13 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>799</v>
+        <v>791</v>
       </c>
       <c r="J7">
         <v>1</v>
@@ -6164,7 +6167,7 @@
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>628</v>
+        <v>625</v>
       </c>
       <c r="F8">
         <v>1</v>
@@ -6184,19 +6187,19 @@
         <v>5</v>
       </c>
       <c r="C9" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="F9">
         <v>3</v>
       </c>
       <c r="G9" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="J9">
         <v>7</v>
       </c>
       <c r="K9" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.25">
@@ -6210,7 +6213,7 @@
         <v>6</v>
       </c>
       <c r="G10" t="s">
-        <v>635</v>
+        <v>632</v>
       </c>
       <c r="J10">
         <v>8</v>
@@ -6224,19 +6227,19 @@
         <v>7</v>
       </c>
       <c r="C11" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="F11">
         <v>7</v>
       </c>
       <c r="G11" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
       <c r="J11">
         <v>11</v>
       </c>
       <c r="K11" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.25">
@@ -6244,19 +6247,19 @@
         <v>8</v>
       </c>
       <c r="C12" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
       <c r="F12">
         <v>8</v>
       </c>
       <c r="G12" t="s">
-        <v>800</v>
+        <v>792</v>
       </c>
       <c r="J12">
         <v>11</v>
       </c>
       <c r="K12" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.25">
@@ -6264,7 +6267,7 @@
         <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
       <c r="F13">
         <v>12</v>
@@ -6276,7 +6279,7 @@
         <v>13</v>
       </c>
       <c r="K13" t="s">
-        <v>688</v>
+        <v>685</v>
       </c>
     </row>
     <row r="14" spans="2:11" x14ac:dyDescent="0.25">
@@ -6290,13 +6293,13 @@
         <v>16</v>
       </c>
       <c r="G14" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="J14">
         <v>15</v>
       </c>
       <c r="K14" t="s">
-        <v>741</v>
+        <v>733</v>
       </c>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.25">
@@ -6304,19 +6307,19 @@
         <v>13</v>
       </c>
       <c r="C15" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
       <c r="F15">
         <v>19</v>
       </c>
       <c r="G15" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
       <c r="J15">
         <v>18</v>
       </c>
       <c r="K15" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.25">
@@ -6324,7 +6327,7 @@
         <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
       <c r="F16">
         <v>20</v>
@@ -6336,7 +6339,7 @@
         <v>20</v>
       </c>
       <c r="K16" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
     </row>
     <row r="17" spans="10:11" x14ac:dyDescent="0.25">
@@ -6344,7 +6347,7 @@
         <v>20</v>
       </c>
       <c r="K17" t="s">
-        <v>638</v>
+        <v>635</v>
       </c>
     </row>
     <row r="18" spans="10:11" x14ac:dyDescent="0.25">
@@ -6352,27 +6355,27 @@
         <v>25</v>
       </c>
       <c r="K18" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
     </row>
     <row r="27" spans="10:11" x14ac:dyDescent="0.25">
       <c r="K27" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
     </row>
     <row r="28" spans="10:11" x14ac:dyDescent="0.25">
       <c r="K28" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
     </row>
     <row r="29" spans="10:11" x14ac:dyDescent="0.25">
       <c r="K29" t="s">
-        <v>630</v>
+        <v>627</v>
       </c>
     </row>
     <row r="30" spans="10:11" x14ac:dyDescent="0.25">
       <c r="K30" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
     </row>
   </sheetData>
@@ -6414,7 +6417,7 @@
         <v>55</v>
       </c>
       <c r="R6" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="V6" t="s">
         <v>66</v>
@@ -6425,7 +6428,7 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -6437,13 +6440,13 @@
         <v>1</v>
       </c>
       <c r="I7" t="s">
+        <v>534</v>
+      </c>
+      <c r="K7">
+        <v>1</v>
+      </c>
+      <c r="L7" t="s">
         <v>537</v>
-      </c>
-      <c r="K7">
-        <v>1</v>
-      </c>
-      <c r="L7" t="s">
-        <v>540</v>
       </c>
       <c r="N7">
         <v>1</v>
@@ -6455,13 +6458,13 @@
         <v>1</v>
       </c>
       <c r="R7" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="U7">
         <v>1</v>
       </c>
       <c r="V7" t="s">
-        <v>723</v>
+        <v>715</v>
       </c>
     </row>
     <row r="8" spans="2:22" x14ac:dyDescent="0.25">
@@ -6469,7 +6472,7 @@
         <v>3</v>
       </c>
       <c r="C8" t="s">
-        <v>590</v>
+        <v>587</v>
       </c>
       <c r="E8">
         <v>4</v>
@@ -6481,13 +6484,13 @@
         <v>1</v>
       </c>
       <c r="I8" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="K8">
         <v>1</v>
       </c>
       <c r="L8" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="N8">
         <v>1</v>
@@ -6499,13 +6502,13 @@
         <v>3</v>
       </c>
       <c r="R8" t="s">
-        <v>720</v>
+        <v>712</v>
       </c>
       <c r="U8">
         <v>2</v>
       </c>
       <c r="V8" t="s">
-        <v>715</v>
+        <v>707</v>
       </c>
     </row>
     <row r="9" spans="2:22" x14ac:dyDescent="0.25">
@@ -6513,13 +6516,13 @@
         <v>5</v>
       </c>
       <c r="C9" t="s">
-        <v>710</v>
+        <v>702</v>
       </c>
       <c r="E9">
         <v>4</v>
       </c>
       <c r="F9" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
       <c r="H9">
         <v>4</v>
@@ -6543,13 +6546,13 @@
         <v>5</v>
       </c>
       <c r="R9" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="U9">
         <v>2</v>
       </c>
       <c r="V9" t="s">
-        <v>711</v>
+        <v>703</v>
       </c>
     </row>
     <row r="10" spans="2:22" x14ac:dyDescent="0.25">
@@ -6557,31 +6560,31 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="E10">
         <v>6</v>
       </c>
       <c r="F10" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
       <c r="H10">
         <v>5</v>
       </c>
       <c r="I10" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="K10">
         <v>8</v>
       </c>
       <c r="L10" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="N10">
         <v>8</v>
       </c>
       <c r="O10" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
       <c r="Q10">
         <v>8</v>
@@ -6593,7 +6596,7 @@
         <v>6</v>
       </c>
       <c r="V10" t="s">
-        <v>721</v>
+        <v>713</v>
       </c>
     </row>
     <row r="11" spans="2:22" x14ac:dyDescent="0.25">
@@ -6601,13 +6604,13 @@
         <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>576</v>
+        <v>573</v>
       </c>
       <c r="E11">
         <v>8</v>
       </c>
       <c r="F11" t="s">
-        <v>592</v>
+        <v>589</v>
       </c>
       <c r="H11">
         <v>7</v>
@@ -6631,13 +6634,13 @@
         <v>10</v>
       </c>
       <c r="R11" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="U11">
         <v>7</v>
       </c>
       <c r="V11" t="s">
-        <v>729</v>
+        <v>721</v>
       </c>
     </row>
     <row r="12" spans="2:22" x14ac:dyDescent="0.25">
@@ -6645,13 +6648,13 @@
         <v>10</v>
       </c>
       <c r="C12" t="s">
-        <v>716</v>
+        <v>708</v>
       </c>
       <c r="E12">
         <v>11</v>
       </c>
       <c r="F12" t="s">
-        <v>594</v>
+        <v>591</v>
       </c>
       <c r="H12">
         <v>8</v>
@@ -6663,25 +6666,25 @@
         <v>12</v>
       </c>
       <c r="L12" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="N12">
         <v>12</v>
       </c>
       <c r="O12" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="Q12">
         <v>12</v>
       </c>
       <c r="R12" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="U12">
         <v>8</v>
       </c>
       <c r="V12" t="s">
-        <v>712</v>
+        <v>704</v>
       </c>
     </row>
     <row r="13" spans="2:22" x14ac:dyDescent="0.25">
@@ -6689,43 +6692,43 @@
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
       <c r="E13">
         <v>14</v>
       </c>
       <c r="F13" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="H13">
         <v>9</v>
       </c>
       <c r="I13" t="s">
-        <v>733</v>
+        <v>725</v>
       </c>
       <c r="K13">
         <v>14</v>
       </c>
       <c r="L13" t="s">
-        <v>595</v>
+        <v>592</v>
       </c>
       <c r="N13">
         <v>14</v>
       </c>
       <c r="O13" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="Q13">
         <v>14</v>
       </c>
       <c r="R13" t="s">
-        <v>809</v>
+        <v>801</v>
       </c>
       <c r="U13">
         <v>9</v>
       </c>
       <c r="V13" t="s">
-        <v>806</v>
+        <v>798</v>
       </c>
     </row>
     <row r="14" spans="2:22" x14ac:dyDescent="0.25">
@@ -6733,7 +6736,7 @@
         <v>14</v>
       </c>
       <c r="C14" t="s">
-        <v>731</v>
+        <v>723</v>
       </c>
       <c r="E14">
         <v>16</v>
@@ -6745,7 +6748,7 @@
         <v>11</v>
       </c>
       <c r="I14" t="s">
-        <v>714</v>
+        <v>706</v>
       </c>
       <c r="K14">
         <v>15</v>
@@ -6763,13 +6766,13 @@
         <v>15</v>
       </c>
       <c r="R14" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="U14">
         <v>14</v>
       </c>
       <c r="V14" t="s">
-        <v>725</v>
+        <v>717</v>
       </c>
     </row>
     <row r="15" spans="2:22" x14ac:dyDescent="0.25">
@@ -6777,43 +6780,43 @@
         <v>15</v>
       </c>
       <c r="C15" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
       <c r="E15">
         <v>18</v>
       </c>
       <c r="F15" t="s">
-        <v>717</v>
+        <v>709</v>
       </c>
       <c r="H15">
         <v>16</v>
       </c>
       <c r="I15" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="K15">
         <v>20</v>
       </c>
       <c r="L15" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="N15">
         <v>16</v>
       </c>
       <c r="O15" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="Q15">
         <v>16</v>
       </c>
       <c r="R15" t="s">
-        <v>724</v>
+        <v>716</v>
       </c>
       <c r="U15">
         <v>17</v>
       </c>
       <c r="V15" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
     </row>
     <row r="16" spans="2:22" x14ac:dyDescent="0.25">
@@ -6827,31 +6830,31 @@
         <v>20</v>
       </c>
       <c r="I16" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="K16">
         <v>20</v>
       </c>
       <c r="L16" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="N16">
         <v>20</v>
       </c>
       <c r="O16" t="s">
-        <v>625</v>
+        <v>622</v>
       </c>
       <c r="Q16">
         <v>20</v>
       </c>
       <c r="R16" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="U16">
         <v>20</v>
       </c>
       <c r="V16" t="s">
-        <v>713</v>
+        <v>705</v>
       </c>
     </row>
     <row r="17" spans="11:22" x14ac:dyDescent="0.25">
@@ -6859,25 +6862,25 @@
         <v>24</v>
       </c>
       <c r="L17" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="N17">
         <v>23</v>
       </c>
       <c r="O17" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="Q17">
         <v>24</v>
       </c>
       <c r="R17" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="U17">
         <v>24</v>
       </c>
       <c r="V17" t="s">
-        <v>722</v>
+        <v>714</v>
       </c>
     </row>
     <row r="18" spans="11:22" x14ac:dyDescent="0.25">
@@ -6885,75 +6888,75 @@
         <v>25</v>
       </c>
       <c r="L18" t="s">
-        <v>597</v>
+        <v>594</v>
       </c>
       <c r="N18">
         <v>25</v>
       </c>
       <c r="O18" t="s">
-        <v>744</v>
+        <v>736</v>
       </c>
       <c r="Q18">
         <v>25</v>
       </c>
       <c r="R18" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="U18">
         <v>25</v>
       </c>
       <c r="V18" t="s">
-        <v>730</v>
+        <v>722</v>
       </c>
     </row>
     <row r="22" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L22" t="s">
-        <v>745</v>
+        <v>737</v>
       </c>
     </row>
     <row r="23" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L23" t="s">
-        <v>732</v>
+        <v>724</v>
       </c>
     </row>
     <row r="24" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L24" t="s">
-        <v>734</v>
+        <v>726</v>
       </c>
     </row>
     <row r="25" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L25" t="s">
-        <v>591</v>
+        <v>588</v>
       </c>
     </row>
     <row r="26" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L26" t="s">
-        <v>593</v>
+        <v>590</v>
       </c>
     </row>
     <row r="27" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L27" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
     </row>
     <row r="28" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L28" t="s">
-        <v>798</v>
+        <v>790</v>
       </c>
     </row>
     <row r="29" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L29" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
     </row>
     <row r="30" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L30" t="s">
-        <v>801</v>
+        <v>793</v>
       </c>
     </row>
     <row r="33" spans="13:13" x14ac:dyDescent="0.25">
       <c r="M33" t="s">
-        <v>726</v>
+        <v>718</v>
       </c>
     </row>
   </sheetData>
@@ -7001,19 +7004,19 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
+        <v>549</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7" t="s">
+        <v>582</v>
+      </c>
+      <c r="K7">
+        <v>1</v>
+      </c>
+      <c r="L7" t="s">
         <v>552</v>
-      </c>
-      <c r="H7">
-        <v>1</v>
-      </c>
-      <c r="I7" t="s">
-        <v>585</v>
-      </c>
-      <c r="K7">
-        <v>1</v>
-      </c>
-      <c r="L7" t="s">
-        <v>555</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
@@ -7027,19 +7030,19 @@
         <v>2</v>
       </c>
       <c r="F8" s="39" t="s">
-        <v>763</v>
+        <v>755</v>
       </c>
       <c r="H8">
         <v>2</v>
       </c>
       <c r="I8" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="K8">
         <v>1</v>
       </c>
       <c r="L8" t="s">
-        <v>589</v>
+        <v>586</v>
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
@@ -7053,7 +7056,7 @@
         <v>3</v>
       </c>
       <c r="F9" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
       <c r="H9">
         <v>5</v>
@@ -7065,7 +7068,7 @@
         <v>3</v>
       </c>
       <c r="L9" t="s">
-        <v>674</v>
+        <v>671</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
@@ -7073,7 +7076,7 @@
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>760</v>
+        <v>752</v>
       </c>
       <c r="E10">
         <v>4</v>
@@ -7085,13 +7088,13 @@
         <v>8</v>
       </c>
       <c r="I10" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="K10">
         <v>4</v>
       </c>
       <c r="L10" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
@@ -7099,7 +7102,7 @@
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>761</v>
+        <v>753</v>
       </c>
       <c r="E11">
         <v>10</v>
@@ -7117,7 +7120,7 @@
         <v>5</v>
       </c>
       <c r="L11" t="s">
-        <v>754</v>
+        <v>746</v>
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
@@ -7131,19 +7134,19 @@
         <v>12</v>
       </c>
       <c r="F12" t="s">
-        <v>664</v>
+        <v>661</v>
       </c>
       <c r="H12">
         <v>11</v>
       </c>
       <c r="I12" t="s">
-        <v>810</v>
+        <v>802</v>
       </c>
       <c r="K12">
         <v>8</v>
       </c>
       <c r="L12" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
@@ -7151,7 +7154,7 @@
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>762</v>
+        <v>754</v>
       </c>
       <c r="E13">
         <v>13</v>
@@ -7163,13 +7166,13 @@
         <v>14</v>
       </c>
       <c r="I13" t="s">
-        <v>666</v>
+        <v>663</v>
       </c>
       <c r="K13">
         <v>10</v>
       </c>
       <c r="L13" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
@@ -7177,13 +7180,13 @@
         <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>764</v>
+        <v>756</v>
       </c>
       <c r="E14">
         <v>16</v>
       </c>
       <c r="F14" t="s">
-        <v>663</v>
+        <v>660</v>
       </c>
       <c r="H14">
         <v>15</v>
@@ -7195,7 +7198,7 @@
         <v>15</v>
       </c>
       <c r="L14" t="s">
-        <v>672</v>
+        <v>669</v>
       </c>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.25">
@@ -7215,13 +7218,13 @@
         <v>17</v>
       </c>
       <c r="I15" t="s">
-        <v>667</v>
+        <v>664</v>
       </c>
       <c r="K15">
         <v>18</v>
       </c>
       <c r="L15" t="s">
-        <v>671</v>
+        <v>668</v>
       </c>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
@@ -7229,25 +7232,25 @@
         <v>15</v>
       </c>
       <c r="C16" s="39" t="s">
-        <v>768</v>
+        <v>760</v>
       </c>
       <c r="E16">
         <v>20</v>
       </c>
       <c r="F16" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="H16">
         <v>20</v>
       </c>
       <c r="I16" t="s">
-        <v>587</v>
+        <v>584</v>
       </c>
       <c r="K16">
         <v>20</v>
       </c>
       <c r="L16" t="s">
-        <v>805</v>
+        <v>797</v>
       </c>
     </row>
     <row r="17" spans="8:12" x14ac:dyDescent="0.25">
@@ -7255,13 +7258,13 @@
         <v>23</v>
       </c>
       <c r="I17" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="K17">
         <v>21</v>
       </c>
       <c r="L17" t="s">
-        <v>673</v>
+        <v>670</v>
       </c>
     </row>
     <row r="18" spans="8:12" x14ac:dyDescent="0.25">
@@ -7269,38 +7272,38 @@
         <v>25</v>
       </c>
       <c r="I18" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="K18">
         <v>25</v>
       </c>
       <c r="L18" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
     </row>
     <row r="22" spans="8:12" x14ac:dyDescent="0.25">
       <c r="I22" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
     </row>
     <row r="23" spans="8:12" x14ac:dyDescent="0.25">
       <c r="I23" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
     </row>
     <row r="24" spans="8:12" x14ac:dyDescent="0.25">
       <c r="I24" t="s">
-        <v>668</v>
+        <v>665</v>
       </c>
     </row>
     <row r="25" spans="8:12" x14ac:dyDescent="0.25">
       <c r="I25" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
     </row>
     <row r="26" spans="8:12" x14ac:dyDescent="0.25">
       <c r="I26" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
     </row>
   </sheetData>
@@ -8671,10 +8674,10 @@
     <row r="7" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B8" s="35" t="s">
-        <v>676</v>
+        <v>673</v>
       </c>
       <c r="C8" s="36" t="s">
-        <v>675</v>
+        <v>672</v>
       </c>
       <c r="H8" t="s">
         <v>12</v>
@@ -8854,7 +8857,7 @@
         <v>248</v>
       </c>
       <c r="M17" t="s">
-        <v>677</v>
+        <v>674</v>
       </c>
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.25">
@@ -9108,7 +9111,7 @@
         <v>63</v>
       </c>
       <c r="I32" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
       <c r="L32" t="s">
         <v>51</v>
@@ -9122,13 +9125,13 @@
         <v>515</v>
       </c>
       <c r="I33" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
       <c r="L33" t="s">
         <v>54</v>
       </c>
       <c r="M33" t="s">
-        <v>573</v>
+        <v>570</v>
       </c>
     </row>
     <row r="34" spans="8:13" x14ac:dyDescent="0.25">
@@ -9136,7 +9139,7 @@
         <v>64</v>
       </c>
       <c r="I34" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="L34" t="s">
         <v>55</v>
@@ -9150,13 +9153,13 @@
         <v>59</v>
       </c>
       <c r="I35" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="L35" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="M35" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
     </row>
     <row r="36" spans="8:13" x14ac:dyDescent="0.25">
@@ -9164,7 +9167,7 @@
         <v>58</v>
       </c>
       <c r="M36" t="s">
-        <v>584</v>
+        <v>581</v>
       </c>
     </row>
     <row r="37" spans="8:13" x14ac:dyDescent="0.25">
@@ -9172,7 +9175,7 @@
         <v>61</v>
       </c>
       <c r="M37" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
     </row>
   </sheetData>
@@ -9190,7 +9193,7 @@
   <sheetData>
     <row r="5" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>678</v>
+        <v>675</v>
       </c>
     </row>
     <row r="6" spans="2:2" x14ac:dyDescent="0.25">
@@ -9200,7 +9203,7 @@
     </row>
     <row r="8" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
     </row>
     <row r="9" spans="2:2" x14ac:dyDescent="0.25">
@@ -9230,7 +9233,7 @@
     </row>
     <row r="16" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
     </row>
   </sheetData>
@@ -9347,13 +9350,13 @@
         <v>2</v>
       </c>
       <c r="L8" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="N8">
         <v>2</v>
       </c>
       <c r="O8" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="Q8">
         <v>2</v>
@@ -9365,7 +9368,7 @@
         <v>2</v>
       </c>
       <c r="U8" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
     </row>
     <row r="9" spans="2:21" x14ac:dyDescent="0.25">
@@ -9461,19 +9464,19 @@
         <v>8</v>
       </c>
       <c r="C11" s="37" t="s">
-        <v>788</v>
+        <v>780</v>
       </c>
       <c r="E11">
         <v>8</v>
       </c>
       <c r="F11" s="37" t="s">
-        <v>789</v>
+        <v>781</v>
       </c>
       <c r="H11">
         <v>8</v>
       </c>
       <c r="I11" s="37" t="s">
-        <v>790</v>
+        <v>782</v>
       </c>
       <c r="K11">
         <v>10</v>
@@ -9511,7 +9514,7 @@
         <v>10</v>
       </c>
       <c r="F12" t="s">
-        <v>679</v>
+        <v>676</v>
       </c>
       <c r="H12">
         <v>10</v>
@@ -9567,25 +9570,25 @@
         <v>14</v>
       </c>
       <c r="L13" t="s">
-        <v>737</v>
+        <v>729</v>
       </c>
       <c r="N13">
         <v>14</v>
       </c>
       <c r="O13" t="s">
-        <v>737</v>
+        <v>729</v>
       </c>
       <c r="Q13">
         <v>14</v>
       </c>
       <c r="R13" t="s">
-        <v>737</v>
+        <v>729</v>
       </c>
       <c r="T13">
         <v>14</v>
       </c>
       <c r="U13" t="s">
-        <v>737</v>
+        <v>729</v>
       </c>
     </row>
     <row r="14" spans="2:21" x14ac:dyDescent="0.25">
@@ -9599,13 +9602,13 @@
         <v>15</v>
       </c>
       <c r="F14" s="39" t="s">
-        <v>736</v>
+        <v>728</v>
       </c>
       <c r="H14">
         <v>15</v>
       </c>
       <c r="I14" s="39" t="s">
-        <v>736</v>
+        <v>728</v>
       </c>
       <c r="K14">
         <v>15</v>
@@ -9693,25 +9696,25 @@
         <v>20</v>
       </c>
       <c r="L16" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
       <c r="N16">
         <v>20</v>
       </c>
       <c r="O16" t="s">
-        <v>619</v>
+        <v>616</v>
       </c>
       <c r="Q16">
         <v>20</v>
       </c>
       <c r="R16" t="s">
-        <v>618</v>
+        <v>615</v>
       </c>
       <c r="T16">
         <v>20</v>
       </c>
       <c r="U16" t="s">
-        <v>607</v>
+        <v>604</v>
       </c>
     </row>
     <row r="17" spans="9:21" x14ac:dyDescent="0.25">
@@ -9768,42 +9771,42 @@
     </row>
     <row r="22" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I22" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
     </row>
     <row r="23" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I23" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
     </row>
     <row r="24" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I24" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
     </row>
     <row r="25" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I25" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
     </row>
     <row r="26" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I26" t="s">
-        <v>616</v>
+        <v>613</v>
       </c>
     </row>
     <row r="27" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I27" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="28" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I28" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
     </row>
     <row r="29" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I29" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
     </row>
     <row r="36" spans="11:11" x14ac:dyDescent="0.25">
@@ -9894,7 +9897,7 @@
         <v>3</v>
       </c>
       <c r="I8" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
       <c r="K8">
         <v>3</v>
@@ -9926,13 +9929,13 @@
         <v>5</v>
       </c>
       <c r="I9" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
       <c r="K9">
         <v>5</v>
       </c>
       <c r="L9" t="s">
-        <v>622</v>
+        <v>619</v>
       </c>
       <c r="N9">
         <v>5</v>
@@ -9958,13 +9961,13 @@
         <v>8</v>
       </c>
       <c r="I10" t="s">
-        <v>680</v>
+        <v>677</v>
       </c>
       <c r="K10">
         <v>8</v>
       </c>
       <c r="L10" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
       <c r="N10">
         <v>6</v>
@@ -10048,25 +10051,25 @@
         <v>14</v>
       </c>
       <c r="F13" s="39" t="s">
-        <v>735</v>
+        <v>727</v>
       </c>
       <c r="H13">
         <v>14</v>
       </c>
       <c r="I13" t="s">
-        <v>807</v>
+        <v>799</v>
       </c>
       <c r="K13">
         <v>14</v>
       </c>
       <c r="L13" t="s">
-        <v>807</v>
+        <v>799</v>
       </c>
       <c r="N13">
         <v>14</v>
       </c>
       <c r="O13" t="s">
-        <v>808</v>
+        <v>800</v>
       </c>
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.25">
@@ -10098,7 +10101,7 @@
         <v>15</v>
       </c>
       <c r="O14" t="s">
-        <v>739</v>
+        <v>731</v>
       </c>
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.25">
@@ -10144,19 +10147,19 @@
         <v>20</v>
       </c>
       <c r="I16" t="s">
-        <v>606</v>
+        <v>603</v>
       </c>
       <c r="K16">
         <v>20</v>
       </c>
       <c r="L16" t="s">
-        <v>604</v>
+        <v>601</v>
       </c>
       <c r="N16">
         <v>21</v>
       </c>
       <c r="O16" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
     </row>
     <row r="17" spans="8:15" x14ac:dyDescent="0.25">
@@ -10201,27 +10204,27 @@
     </row>
     <row r="22" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I22" t="s">
-        <v>706</v>
+        <v>698</v>
       </c>
     </row>
     <row r="23" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I23" t="s">
-        <v>708</v>
+        <v>700</v>
       </c>
     </row>
     <row r="24" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I24" t="s">
-        <v>709</v>
+        <v>701</v>
       </c>
     </row>
     <row r="25" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I25" t="s">
-        <v>707</v>
+        <v>699</v>
       </c>
     </row>
     <row r="26" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I26" t="s">
-        <v>624</v>
+        <v>621</v>
       </c>
     </row>
   </sheetData>
@@ -10329,7 +10332,7 @@
         <v>4</v>
       </c>
       <c r="C9" t="s">
-        <v>791</v>
+        <v>783</v>
       </c>
       <c r="E9">
         <v>4</v>
@@ -10367,7 +10370,7 @@
         <v>4</v>
       </c>
       <c r="F10" t="s">
-        <v>728</v>
+        <v>720</v>
       </c>
       <c r="H10">
         <v>8</v>
@@ -10379,7 +10382,7 @@
         <v>7</v>
       </c>
       <c r="L10" t="s">
-        <v>793</v>
+        <v>785</v>
       </c>
       <c r="N10">
         <v>5</v>
@@ -10431,7 +10434,7 @@
         <v>8</v>
       </c>
       <c r="F12" t="s">
-        <v>792</v>
+        <v>784</v>
       </c>
       <c r="H12">
         <v>12</v>
@@ -10443,7 +10446,7 @@
         <v>10</v>
       </c>
       <c r="L12" t="s">
-        <v>787</v>
+        <v>779</v>
       </c>
       <c r="N12">
         <v>10</v>
@@ -10489,7 +10492,7 @@
         <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>727</v>
+        <v>719</v>
       </c>
       <c r="E14">
         <v>14</v>
@@ -10507,7 +10510,7 @@
         <v>15</v>
       </c>
       <c r="L14" t="s">
-        <v>743</v>
+        <v>735</v>
       </c>
       <c r="N14">
         <v>17</v>
@@ -10533,7 +10536,7 @@
         <v>16</v>
       </c>
       <c r="I15" t="s">
-        <v>786</v>
+        <v>778</v>
       </c>
       <c r="K15">
         <v>16</v>
@@ -10571,7 +10574,7 @@
         <v>17</v>
       </c>
       <c r="L16" t="s">
-        <v>780</v>
+        <v>772</v>
       </c>
       <c r="N16">
         <v>21</v>
@@ -10617,7 +10620,7 @@
         <v>25</v>
       </c>
       <c r="O18" t="s">
-        <v>691</v>
+        <v>687</v>
       </c>
     </row>
   </sheetData>
@@ -10674,7 +10677,7 @@
         <v>1</v>
       </c>
       <c r="L7" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
@@ -10726,7 +10729,7 @@
         <v>5</v>
       </c>
       <c r="L9" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
@@ -10766,7 +10769,7 @@
         <v>10</v>
       </c>
       <c r="F11" t="s">
-        <v>719</v>
+        <v>711</v>
       </c>
       <c r="H11">
         <v>10</v>
@@ -10778,7 +10781,7 @@
         <v>7</v>
       </c>
       <c r="L11" t="s">
-        <v>797</v>
+        <v>789</v>
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
@@ -10804,7 +10807,7 @@
         <v>9</v>
       </c>
       <c r="L12" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
@@ -10812,13 +10815,13 @@
         <v>10</v>
       </c>
       <c r="C13" t="s">
-        <v>718</v>
+        <v>710</v>
       </c>
       <c r="E13">
         <v>14</v>
       </c>
       <c r="F13" s="39" t="s">
-        <v>750</v>
+        <v>742</v>
       </c>
       <c r="H13">
         <v>14</v>
@@ -10830,7 +10833,7 @@
         <v>11</v>
       </c>
       <c r="L13" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
@@ -10850,7 +10853,7 @@
         <v>15</v>
       </c>
       <c r="I14" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
       <c r="K14">
         <v>16</v>
@@ -10876,13 +10879,13 @@
         <v>16</v>
       </c>
       <c r="I15" t="s">
-        <v>785</v>
+        <v>777</v>
       </c>
       <c r="K15">
         <v>20</v>
       </c>
       <c r="L15" t="s">
-        <v>783</v>
+        <v>775</v>
       </c>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
@@ -10922,7 +10925,7 @@
         <v>22</v>
       </c>
       <c r="L17" t="s">
-        <v>794</v>
+        <v>786</v>
       </c>
     </row>
     <row r="18" spans="8:12" x14ac:dyDescent="0.25">
@@ -10936,7 +10939,7 @@
         <v>25</v>
       </c>
       <c r="L18" t="s">
-        <v>784</v>
+        <v>776</v>
       </c>
     </row>
   </sheetData>
@@ -11159,7 +11162,7 @@
         <v>8</v>
       </c>
       <c r="U10" t="s">
-        <v>765</v>
+        <v>757</v>
       </c>
     </row>
     <row r="11" spans="2:21" x14ac:dyDescent="0.25">
@@ -11191,19 +11194,19 @@
         <v>9</v>
       </c>
       <c r="O11" t="s">
-        <v>738</v>
+        <v>730</v>
       </c>
       <c r="Q11">
         <v>9</v>
       </c>
       <c r="R11" t="s">
-        <v>738</v>
+        <v>730</v>
       </c>
       <c r="T11">
         <v>9</v>
       </c>
       <c r="U11" t="s">
-        <v>738</v>
+        <v>730</v>
       </c>
     </row>
     <row r="12" spans="2:21" x14ac:dyDescent="0.25">
@@ -11279,19 +11282,19 @@
         <v>14</v>
       </c>
       <c r="O13" t="s">
-        <v>755</v>
+        <v>747</v>
       </c>
       <c r="Q13">
         <v>14</v>
       </c>
       <c r="R13" t="s">
-        <v>757</v>
+        <v>749</v>
       </c>
       <c r="T13">
         <v>14</v>
       </c>
       <c r="U13" t="s">
-        <v>759</v>
+        <v>751</v>
       </c>
     </row>
     <row r="14" spans="2:21" x14ac:dyDescent="0.25">
@@ -11335,7 +11338,7 @@
         <v>15</v>
       </c>
       <c r="U14" t="s">
-        <v>758</v>
+        <v>750</v>
       </c>
     </row>
     <row r="15" spans="2:21" x14ac:dyDescent="0.25">
@@ -11367,19 +11370,19 @@
         <v>17</v>
       </c>
       <c r="O15" t="s">
-        <v>686</v>
+        <v>683</v>
       </c>
       <c r="Q15">
         <v>17</v>
       </c>
       <c r="R15" t="s">
-        <v>685</v>
+        <v>682</v>
       </c>
       <c r="T15">
         <v>17</v>
       </c>
       <c r="U15" t="s">
-        <v>687</v>
+        <v>684</v>
       </c>
     </row>
     <row r="16" spans="2:21" x14ac:dyDescent="0.25">
@@ -11411,7 +11414,7 @@
         <v>21</v>
       </c>
       <c r="O16" t="s">
-        <v>756</v>
+        <v>748</v>
       </c>
       <c r="Q16">
         <v>21</v>
@@ -11431,19 +11434,19 @@
         <v>22</v>
       </c>
       <c r="O17" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
       <c r="Q17">
         <v>22</v>
       </c>
       <c r="R17" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
       <c r="T17">
         <v>22</v>
       </c>
       <c r="U17" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
     </row>
     <row r="18" spans="9:21" x14ac:dyDescent="0.25">
@@ -11498,7 +11501,7 @@
     </row>
     <row r="30" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I30" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
quitado el texto de las fases y más ataques y más correcciones de las lineas
</commit_message>
<xml_diff>
--- a/arquetiposZ.xlsx
+++ b/arquetiposZ.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sergius\Desktop\Proyectos\hyperbole\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1353EF6-C2CB-4A48-AF6E-B8D962E7D4D1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CF67934-CC51-47B7-B03C-EB74BD0A289F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="644" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="644" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RESUMEN" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1145" uniqueCount="812">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1146" uniqueCount="814">
   <si>
     <t>daños:</t>
   </si>
@@ -1471,12 +1471,6 @@
     <t>bufudyne strike</t>
   </si>
   <si>
-    <t>hamaon strike</t>
-  </si>
-  <si>
-    <t>mudoon strike</t>
-  </si>
-  <si>
     <t>lanza, espada, florete, escudo</t>
   </si>
   <si>
@@ -1516,9 +1510,6 @@
     <t>holy protection</t>
   </si>
   <si>
-    <t>holy protection: todo el daño recibido se reduce a la mitad si hay un escudo equipado</t>
-  </si>
-  <si>
     <t>aum mucho lanza</t>
   </si>
   <si>
@@ -1999,9 +1990,6 @@
     <t>space aura y time aura mejoran un poco ursa, cassiopeia y pleiyades y slow y haste respectivamente</t>
   </si>
   <si>
-    <t>ahorro space</t>
-  </si>
-  <si>
     <t>ahorro time</t>
   </si>
   <si>
@@ -2480,6 +2468,24 @@
   </si>
   <si>
     <t>invoc hielo leve x4-5 todos IR mareo</t>
+  </si>
+  <si>
+    <t>ursa ag</t>
+  </si>
+  <si>
+    <t>[espada 7]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         </t>
+  </si>
+  <si>
+    <t>ursa sue</t>
+  </si>
+  <si>
+    <t>holy protection: puede equipar dos escudos. todo el daño recibido se reduce a la mitad si hay dos escudos equipados</t>
+  </si>
+  <si>
+    <t>knight's proclamation</t>
   </si>
 </sst>
 </file>
@@ -3136,15 +3142,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>295275</xdr:colOff>
+      <xdr:colOff>276225</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
+      <xdr:rowOff>66675</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>39033</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>9560</xdr:rowOff>
+      <xdr:colOff>19983</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>123860</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3167,7 +3173,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6791325" y="5857875"/>
+          <a:off x="6772275" y="5781675"/>
           <a:ext cx="6687483" cy="247685"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4219,7 +4225,7 @@
         <v>43</v>
       </c>
       <c r="L26" s="5" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
       <c r="M26" s="5"/>
       <c r="N26" s="5"/>
@@ -4364,7 +4370,7 @@
         <v>54</v>
       </c>
       <c r="L31" s="5" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="M31" s="5"/>
       <c r="N31" s="5"/>
@@ -4391,7 +4397,7 @@
         <v>55</v>
       </c>
       <c r="L32" s="5" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="M32" s="5"/>
       <c r="N32" s="5"/>
@@ -4414,13 +4420,13 @@
       <c r="H33" s="5"/>
       <c r="I33" s="1"/>
       <c r="J33" s="5" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="K33" s="5" t="s">
         <v>66</v>
       </c>
       <c r="L33" s="5" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="M33" s="5"/>
       <c r="N33" s="5"/>
@@ -4451,7 +4457,7 @@
         <v>58</v>
       </c>
       <c r="L34" s="5" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="M34" s="5"/>
       <c r="N34" s="5"/>
@@ -4746,7 +4752,7 @@
         <v>15</v>
       </c>
       <c r="G12" t="s">
-        <v>743</v>
+        <v>739</v>
       </c>
       <c r="J12">
         <v>10</v>
@@ -4828,7 +4834,7 @@
         <v>24</v>
       </c>
       <c r="K17" t="s">
-        <v>787</v>
+        <v>783</v>
       </c>
     </row>
     <row r="18" spans="8:11" x14ac:dyDescent="0.25">
@@ -4871,7 +4877,7 @@
     </row>
     <row r="30" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H30" t="s">
-        <v>744</v>
+        <v>740</v>
       </c>
     </row>
     <row r="31" spans="8:11" x14ac:dyDescent="0.25">
@@ -4881,7 +4887,7 @@
     </row>
     <row r="32" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H32" t="s">
-        <v>732</v>
+        <v>728</v>
       </c>
     </row>
     <row r="33" spans="8:8" x14ac:dyDescent="0.25">
@@ -4896,7 +4902,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC616436-1C76-440D-9462-77F99D101652}">
-  <dimension ref="B6:U37"/>
+  <dimension ref="B6:V37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="4.28515625" customWidth="1"/>
@@ -4906,9 +4912,10 @@
     <col min="14" max="14" width="5" customWidth="1"/>
     <col min="17" max="17" width="4.7109375" customWidth="1"/>
     <col min="20" max="20" width="5.140625" customWidth="1"/>
+    <col min="21" max="21" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="6" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
         <v>38</v>
       </c>
@@ -4931,7 +4938,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="7" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B7">
         <v>1</v>
       </c>
@@ -4942,13 +4949,13 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>466</v>
+        <v>813</v>
       </c>
       <c r="H7">
         <v>1</v>
       </c>
       <c r="I7" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="K7">
         <v>1</v>
@@ -4960,13 +4967,13 @@
         <v>1</v>
       </c>
       <c r="O7" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
       <c r="Q7">
         <v>1</v>
       </c>
       <c r="R7" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="T7">
         <v>1</v>
@@ -4975,7 +4982,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="8" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B8">
         <v>3</v>
       </c>
@@ -4998,7 +5005,7 @@
         <v>2</v>
       </c>
       <c r="L8" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="N8">
         <v>4</v>
@@ -5019,7 +5026,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="9" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B9">
         <v>5</v>
       </c>
@@ -5042,7 +5049,7 @@
         <v>5</v>
       </c>
       <c r="L9" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="N9">
         <v>5</v>
@@ -5054,7 +5061,7 @@
         <v>6</v>
       </c>
       <c r="R9" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="T9">
         <v>3</v>
@@ -5063,7 +5070,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="10" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B10">
         <v>6</v>
       </c>
@@ -5080,7 +5087,7 @@
         <v>6</v>
       </c>
       <c r="I10" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K10">
         <v>8</v>
@@ -5098,7 +5105,7 @@
         <v>8</v>
       </c>
       <c r="R10" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
       <c r="T10">
         <v>3</v>
@@ -5107,7 +5114,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="11" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B11">
         <v>8</v>
       </c>
@@ -5124,7 +5131,7 @@
         <v>7</v>
       </c>
       <c r="I11" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="K11">
         <v>10</v>
@@ -5136,13 +5143,13 @@
         <v>9</v>
       </c>
       <c r="O11" t="s">
-        <v>741</v>
+        <v>737</v>
       </c>
       <c r="Q11">
         <v>10</v>
       </c>
       <c r="R11" t="s">
-        <v>676</v>
+        <v>672</v>
       </c>
       <c r="T11">
         <v>6</v>
@@ -5151,7 +5158,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="12" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B12">
         <v>8</v>
       </c>
@@ -5168,34 +5175,34 @@
         <v>10</v>
       </c>
       <c r="I12" t="s">
-        <v>773</v>
+        <v>769</v>
       </c>
       <c r="K12">
         <v>12</v>
       </c>
       <c r="L12" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="N12">
         <v>10</v>
       </c>
       <c r="O12" t="s">
-        <v>739</v>
+        <v>735</v>
       </c>
       <c r="Q12">
         <v>12</v>
       </c>
       <c r="R12" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="T12">
         <v>9</v>
       </c>
       <c r="U12" t="s">
-        <v>495</v>
-      </c>
-    </row>
-    <row r="13" spans="2:21" x14ac:dyDescent="0.25">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="13" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B13">
         <v>11</v>
       </c>
@@ -5212,7 +5219,7 @@
         <v>10</v>
       </c>
       <c r="I13" t="s">
-        <v>774</v>
+        <v>770</v>
       </c>
       <c r="K13">
         <v>14</v>
@@ -5224,27 +5231,27 @@
         <v>11</v>
       </c>
       <c r="O13" t="s">
-        <v>738</v>
+        <v>734</v>
       </c>
       <c r="Q13">
         <v>14</v>
       </c>
       <c r="R13" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="T13">
         <v>12</v>
       </c>
       <c r="U13" t="s">
-        <v>496</v>
-      </c>
-    </row>
-    <row r="14" spans="2:21" x14ac:dyDescent="0.25">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="14" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B14">
         <v>13</v>
       </c>
       <c r="C14" s="39" t="s">
-        <v>758</v>
+        <v>754</v>
       </c>
       <c r="E14">
         <v>16</v>
@@ -5256,34 +5263,34 @@
         <v>12</v>
       </c>
       <c r="I14" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="K14">
         <v>15</v>
       </c>
       <c r="L14" t="s">
-        <v>796</v>
+        <v>792</v>
       </c>
       <c r="N14">
         <v>12</v>
       </c>
       <c r="O14" t="s">
-        <v>740</v>
+        <v>736</v>
       </c>
       <c r="Q14">
         <v>15</v>
       </c>
       <c r="R14" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="T14">
         <v>15</v>
       </c>
       <c r="U14" t="s">
-        <v>497</v>
-      </c>
-    </row>
-    <row r="15" spans="2:21" x14ac:dyDescent="0.25">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="15" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B15">
         <v>15</v>
       </c>
@@ -5294,7 +5301,7 @@
         <v>18</v>
       </c>
       <c r="F15" t="s">
-        <v>795</v>
+        <v>791</v>
       </c>
       <c r="H15">
         <v>16</v>
@@ -5306,28 +5313,28 @@
         <v>16</v>
       </c>
       <c r="L15" t="s">
-        <v>788</v>
+        <v>784</v>
       </c>
       <c r="N15">
         <v>13</v>
       </c>
       <c r="O15" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="Q15">
         <v>16</v>
       </c>
       <c r="R15" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="T15">
         <v>17</v>
       </c>
       <c r="U15" t="s">
-        <v>475</v>
-      </c>
-    </row>
-    <row r="16" spans="2:21" x14ac:dyDescent="0.25">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="16" spans="2:22" x14ac:dyDescent="0.25">
       <c r="E16">
         <v>20</v>
       </c>
@@ -5338,31 +5345,34 @@
         <v>20</v>
       </c>
       <c r="I16" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="K16">
         <v>20</v>
       </c>
       <c r="L16" t="s">
-        <v>745</v>
+        <v>741</v>
       </c>
       <c r="N16">
         <v>15</v>
       </c>
       <c r="O16" t="s">
-        <v>734</v>
+        <v>730</v>
       </c>
       <c r="Q16">
         <v>20</v>
       </c>
       <c r="R16" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="T16">
         <v>19</v>
       </c>
       <c r="U16" t="s">
-        <v>476</v>
+        <v>493</v>
+      </c>
+      <c r="V16" t="s">
+        <v>810</v>
       </c>
     </row>
     <row r="17" spans="9:21" x14ac:dyDescent="0.25">
@@ -5376,19 +5386,19 @@
         <v>20</v>
       </c>
       <c r="O17" t="s">
-        <v>794</v>
+        <v>790</v>
       </c>
       <c r="Q17">
         <v>23</v>
       </c>
       <c r="R17" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="T17">
         <v>23</v>
       </c>
       <c r="U17" t="s">
-        <v>503</v>
+        <v>809</v>
       </c>
     </row>
     <row r="18" spans="9:21" x14ac:dyDescent="0.25">
@@ -5396,25 +5406,25 @@
         <v>25</v>
       </c>
       <c r="L18" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="N18">
         <v>25</v>
       </c>
       <c r="O18" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="Q18">
         <v>25</v>
       </c>
       <c r="R18" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="T18">
         <v>25</v>
       </c>
       <c r="U18" t="s">
-        <v>696</v>
+        <v>692</v>
       </c>
     </row>
     <row r="21" spans="9:21" x14ac:dyDescent="0.25">
@@ -5474,32 +5484,32 @@
     </row>
     <row r="32" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I32" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
     </row>
     <row r="33" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I33" t="s">
-        <v>490</v>
+        <v>812</v>
       </c>
     </row>
     <row r="34" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I34" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
     </row>
     <row r="35" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I35" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
     </row>
     <row r="36" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I36" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
     </row>
     <row r="37" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I37" t="s">
-        <v>697</v>
+        <v>693</v>
       </c>
     </row>
   </sheetData>
@@ -5564,7 +5574,7 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>805</v>
+        <v>801</v>
       </c>
       <c r="H7">
         <v>1</v>
@@ -5576,7 +5586,7 @@
         <v>1</v>
       </c>
       <c r="L7" t="s">
-        <v>689</v>
+        <v>685</v>
       </c>
       <c r="N7">
         <v>1</v>
@@ -5588,13 +5598,13 @@
         <v>1</v>
       </c>
       <c r="R7" t="s">
-        <v>764</v>
+        <v>811</v>
       </c>
       <c r="T7">
         <v>1</v>
       </c>
       <c r="U7" s="39" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
     </row>
     <row r="8" spans="2:21" x14ac:dyDescent="0.25">
@@ -5620,25 +5630,25 @@
         <v>1</v>
       </c>
       <c r="L8" t="s">
-        <v>690</v>
+        <v>686</v>
       </c>
       <c r="N8">
         <v>1</v>
       </c>
       <c r="O8" t="s">
-        <v>654</v>
+        <v>650</v>
       </c>
       <c r="Q8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R8" t="s">
+        <v>176</v>
+      </c>
+      <c r="T8">
+        <v>1</v>
+      </c>
+      <c r="U8" t="s">
         <v>765</v>
-      </c>
-      <c r="T8">
-        <v>1</v>
-      </c>
-      <c r="U8" t="s">
-        <v>769</v>
       </c>
     </row>
     <row r="9" spans="2:21" x14ac:dyDescent="0.25">
@@ -5646,7 +5656,7 @@
         <v>4</v>
       </c>
       <c r="C9" t="s">
-        <v>691</v>
+        <v>687</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -5664,7 +5674,7 @@
         <v>1</v>
       </c>
       <c r="L9" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="N9">
         <v>1</v>
@@ -5673,16 +5683,16 @@
         <v>293</v>
       </c>
       <c r="Q9">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="R9" t="s">
+        <v>760</v>
+      </c>
+      <c r="T9">
+        <v>1</v>
+      </c>
+      <c r="U9" t="s">
         <v>766</v>
-      </c>
-      <c r="T9">
-        <v>1</v>
-      </c>
-      <c r="U9" t="s">
-        <v>770</v>
       </c>
     </row>
     <row r="10" spans="2:21" x14ac:dyDescent="0.25">
@@ -5690,37 +5700,37 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>692</v>
+        <v>688</v>
       </c>
       <c r="E10">
         <v>5</v>
       </c>
       <c r="F10" t="s">
-        <v>809</v>
+        <v>805</v>
       </c>
       <c r="H10">
         <v>7</v>
       </c>
       <c r="I10" t="s">
-        <v>111</v>
+        <v>758</v>
       </c>
       <c r="K10">
         <v>5</v>
       </c>
       <c r="L10" t="s">
-        <v>686</v>
+        <v>682</v>
       </c>
       <c r="N10">
         <v>5</v>
       </c>
       <c r="O10" t="s">
-        <v>803</v>
+        <v>799</v>
       </c>
       <c r="Q10">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="R10" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="T10">
         <v>3</v>
@@ -5734,13 +5744,13 @@
         <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>693</v>
+        <v>689</v>
       </c>
       <c r="E11">
         <v>10</v>
       </c>
       <c r="F11" t="s">
-        <v>804</v>
+        <v>800</v>
       </c>
       <c r="H11">
         <v>10</v>
@@ -5752,7 +5762,7 @@
         <v>9</v>
       </c>
       <c r="L11" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="N11">
         <v>10</v>
@@ -5761,16 +5771,16 @@
         <v>106</v>
       </c>
       <c r="Q11">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="R11" t="s">
-        <v>651</v>
+        <v>716</v>
       </c>
       <c r="T11">
         <v>7</v>
       </c>
       <c r="U11" t="s">
-        <v>652</v>
+        <v>110</v>
       </c>
     </row>
     <row r="12" spans="2:21" x14ac:dyDescent="0.25">
@@ -5784,19 +5794,19 @@
         <v>12</v>
       </c>
       <c r="F12" s="39" t="s">
-        <v>759</v>
+        <v>755</v>
       </c>
       <c r="H12">
         <v>15</v>
       </c>
       <c r="I12" t="s">
-        <v>172</v>
+        <v>759</v>
       </c>
       <c r="K12">
         <v>11</v>
       </c>
       <c r="L12" t="s">
-        <v>810</v>
+        <v>806</v>
       </c>
       <c r="N12">
         <v>12</v>
@@ -5805,10 +5815,10 @@
         <v>103</v>
       </c>
       <c r="Q12">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="R12" t="s">
-        <v>179</v>
+        <v>761</v>
       </c>
       <c r="T12">
         <v>10</v>
@@ -5828,19 +5838,19 @@
         <v>17</v>
       </c>
       <c r="F13" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="H13">
         <v>15</v>
       </c>
       <c r="I13" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="K13">
         <v>14</v>
       </c>
       <c r="L13" t="s">
-        <v>807</v>
+        <v>803</v>
       </c>
       <c r="N13">
         <v>12</v>
@@ -5849,10 +5859,10 @@
         <v>104</v>
       </c>
       <c r="Q13">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="R13" t="s">
-        <v>720</v>
+        <v>762</v>
       </c>
       <c r="T13">
         <v>11</v>
@@ -5866,7 +5876,7 @@
         <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="E14">
         <v>18</v>
@@ -5878,22 +5888,22 @@
         <v>19</v>
       </c>
       <c r="I14" t="s">
-        <v>761</v>
+        <v>173</v>
       </c>
       <c r="K14">
         <v>16</v>
       </c>
       <c r="L14" t="s">
-        <v>806</v>
+        <v>802</v>
       </c>
       <c r="N14">
         <v>15</v>
       </c>
       <c r="O14" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="Q14">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="R14" t="s">
         <v>111</v>
@@ -5910,25 +5920,25 @@
         <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="E15">
         <v>19</v>
       </c>
       <c r="F15" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="H15">
         <v>20</v>
       </c>
       <c r="I15" t="s">
-        <v>762</v>
+        <v>808</v>
       </c>
       <c r="K15">
         <v>18</v>
       </c>
       <c r="L15" t="s">
-        <v>808</v>
+        <v>804</v>
       </c>
       <c r="N15">
         <v>18</v>
@@ -5937,7 +5947,7 @@
         <v>297</v>
       </c>
       <c r="Q15">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="R15" t="s">
         <v>114</v>
@@ -5946,7 +5956,7 @@
         <v>15</v>
       </c>
       <c r="U15" t="s">
-        <v>110</v>
+        <v>648</v>
       </c>
     </row>
     <row r="16" spans="2:21" x14ac:dyDescent="0.25">
@@ -5954,25 +5964,25 @@
         <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>719</v>
+        <v>715</v>
       </c>
       <c r="E16">
         <v>20</v>
       </c>
       <c r="F16" t="s">
-        <v>688</v>
+        <v>684</v>
       </c>
       <c r="H16">
         <v>20</v>
       </c>
       <c r="I16" t="s">
-        <v>763</v>
+        <v>757</v>
       </c>
       <c r="K16">
         <v>21</v>
       </c>
       <c r="L16" t="s">
-        <v>811</v>
+        <v>807</v>
       </c>
       <c r="N16">
         <v>20</v>
@@ -5981,7 +5991,7 @@
         <v>105</v>
       </c>
       <c r="Q16">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="R16" t="s">
         <v>113</v>
@@ -5990,7 +6000,7 @@
         <v>19</v>
       </c>
       <c r="U16" t="s">
-        <v>655</v>
+        <v>651</v>
       </c>
     </row>
     <row r="17" spans="10:21" x14ac:dyDescent="0.25">
@@ -5998,7 +6008,7 @@
         <v>22</v>
       </c>
       <c r="L17" t="s">
-        <v>694</v>
+        <v>690</v>
       </c>
       <c r="N17">
         <v>20</v>
@@ -6024,7 +6034,7 @@
         <v>25</v>
       </c>
       <c r="L18" t="s">
-        <v>695</v>
+        <v>691</v>
       </c>
       <c r="N18">
         <v>25</v>
@@ -6062,22 +6072,22 @@
     </row>
     <row r="25" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J25" t="s">
-        <v>767</v>
+        <v>763</v>
       </c>
     </row>
     <row r="26" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J26" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
     </row>
     <row r="27" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J27" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
     </row>
     <row r="28" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J28" t="s">
-        <v>768</v>
+        <v>764</v>
       </c>
     </row>
     <row r="29" spans="10:21" x14ac:dyDescent="0.25">
@@ -6092,27 +6102,27 @@
     </row>
     <row r="31" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J31" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
     </row>
     <row r="32" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J32" t="s">
-        <v>653</v>
+        <v>649</v>
       </c>
     </row>
     <row r="33" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J33" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
     </row>
     <row r="34" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J34" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
     </row>
     <row r="35" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J35" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
     </row>
   </sheetData>
@@ -6147,19 +6157,19 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>791</v>
+        <v>787</v>
       </c>
       <c r="J7">
         <v>1</v>
       </c>
       <c r="K7" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.25">
@@ -6167,7 +6177,7 @@
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>625</v>
+        <v>622</v>
       </c>
       <c r="F8">
         <v>1</v>
@@ -6187,19 +6197,19 @@
         <v>5</v>
       </c>
       <c r="C9" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
       <c r="F9">
         <v>3</v>
       </c>
       <c r="G9" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
       <c r="J9">
         <v>7</v>
       </c>
       <c r="K9" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.25">
@@ -6213,7 +6223,7 @@
         <v>6</v>
       </c>
       <c r="G10" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="J10">
         <v>8</v>
@@ -6227,19 +6237,19 @@
         <v>7</v>
       </c>
       <c r="C11" t="s">
-        <v>630</v>
+        <v>627</v>
       </c>
       <c r="F11">
         <v>7</v>
       </c>
       <c r="G11" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="J11">
         <v>11</v>
       </c>
       <c r="K11" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.25">
@@ -6247,19 +6257,19 @@
         <v>8</v>
       </c>
       <c r="C12" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
       <c r="F12">
         <v>8</v>
       </c>
       <c r="G12" t="s">
-        <v>792</v>
+        <v>788</v>
       </c>
       <c r="J12">
         <v>11</v>
       </c>
       <c r="K12" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.25">
@@ -6267,7 +6277,7 @@
         <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>638</v>
+        <v>635</v>
       </c>
       <c r="F13">
         <v>12</v>
@@ -6279,7 +6289,7 @@
         <v>13</v>
       </c>
       <c r="K13" t="s">
-        <v>685</v>
+        <v>681</v>
       </c>
     </row>
     <row r="14" spans="2:11" x14ac:dyDescent="0.25">
@@ -6293,13 +6303,13 @@
         <v>16</v>
       </c>
       <c r="G14" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="J14">
         <v>15</v>
       </c>
       <c r="K14" t="s">
-        <v>733</v>
+        <v>729</v>
       </c>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.25">
@@ -6307,19 +6317,19 @@
         <v>13</v>
       </c>
       <c r="C15" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
       <c r="F15">
         <v>19</v>
       </c>
       <c r="G15" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="J15">
         <v>18</v>
       </c>
       <c r="K15" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.25">
@@ -6327,19 +6337,19 @@
         <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="F16">
         <v>20</v>
       </c>
       <c r="G16" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="J16">
         <v>20</v>
       </c>
       <c r="K16" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
     </row>
     <row r="17" spans="10:11" x14ac:dyDescent="0.25">
@@ -6347,7 +6357,7 @@
         <v>20</v>
       </c>
       <c r="K17" t="s">
-        <v>635</v>
+        <v>632</v>
       </c>
     </row>
     <row r="18" spans="10:11" x14ac:dyDescent="0.25">
@@ -6355,27 +6365,27 @@
         <v>25</v>
       </c>
       <c r="K18" t="s">
-        <v>624</v>
+        <v>621</v>
       </c>
     </row>
     <row r="27" spans="10:11" x14ac:dyDescent="0.25">
       <c r="K27" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
     </row>
     <row r="28" spans="10:11" x14ac:dyDescent="0.25">
       <c r="K28" t="s">
-        <v>628</v>
+        <v>625</v>
       </c>
     </row>
     <row r="29" spans="10:11" x14ac:dyDescent="0.25">
       <c r="K29" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
     </row>
     <row r="30" spans="10:11" x14ac:dyDescent="0.25">
       <c r="K30" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
     </row>
   </sheetData>
@@ -6408,7 +6418,7 @@
         <v>63</v>
       </c>
       <c r="I6" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="L6" t="s">
         <v>54</v>
@@ -6417,7 +6427,7 @@
         <v>55</v>
       </c>
       <c r="R6" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="V6" t="s">
         <v>66</v>
@@ -6428,7 +6438,7 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -6440,31 +6450,31 @@
         <v>1</v>
       </c>
       <c r="I7" t="s">
+        <v>531</v>
+      </c>
+      <c r="K7">
+        <v>1</v>
+      </c>
+      <c r="L7" t="s">
         <v>534</v>
       </c>
-      <c r="K7">
-        <v>1</v>
-      </c>
-      <c r="L7" t="s">
-        <v>537</v>
-      </c>
       <c r="N7">
         <v>1</v>
       </c>
       <c r="O7" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="Q7">
         <v>1</v>
       </c>
       <c r="R7" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="U7">
         <v>1</v>
       </c>
       <c r="V7" t="s">
-        <v>715</v>
+        <v>711</v>
       </c>
     </row>
     <row r="8" spans="2:22" x14ac:dyDescent="0.25">
@@ -6472,7 +6482,7 @@
         <v>3</v>
       </c>
       <c r="C8" t="s">
-        <v>587</v>
+        <v>584</v>
       </c>
       <c r="E8">
         <v>4</v>
@@ -6484,13 +6494,13 @@
         <v>1</v>
       </c>
       <c r="I8" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="K8">
         <v>1</v>
       </c>
       <c r="L8" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="N8">
         <v>1</v>
@@ -6502,13 +6512,13 @@
         <v>3</v>
       </c>
       <c r="R8" t="s">
-        <v>712</v>
+        <v>708</v>
       </c>
       <c r="U8">
         <v>2</v>
       </c>
       <c r="V8" t="s">
-        <v>707</v>
+        <v>703</v>
       </c>
     </row>
     <row r="9" spans="2:22" x14ac:dyDescent="0.25">
@@ -6516,13 +6526,13 @@
         <v>5</v>
       </c>
       <c r="C9" t="s">
-        <v>702</v>
+        <v>698</v>
       </c>
       <c r="E9">
         <v>4</v>
       </c>
       <c r="F9" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
       <c r="H9">
         <v>4</v>
@@ -6546,13 +6556,13 @@
         <v>5</v>
       </c>
       <c r="R9" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="U9">
         <v>2</v>
       </c>
       <c r="V9" t="s">
-        <v>703</v>
+        <v>699</v>
       </c>
     </row>
     <row r="10" spans="2:22" x14ac:dyDescent="0.25">
@@ -6560,43 +6570,43 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="E10">
         <v>6</v>
       </c>
       <c r="F10" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
       <c r="H10">
         <v>5</v>
       </c>
       <c r="I10" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="K10">
         <v>8</v>
       </c>
       <c r="L10" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="N10">
         <v>8</v>
       </c>
       <c r="O10" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="Q10">
         <v>8</v>
       </c>
       <c r="R10" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="U10">
         <v>6</v>
       </c>
       <c r="V10" t="s">
-        <v>713</v>
+        <v>709</v>
       </c>
     </row>
     <row r="11" spans="2:22" x14ac:dyDescent="0.25">
@@ -6604,19 +6614,19 @@
         <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>573</v>
+        <v>570</v>
       </c>
       <c r="E11">
         <v>8</v>
       </c>
       <c r="F11" t="s">
-        <v>589</v>
+        <v>586</v>
       </c>
       <c r="H11">
         <v>7</v>
       </c>
       <c r="I11" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="K11">
         <v>10</v>
@@ -6634,13 +6644,13 @@
         <v>10</v>
       </c>
       <c r="R11" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="U11">
         <v>7</v>
       </c>
       <c r="V11" t="s">
-        <v>721</v>
+        <v>717</v>
       </c>
     </row>
     <row r="12" spans="2:22" x14ac:dyDescent="0.25">
@@ -6648,43 +6658,43 @@
         <v>10</v>
       </c>
       <c r="C12" t="s">
-        <v>708</v>
+        <v>704</v>
       </c>
       <c r="E12">
         <v>11</v>
       </c>
       <c r="F12" t="s">
-        <v>591</v>
+        <v>588</v>
       </c>
       <c r="H12">
         <v>8</v>
       </c>
       <c r="I12" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="K12">
         <v>12</v>
       </c>
       <c r="L12" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="N12">
         <v>12</v>
       </c>
       <c r="O12" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="Q12">
         <v>12</v>
       </c>
       <c r="R12" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="U12">
         <v>8</v>
       </c>
       <c r="V12" t="s">
-        <v>704</v>
+        <v>700</v>
       </c>
     </row>
     <row r="13" spans="2:22" x14ac:dyDescent="0.25">
@@ -6692,43 +6702,43 @@
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="E13">
         <v>14</v>
       </c>
       <c r="F13" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="H13">
         <v>9</v>
       </c>
       <c r="I13" t="s">
-        <v>725</v>
+        <v>721</v>
       </c>
       <c r="K13">
         <v>14</v>
       </c>
       <c r="L13" t="s">
-        <v>592</v>
+        <v>589</v>
       </c>
       <c r="N13">
         <v>14</v>
       </c>
       <c r="O13" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="Q13">
         <v>14</v>
       </c>
       <c r="R13" t="s">
-        <v>801</v>
+        <v>797</v>
       </c>
       <c r="U13">
         <v>9</v>
       </c>
       <c r="V13" t="s">
-        <v>798</v>
+        <v>794</v>
       </c>
     </row>
     <row r="14" spans="2:22" x14ac:dyDescent="0.25">
@@ -6736,7 +6746,7 @@
         <v>14</v>
       </c>
       <c r="C14" t="s">
-        <v>723</v>
+        <v>719</v>
       </c>
       <c r="E14">
         <v>16</v>
@@ -6748,7 +6758,7 @@
         <v>11</v>
       </c>
       <c r="I14" t="s">
-        <v>706</v>
+        <v>702</v>
       </c>
       <c r="K14">
         <v>15</v>
@@ -6766,13 +6776,13 @@
         <v>15</v>
       </c>
       <c r="R14" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="U14">
         <v>14</v>
       </c>
       <c r="V14" t="s">
-        <v>717</v>
+        <v>713</v>
       </c>
     </row>
     <row r="15" spans="2:22" x14ac:dyDescent="0.25">
@@ -6780,43 +6790,43 @@
         <v>15</v>
       </c>
       <c r="C15" t="s">
-        <v>593</v>
+        <v>590</v>
       </c>
       <c r="E15">
         <v>18</v>
       </c>
       <c r="F15" t="s">
-        <v>709</v>
+        <v>705</v>
       </c>
       <c r="H15">
         <v>16</v>
       </c>
       <c r="I15" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
       <c r="K15">
         <v>20</v>
       </c>
       <c r="L15" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="N15">
         <v>16</v>
       </c>
       <c r="O15" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="Q15">
         <v>16</v>
       </c>
       <c r="R15" t="s">
-        <v>716</v>
+        <v>712</v>
       </c>
       <c r="U15">
         <v>17</v>
       </c>
       <c r="V15" t="s">
-        <v>597</v>
+        <v>594</v>
       </c>
     </row>
     <row r="16" spans="2:22" x14ac:dyDescent="0.25">
@@ -6824,37 +6834,37 @@
         <v>20</v>
       </c>
       <c r="F16" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="H16">
         <v>20</v>
       </c>
       <c r="I16" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="K16">
         <v>20</v>
       </c>
       <c r="L16" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="N16">
         <v>20</v>
       </c>
       <c r="O16" t="s">
-        <v>622</v>
+        <v>619</v>
       </c>
       <c r="Q16">
         <v>20</v>
       </c>
       <c r="R16" t="s">
-        <v>595</v>
+        <v>592</v>
       </c>
       <c r="U16">
         <v>20</v>
       </c>
       <c r="V16" t="s">
-        <v>705</v>
+        <v>701</v>
       </c>
     </row>
     <row r="17" spans="11:22" x14ac:dyDescent="0.25">
@@ -6862,25 +6872,25 @@
         <v>24</v>
       </c>
       <c r="L17" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="N17">
         <v>23</v>
       </c>
       <c r="O17" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="Q17">
         <v>24</v>
       </c>
       <c r="R17" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="U17">
         <v>24</v>
       </c>
       <c r="V17" t="s">
-        <v>714</v>
+        <v>710</v>
       </c>
     </row>
     <row r="18" spans="11:22" x14ac:dyDescent="0.25">
@@ -6888,75 +6898,75 @@
         <v>25</v>
       </c>
       <c r="L18" t="s">
-        <v>594</v>
+        <v>591</v>
       </c>
       <c r="N18">
         <v>25</v>
       </c>
       <c r="O18" t="s">
-        <v>736</v>
+        <v>732</v>
       </c>
       <c r="Q18">
         <v>25</v>
       </c>
       <c r="R18" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
       <c r="U18">
         <v>25</v>
       </c>
       <c r="V18" t="s">
-        <v>722</v>
+        <v>718</v>
       </c>
     </row>
     <row r="22" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L22" t="s">
-        <v>737</v>
+        <v>733</v>
       </c>
     </row>
     <row r="23" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L23" t="s">
-        <v>724</v>
+        <v>720</v>
       </c>
     </row>
     <row r="24" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L24" t="s">
-        <v>726</v>
+        <v>722</v>
       </c>
     </row>
     <row r="25" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L25" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
     </row>
     <row r="26" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L26" t="s">
-        <v>590</v>
+        <v>587</v>
       </c>
     </row>
     <row r="27" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L27" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
     </row>
     <row r="28" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L28" t="s">
-        <v>790</v>
+        <v>786</v>
       </c>
     </row>
     <row r="29" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L29" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
     </row>
     <row r="30" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L30" t="s">
-        <v>793</v>
+        <v>789</v>
       </c>
     </row>
     <row r="33" spans="13:13" x14ac:dyDescent="0.25">
       <c r="M33" t="s">
-        <v>718</v>
+        <v>714</v>
       </c>
     </row>
   </sheetData>
@@ -7004,19 +7014,19 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
+        <v>546</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7" t="s">
+        <v>579</v>
+      </c>
+      <c r="K7">
+        <v>1</v>
+      </c>
+      <c r="L7" t="s">
         <v>549</v>
-      </c>
-      <c r="H7">
-        <v>1</v>
-      </c>
-      <c r="I7" t="s">
-        <v>582</v>
-      </c>
-      <c r="K7">
-        <v>1</v>
-      </c>
-      <c r="L7" t="s">
-        <v>552</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
@@ -7030,19 +7040,19 @@
         <v>2</v>
       </c>
       <c r="F8" s="39" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="H8">
         <v>2</v>
       </c>
       <c r="I8" t="s">
-        <v>662</v>
+        <v>658</v>
       </c>
       <c r="K8">
         <v>1</v>
       </c>
       <c r="L8" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
@@ -7056,7 +7066,7 @@
         <v>3</v>
       </c>
       <c r="F9" t="s">
-        <v>658</v>
+        <v>654</v>
       </c>
       <c r="H9">
         <v>5</v>
@@ -7068,7 +7078,7 @@
         <v>3</v>
       </c>
       <c r="L9" t="s">
-        <v>671</v>
+        <v>667</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
@@ -7076,7 +7086,7 @@
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="E10">
         <v>4</v>
@@ -7088,13 +7098,13 @@
         <v>8</v>
       </c>
       <c r="I10" t="s">
-        <v>659</v>
+        <v>655</v>
       </c>
       <c r="K10">
         <v>4</v>
       </c>
       <c r="L10" t="s">
-        <v>667</v>
+        <v>663</v>
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
@@ -7102,7 +7112,7 @@
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>753</v>
+        <v>749</v>
       </c>
       <c r="E11">
         <v>10</v>
@@ -7120,7 +7130,7 @@
         <v>5</v>
       </c>
       <c r="L11" t="s">
-        <v>746</v>
+        <v>742</v>
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
@@ -7134,19 +7144,19 @@
         <v>12</v>
       </c>
       <c r="F12" t="s">
-        <v>661</v>
+        <v>657</v>
       </c>
       <c r="H12">
         <v>11</v>
       </c>
       <c r="I12" t="s">
-        <v>802</v>
+        <v>798</v>
       </c>
       <c r="K12">
         <v>8</v>
       </c>
       <c r="L12" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
@@ -7154,7 +7164,7 @@
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>754</v>
+        <v>750</v>
       </c>
       <c r="E13">
         <v>13</v>
@@ -7166,13 +7176,13 @@
         <v>14</v>
       </c>
       <c r="I13" t="s">
-        <v>663</v>
+        <v>659</v>
       </c>
       <c r="K13">
         <v>10</v>
       </c>
       <c r="L13" t="s">
-        <v>585</v>
+        <v>582</v>
       </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
@@ -7180,13 +7190,13 @@
         <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>756</v>
+        <v>752</v>
       </c>
       <c r="E14">
         <v>16</v>
       </c>
       <c r="F14" t="s">
-        <v>660</v>
+        <v>656</v>
       </c>
       <c r="H14">
         <v>15</v>
@@ -7198,7 +7208,7 @@
         <v>15</v>
       </c>
       <c r="L14" t="s">
-        <v>669</v>
+        <v>665</v>
       </c>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.25">
@@ -7218,13 +7228,13 @@
         <v>17</v>
       </c>
       <c r="I15" t="s">
-        <v>664</v>
+        <v>660</v>
       </c>
       <c r="K15">
         <v>18</v>
       </c>
       <c r="L15" t="s">
-        <v>668</v>
+        <v>664</v>
       </c>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
@@ -7232,25 +7242,25 @@
         <v>15</v>
       </c>
       <c r="C16" s="39" t="s">
-        <v>760</v>
+        <v>756</v>
       </c>
       <c r="E16">
         <v>20</v>
       </c>
       <c r="F16" t="s">
-        <v>666</v>
+        <v>662</v>
       </c>
       <c r="H16">
         <v>20</v>
       </c>
       <c r="I16" t="s">
-        <v>584</v>
+        <v>581</v>
       </c>
       <c r="K16">
         <v>20</v>
       </c>
       <c r="L16" t="s">
-        <v>797</v>
+        <v>793</v>
       </c>
     </row>
     <row r="17" spans="8:12" x14ac:dyDescent="0.25">
@@ -7258,13 +7268,13 @@
         <v>23</v>
       </c>
       <c r="I17" t="s">
-        <v>546</v>
+        <v>543</v>
       </c>
       <c r="K17">
         <v>21</v>
       </c>
       <c r="L17" t="s">
-        <v>670</v>
+        <v>666</v>
       </c>
     </row>
     <row r="18" spans="8:12" x14ac:dyDescent="0.25">
@@ -7272,38 +7282,38 @@
         <v>25</v>
       </c>
       <c r="I18" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="K18">
         <v>25</v>
       </c>
       <c r="L18" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
     </row>
     <row r="22" spans="8:12" x14ac:dyDescent="0.25">
       <c r="I22" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
     </row>
     <row r="23" spans="8:12" x14ac:dyDescent="0.25">
       <c r="I23" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
     </row>
     <row r="24" spans="8:12" x14ac:dyDescent="0.25">
       <c r="I24" t="s">
-        <v>665</v>
+        <v>661</v>
       </c>
     </row>
     <row r="25" spans="8:12" x14ac:dyDescent="0.25">
       <c r="I25" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
     </row>
     <row r="26" spans="8:12" x14ac:dyDescent="0.25">
       <c r="I26" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
     </row>
   </sheetData>
@@ -8674,10 +8684,10 @@
     <row r="7" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B8" s="35" t="s">
-        <v>673</v>
+        <v>669</v>
       </c>
       <c r="C8" s="36" t="s">
-        <v>672</v>
+        <v>668</v>
       </c>
       <c r="H8" t="s">
         <v>12</v>
@@ -8857,7 +8867,7 @@
         <v>248</v>
       </c>
       <c r="M17" t="s">
-        <v>674</v>
+        <v>670</v>
       </c>
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.25">
@@ -9047,7 +9057,7 @@
         <v>49</v>
       </c>
       <c r="M27" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
     </row>
     <row r="28" spans="2:13" x14ac:dyDescent="0.25">
@@ -9111,7 +9121,7 @@
         <v>63</v>
       </c>
       <c r="I32" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="L32" t="s">
         <v>51</v>
@@ -9122,16 +9132,16 @@
     </row>
     <row r="33" spans="8:13" x14ac:dyDescent="0.25">
       <c r="H33" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="I33" t="s">
-        <v>576</v>
+        <v>573</v>
       </c>
       <c r="L33" t="s">
         <v>54</v>
       </c>
       <c r="M33" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
     </row>
     <row r="34" spans="8:13" x14ac:dyDescent="0.25">
@@ -9139,7 +9149,7 @@
         <v>64</v>
       </c>
       <c r="I34" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="L34" t="s">
         <v>55</v>
@@ -9153,13 +9163,13 @@
         <v>59</v>
       </c>
       <c r="I35" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="L35" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="M35" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
     </row>
     <row r="36" spans="8:13" x14ac:dyDescent="0.25">
@@ -9167,7 +9177,7 @@
         <v>58</v>
       </c>
       <c r="M36" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
     </row>
     <row r="37" spans="8:13" x14ac:dyDescent="0.25">
@@ -9175,7 +9185,7 @@
         <v>61</v>
       </c>
       <c r="M37" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
     </row>
   </sheetData>
@@ -9193,7 +9203,7 @@
   <sheetData>
     <row r="5" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>675</v>
+        <v>671</v>
       </c>
     </row>
     <row r="6" spans="2:2" x14ac:dyDescent="0.25">
@@ -9203,7 +9213,7 @@
     </row>
     <row r="8" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
     </row>
     <row r="9" spans="2:2" x14ac:dyDescent="0.25">
@@ -9233,7 +9243,7 @@
     </row>
     <row r="16" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
     </row>
   </sheetData>
@@ -9350,13 +9360,13 @@
         <v>2</v>
       </c>
       <c r="L8" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="N8">
         <v>2</v>
       </c>
       <c r="O8" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
       <c r="Q8">
         <v>2</v>
@@ -9368,7 +9378,7 @@
         <v>2</v>
       </c>
       <c r="U8" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
     </row>
     <row r="9" spans="2:21" x14ac:dyDescent="0.25">
@@ -9464,19 +9474,19 @@
         <v>8</v>
       </c>
       <c r="C11" s="37" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="E11">
         <v>8</v>
       </c>
       <c r="F11" s="37" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="H11">
         <v>8</v>
       </c>
       <c r="I11" s="37" t="s">
-        <v>782</v>
+        <v>778</v>
       </c>
       <c r="K11">
         <v>10</v>
@@ -9514,7 +9524,7 @@
         <v>10</v>
       </c>
       <c r="F12" t="s">
-        <v>676</v>
+        <v>672</v>
       </c>
       <c r="H12">
         <v>10</v>
@@ -9570,25 +9580,25 @@
         <v>14</v>
       </c>
       <c r="L13" t="s">
-        <v>729</v>
+        <v>725</v>
       </c>
       <c r="N13">
         <v>14</v>
       </c>
       <c r="O13" t="s">
-        <v>729</v>
+        <v>725</v>
       </c>
       <c r="Q13">
         <v>14</v>
       </c>
       <c r="R13" t="s">
-        <v>729</v>
+        <v>725</v>
       </c>
       <c r="T13">
         <v>14</v>
       </c>
       <c r="U13" t="s">
-        <v>729</v>
+        <v>725</v>
       </c>
     </row>
     <row r="14" spans="2:21" x14ac:dyDescent="0.25">
@@ -9602,13 +9612,13 @@
         <v>15</v>
       </c>
       <c r="F14" s="39" t="s">
-        <v>728</v>
+        <v>724</v>
       </c>
       <c r="H14">
         <v>15</v>
       </c>
       <c r="I14" s="39" t="s">
-        <v>728</v>
+        <v>724</v>
       </c>
       <c r="K14">
         <v>15</v>
@@ -9696,25 +9706,25 @@
         <v>20</v>
       </c>
       <c r="L16" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="N16">
         <v>20</v>
       </c>
       <c r="O16" t="s">
-        <v>616</v>
+        <v>613</v>
       </c>
       <c r="Q16">
         <v>20</v>
       </c>
       <c r="R16" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="T16">
         <v>20</v>
       </c>
       <c r="U16" t="s">
-        <v>604</v>
+        <v>601</v>
       </c>
     </row>
     <row r="17" spans="9:21" x14ac:dyDescent="0.25">
@@ -9771,42 +9781,42 @@
     </row>
     <row r="22" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I22" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
     </row>
     <row r="23" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I23" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
     </row>
     <row r="24" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I24" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
     </row>
     <row r="25" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I25" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
     </row>
     <row r="26" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I26" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
     </row>
     <row r="27" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I27" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
     </row>
     <row r="28" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I28" t="s">
-        <v>606</v>
+        <v>603</v>
       </c>
     </row>
     <row r="29" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I29" t="s">
-        <v>607</v>
+        <v>604</v>
       </c>
     </row>
     <row r="36" spans="11:11" x14ac:dyDescent="0.25">
@@ -9897,7 +9907,7 @@
         <v>3</v>
       </c>
       <c r="I8" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="K8">
         <v>3</v>
@@ -9929,13 +9939,13 @@
         <v>5</v>
       </c>
       <c r="I9" t="s">
-        <v>618</v>
+        <v>615</v>
       </c>
       <c r="K9">
         <v>5</v>
       </c>
       <c r="L9" t="s">
-        <v>619</v>
+        <v>616</v>
       </c>
       <c r="N9">
         <v>5</v>
@@ -9961,13 +9971,13 @@
         <v>8</v>
       </c>
       <c r="I10" t="s">
-        <v>677</v>
+        <v>673</v>
       </c>
       <c r="K10">
         <v>8</v>
       </c>
       <c r="L10" t="s">
-        <v>678</v>
+        <v>674</v>
       </c>
       <c r="N10">
         <v>6</v>
@@ -10051,25 +10061,25 @@
         <v>14</v>
       </c>
       <c r="F13" s="39" t="s">
-        <v>727</v>
+        <v>723</v>
       </c>
       <c r="H13">
         <v>14</v>
       </c>
       <c r="I13" t="s">
-        <v>799</v>
+        <v>795</v>
       </c>
       <c r="K13">
         <v>14</v>
       </c>
       <c r="L13" t="s">
-        <v>799</v>
+        <v>795</v>
       </c>
       <c r="N13">
         <v>14</v>
       </c>
       <c r="O13" t="s">
-        <v>800</v>
+        <v>796</v>
       </c>
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.25">
@@ -10101,7 +10111,7 @@
         <v>15</v>
       </c>
       <c r="O14" t="s">
-        <v>731</v>
+        <v>727</v>
       </c>
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.25">
@@ -10147,19 +10157,19 @@
         <v>20</v>
       </c>
       <c r="I16" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="K16">
         <v>20</v>
       </c>
       <c r="L16" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="N16">
         <v>21</v>
       </c>
       <c r="O16" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
     </row>
     <row r="17" spans="8:15" x14ac:dyDescent="0.25">
@@ -10187,13 +10197,13 @@
         <v>25</v>
       </c>
       <c r="I18" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="K18">
         <v>25</v>
       </c>
       <c r="L18" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
       <c r="N18">
         <v>25</v>
@@ -10204,27 +10214,27 @@
     </row>
     <row r="22" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I22" t="s">
-        <v>698</v>
+        <v>694</v>
       </c>
     </row>
     <row r="23" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I23" t="s">
-        <v>700</v>
+        <v>696</v>
       </c>
     </row>
     <row r="24" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I24" t="s">
-        <v>701</v>
+        <v>697</v>
       </c>
     </row>
     <row r="25" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I25" t="s">
-        <v>699</v>
+        <v>695</v>
       </c>
     </row>
     <row r="26" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I26" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
     </row>
   </sheetData>
@@ -10332,7 +10342,7 @@
         <v>4</v>
       </c>
       <c r="C9" t="s">
-        <v>783</v>
+        <v>779</v>
       </c>
       <c r="E9">
         <v>4</v>
@@ -10344,7 +10354,7 @@
         <v>5</v>
       </c>
       <c r="I9" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="K9">
         <v>5</v>
@@ -10370,7 +10380,7 @@
         <v>4</v>
       </c>
       <c r="F10" t="s">
-        <v>720</v>
+        <v>716</v>
       </c>
       <c r="H10">
         <v>8</v>
@@ -10382,7 +10392,7 @@
         <v>7</v>
       </c>
       <c r="L10" t="s">
-        <v>785</v>
+        <v>781</v>
       </c>
       <c r="N10">
         <v>5</v>
@@ -10434,7 +10444,7 @@
         <v>8</v>
       </c>
       <c r="F12" t="s">
-        <v>784</v>
+        <v>780</v>
       </c>
       <c r="H12">
         <v>12</v>
@@ -10446,7 +10456,7 @@
         <v>10</v>
       </c>
       <c r="L12" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="N12">
         <v>10</v>
@@ -10466,7 +10476,7 @@
         <v>11</v>
       </c>
       <c r="F13" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="H13">
         <v>14</v>
@@ -10492,7 +10502,7 @@
         <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>719</v>
+        <v>715</v>
       </c>
       <c r="E14">
         <v>14</v>
@@ -10510,7 +10520,7 @@
         <v>15</v>
       </c>
       <c r="L14" t="s">
-        <v>735</v>
+        <v>731</v>
       </c>
       <c r="N14">
         <v>17</v>
@@ -10536,7 +10546,7 @@
         <v>16</v>
       </c>
       <c r="I15" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="K15">
         <v>16</v>
@@ -10574,7 +10584,7 @@
         <v>17</v>
       </c>
       <c r="L16" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="N16">
         <v>21</v>
@@ -10620,7 +10630,7 @@
         <v>25</v>
       </c>
       <c r="O18" t="s">
-        <v>687</v>
+        <v>683</v>
       </c>
     </row>
   </sheetData>
@@ -10677,7 +10687,7 @@
         <v>1</v>
       </c>
       <c r="L7" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
@@ -10723,13 +10733,13 @@
         <v>5</v>
       </c>
       <c r="I9" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="K9">
         <v>5</v>
       </c>
       <c r="L9" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
@@ -10769,7 +10779,7 @@
         <v>10</v>
       </c>
       <c r="F11" t="s">
-        <v>711</v>
+        <v>707</v>
       </c>
       <c r="H11">
         <v>10</v>
@@ -10781,7 +10791,7 @@
         <v>7</v>
       </c>
       <c r="L11" t="s">
-        <v>789</v>
+        <v>785</v>
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
@@ -10807,7 +10817,7 @@
         <v>9</v>
       </c>
       <c r="L12" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
@@ -10815,13 +10825,13 @@
         <v>10</v>
       </c>
       <c r="C13" t="s">
-        <v>710</v>
+        <v>706</v>
       </c>
       <c r="E13">
         <v>14</v>
       </c>
       <c r="F13" s="39" t="s">
-        <v>742</v>
+        <v>738</v>
       </c>
       <c r="H13">
         <v>14</v>
@@ -10833,7 +10843,7 @@
         <v>11</v>
       </c>
       <c r="L13" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
@@ -10853,7 +10863,7 @@
         <v>15</v>
       </c>
       <c r="I14" t="s">
-        <v>654</v>
+        <v>650</v>
       </c>
       <c r="K14">
         <v>16</v>
@@ -10879,13 +10889,13 @@
         <v>16</v>
       </c>
       <c r="I15" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="K15">
         <v>20</v>
       </c>
       <c r="L15" t="s">
-        <v>775</v>
+        <v>771</v>
       </c>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
@@ -10925,7 +10935,7 @@
         <v>22</v>
       </c>
       <c r="L17" t="s">
-        <v>786</v>
+        <v>782</v>
       </c>
     </row>
     <row r="18" spans="8:12" x14ac:dyDescent="0.25">
@@ -10939,7 +10949,7 @@
         <v>25</v>
       </c>
       <c r="L18" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
     </row>
   </sheetData>
@@ -11162,7 +11172,7 @@
         <v>8</v>
       </c>
       <c r="U10" t="s">
-        <v>757</v>
+        <v>753</v>
       </c>
     </row>
     <row r="11" spans="2:21" x14ac:dyDescent="0.25">
@@ -11188,25 +11198,25 @@
         <v>10</v>
       </c>
       <c r="L11" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="N11">
         <v>9</v>
       </c>
       <c r="O11" t="s">
-        <v>730</v>
+        <v>726</v>
       </c>
       <c r="Q11">
         <v>9</v>
       </c>
       <c r="R11" t="s">
-        <v>730</v>
+        <v>726</v>
       </c>
       <c r="T11">
         <v>9</v>
       </c>
       <c r="U11" t="s">
-        <v>730</v>
+        <v>726</v>
       </c>
     </row>
     <row r="12" spans="2:21" x14ac:dyDescent="0.25">
@@ -11250,7 +11260,7 @@
         <v>12</v>
       </c>
       <c r="U12" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="13" spans="2:21" x14ac:dyDescent="0.25">
@@ -11282,19 +11292,19 @@
         <v>14</v>
       </c>
       <c r="O13" t="s">
-        <v>747</v>
+        <v>743</v>
       </c>
       <c r="Q13">
         <v>14</v>
       </c>
       <c r="R13" t="s">
-        <v>749</v>
+        <v>745</v>
       </c>
       <c r="T13">
         <v>14</v>
       </c>
       <c r="U13" t="s">
-        <v>751</v>
+        <v>747</v>
       </c>
     </row>
     <row r="14" spans="2:21" x14ac:dyDescent="0.25">
@@ -11338,7 +11348,7 @@
         <v>15</v>
       </c>
       <c r="U14" t="s">
-        <v>750</v>
+        <v>746</v>
       </c>
     </row>
     <row r="15" spans="2:21" x14ac:dyDescent="0.25">
@@ -11370,19 +11380,19 @@
         <v>17</v>
       </c>
       <c r="O15" t="s">
-        <v>683</v>
+        <v>679</v>
       </c>
       <c r="Q15">
         <v>17</v>
       </c>
       <c r="R15" t="s">
-        <v>682</v>
+        <v>678</v>
       </c>
       <c r="T15">
         <v>17</v>
       </c>
       <c r="U15" t="s">
-        <v>684</v>
+        <v>680</v>
       </c>
     </row>
     <row r="16" spans="2:21" x14ac:dyDescent="0.25">
@@ -11414,7 +11424,7 @@
         <v>21</v>
       </c>
       <c r="O16" t="s">
-        <v>748</v>
+        <v>744</v>
       </c>
       <c r="Q16">
         <v>21</v>
@@ -11426,7 +11436,7 @@
         <v>21</v>
       </c>
       <c r="U16" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
     </row>
     <row r="17" spans="9:21" x14ac:dyDescent="0.25">
@@ -11434,19 +11444,19 @@
         <v>22</v>
       </c>
       <c r="O17" t="s">
-        <v>679</v>
+        <v>675</v>
       </c>
       <c r="Q17">
         <v>22</v>
       </c>
       <c r="R17" t="s">
-        <v>680</v>
+        <v>676</v>
       </c>
       <c r="T17">
         <v>22</v>
       </c>
       <c r="U17" t="s">
-        <v>681</v>
+        <v>677</v>
       </c>
     </row>
     <row r="18" spans="9:21" x14ac:dyDescent="0.25">
@@ -11501,7 +11511,7 @@
     </row>
     <row r="30" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I30" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
restauro las fases y añadidos por fin TODAS las skills
</commit_message>
<xml_diff>
--- a/arquetiposZ.xlsx
+++ b/arquetiposZ.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sergius\Desktop\Proyectos\hyperbole\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CF67934-CC51-47B7-B03C-EB74BD0A289F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{850299BE-B260-4CE5-906E-5FC3ABA798CB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="644" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="644" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RESUMEN" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1146" uniqueCount="814">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1147" uniqueCount="814">
   <si>
     <t>daños:</t>
   </si>
@@ -1741,9 +1741,6 @@
     <t>almighty fis leve dinero</t>
   </si>
   <si>
-    <t>aum fuerza dinero</t>
-  </si>
-  <si>
     <t>daga, florete</t>
   </si>
   <si>
@@ -2290,21 +2287,9 @@
     <t>[ballesta 7]</t>
   </si>
   <si>
-    <t>resistir quemadura/congelacion</t>
-  </si>
-  <si>
-    <t>resistir paralisis/mareo</t>
-  </si>
-  <si>
-    <t>resistir veneno/amnesia</t>
-  </si>
-  <si>
     <t>+10% precision</t>
   </si>
   <si>
-    <t>resistir sueño/furia</t>
-  </si>
-  <si>
     <t>[ballesta 3 back confusión]</t>
   </si>
   <si>
@@ -2486,6 +2471,21 @@
   </si>
   <si>
     <t>knight's proclamation</t>
+  </si>
+  <si>
+    <t>resistir miedo/desesp/sueño</t>
+  </si>
+  <si>
+    <t>resistir veneno/furia</t>
+  </si>
+  <si>
+    <t>resistir lavado/amnesia</t>
+  </si>
+  <si>
+    <t>resistir quemadura/mareo</t>
+  </si>
+  <si>
+    <t>resistir paralisis/cong</t>
   </si>
 </sst>
 </file>
@@ -4752,7 +4752,7 @@
         <v>15</v>
       </c>
       <c r="G12" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="J12">
         <v>10</v>
@@ -4818,15 +4818,15 @@
         <v>17</v>
       </c>
       <c r="K15" t="s">
-        <v>400</v>
+        <v>412</v>
       </c>
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.25">
       <c r="J16">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="K16" t="s">
-        <v>412</v>
+        <v>400</v>
       </c>
     </row>
     <row r="17" spans="8:11" x14ac:dyDescent="0.25">
@@ -4834,7 +4834,7 @@
         <v>24</v>
       </c>
       <c r="K17" t="s">
-        <v>783</v>
+        <v>778</v>
       </c>
     </row>
     <row r="18" spans="8:11" x14ac:dyDescent="0.25">
@@ -4877,7 +4877,7 @@
     </row>
     <row r="30" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H30" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
     </row>
     <row r="31" spans="8:11" x14ac:dyDescent="0.25">
@@ -4887,7 +4887,7 @@
     </row>
     <row r="32" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H32" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
     </row>
     <row r="33" spans="8:8" x14ac:dyDescent="0.25">
@@ -4949,7 +4949,7 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>813</v>
+        <v>808</v>
       </c>
       <c r="H7">
         <v>1</v>
@@ -4967,7 +4967,7 @@
         <v>1</v>
       </c>
       <c r="O7" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="Q7">
         <v>1</v>
@@ -5143,13 +5143,13 @@
         <v>9</v>
       </c>
       <c r="O11" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="Q11">
         <v>10</v>
       </c>
       <c r="R11" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="T11">
         <v>6</v>
@@ -5175,7 +5175,7 @@
         <v>10</v>
       </c>
       <c r="I12" t="s">
-        <v>769</v>
+        <v>764</v>
       </c>
       <c r="K12">
         <v>12</v>
@@ -5187,7 +5187,7 @@
         <v>10</v>
       </c>
       <c r="O12" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="Q12">
         <v>12</v>
@@ -5219,7 +5219,7 @@
         <v>10</v>
       </c>
       <c r="I13" t="s">
-        <v>770</v>
+        <v>765</v>
       </c>
       <c r="K13">
         <v>14</v>
@@ -5231,7 +5231,7 @@
         <v>11</v>
       </c>
       <c r="O13" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="Q13">
         <v>14</v>
@@ -5243,7 +5243,7 @@
         <v>12</v>
       </c>
       <c r="U13" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="14" spans="2:22" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>13</v>
       </c>
       <c r="C14" s="39" t="s">
-        <v>754</v>
+        <v>749</v>
       </c>
       <c r="E14">
         <v>16</v>
@@ -5269,13 +5269,13 @@
         <v>15</v>
       </c>
       <c r="L14" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="N14">
         <v>12</v>
       </c>
       <c r="O14" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="Q14">
         <v>15</v>
@@ -5301,7 +5301,7 @@
         <v>18</v>
       </c>
       <c r="F15" t="s">
-        <v>791</v>
+        <v>786</v>
       </c>
       <c r="H15">
         <v>16</v>
@@ -5313,7 +5313,7 @@
         <v>16</v>
       </c>
       <c r="L15" t="s">
-        <v>784</v>
+        <v>779</v>
       </c>
       <c r="N15">
         <v>13</v>
@@ -5351,13 +5351,13 @@
         <v>20</v>
       </c>
       <c r="L16" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="N16">
         <v>15</v>
       </c>
       <c r="O16" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="Q16">
         <v>20</v>
@@ -5372,7 +5372,7 @@
         <v>493</v>
       </c>
       <c r="V16" t="s">
-        <v>810</v>
+        <v>805</v>
       </c>
     </row>
     <row r="17" spans="9:21" x14ac:dyDescent="0.25">
@@ -5386,7 +5386,7 @@
         <v>20</v>
       </c>
       <c r="O17" t="s">
-        <v>790</v>
+        <v>785</v>
       </c>
       <c r="Q17">
         <v>23</v>
@@ -5398,7 +5398,7 @@
         <v>23</v>
       </c>
       <c r="U17" t="s">
-        <v>809</v>
+        <v>804</v>
       </c>
     </row>
     <row r="18" spans="9:21" x14ac:dyDescent="0.25">
@@ -5424,7 +5424,7 @@
         <v>25</v>
       </c>
       <c r="U18" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="21" spans="9:21" x14ac:dyDescent="0.25">
@@ -5489,7 +5489,7 @@
     </row>
     <row r="33" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I33" t="s">
-        <v>812</v>
+        <v>807</v>
       </c>
     </row>
     <row r="34" spans="9:9" x14ac:dyDescent="0.25">
@@ -5509,7 +5509,7 @@
     </row>
     <row r="37" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I37" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
   </sheetData>
@@ -5574,7 +5574,7 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>801</v>
+        <v>796</v>
       </c>
       <c r="H7">
         <v>1</v>
@@ -5586,7 +5586,7 @@
         <v>1</v>
       </c>
       <c r="L7" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="N7">
         <v>1</v>
@@ -5598,13 +5598,13 @@
         <v>1</v>
       </c>
       <c r="R7" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="T7">
         <v>1</v>
       </c>
       <c r="U7" s="39" t="s">
-        <v>767</v>
+        <v>762</v>
       </c>
     </row>
     <row r="8" spans="2:21" x14ac:dyDescent="0.25">
@@ -5630,13 +5630,13 @@
         <v>1</v>
       </c>
       <c r="L8" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="N8">
         <v>1</v>
       </c>
       <c r="O8" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="Q8">
         <v>3</v>
@@ -5648,7 +5648,7 @@
         <v>1</v>
       </c>
       <c r="U8" t="s">
-        <v>765</v>
+        <v>760</v>
       </c>
     </row>
     <row r="9" spans="2:21" x14ac:dyDescent="0.25">
@@ -5656,7 +5656,7 @@
         <v>4</v>
       </c>
       <c r="C9" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -5686,13 +5686,13 @@
         <v>7</v>
       </c>
       <c r="R9" t="s">
-        <v>760</v>
+        <v>755</v>
       </c>
       <c r="T9">
         <v>1</v>
       </c>
       <c r="U9" t="s">
-        <v>766</v>
+        <v>761</v>
       </c>
     </row>
     <row r="10" spans="2:21" x14ac:dyDescent="0.25">
@@ -5700,31 +5700,31 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E10">
         <v>5</v>
       </c>
       <c r="F10" t="s">
-        <v>805</v>
+        <v>800</v>
       </c>
       <c r="H10">
         <v>7</v>
       </c>
       <c r="I10" t="s">
-        <v>758</v>
+        <v>753</v>
       </c>
       <c r="K10">
         <v>5</v>
       </c>
       <c r="L10" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="N10">
         <v>5</v>
       </c>
       <c r="O10" t="s">
-        <v>799</v>
+        <v>794</v>
       </c>
       <c r="Q10">
         <v>10</v>
@@ -5744,13 +5744,13 @@
         <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="E11">
         <v>10</v>
       </c>
       <c r="F11" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="H11">
         <v>10</v>
@@ -5774,7 +5774,7 @@
         <v>11</v>
       </c>
       <c r="R11" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="T11">
         <v>7</v>
@@ -5794,19 +5794,19 @@
         <v>12</v>
       </c>
       <c r="F12" s="39" t="s">
-        <v>755</v>
+        <v>750</v>
       </c>
       <c r="H12">
         <v>15</v>
       </c>
       <c r="I12" t="s">
-        <v>759</v>
+        <v>754</v>
       </c>
       <c r="K12">
         <v>11</v>
       </c>
       <c r="L12" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
       <c r="N12">
         <v>12</v>
@@ -5818,7 +5818,7 @@
         <v>12</v>
       </c>
       <c r="R12" t="s">
-        <v>761</v>
+        <v>756</v>
       </c>
       <c r="T12">
         <v>10</v>
@@ -5850,7 +5850,7 @@
         <v>14</v>
       </c>
       <c r="L13" t="s">
-        <v>803</v>
+        <v>798</v>
       </c>
       <c r="N13">
         <v>12</v>
@@ -5862,7 +5862,7 @@
         <v>12</v>
       </c>
       <c r="R13" t="s">
-        <v>762</v>
+        <v>757</v>
       </c>
       <c r="T13">
         <v>11</v>
@@ -5894,7 +5894,7 @@
         <v>16</v>
       </c>
       <c r="L14" t="s">
-        <v>802</v>
+        <v>797</v>
       </c>
       <c r="N14">
         <v>15</v>
@@ -5932,13 +5932,13 @@
         <v>20</v>
       </c>
       <c r="I15" t="s">
-        <v>808</v>
+        <v>803</v>
       </c>
       <c r="K15">
         <v>18</v>
       </c>
       <c r="L15" t="s">
-        <v>804</v>
+        <v>799</v>
       </c>
       <c r="N15">
         <v>18</v>
@@ -5956,7 +5956,7 @@
         <v>15</v>
       </c>
       <c r="U15" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
     </row>
     <row r="16" spans="2:21" x14ac:dyDescent="0.25">
@@ -5964,25 +5964,25 @@
         <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="E16">
         <v>20</v>
       </c>
       <c r="F16" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="H16">
         <v>20</v>
       </c>
       <c r="I16" t="s">
-        <v>757</v>
+        <v>752</v>
       </c>
       <c r="K16">
         <v>21</v>
       </c>
       <c r="L16" t="s">
-        <v>807</v>
+        <v>802</v>
       </c>
       <c r="N16">
         <v>20</v>
@@ -6000,7 +6000,7 @@
         <v>19</v>
       </c>
       <c r="U16" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
     <row r="17" spans="10:21" x14ac:dyDescent="0.25">
@@ -6008,7 +6008,7 @@
         <v>22</v>
       </c>
       <c r="L17" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="N17">
         <v>20</v>
@@ -6034,7 +6034,7 @@
         <v>25</v>
       </c>
       <c r="L18" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="N18">
         <v>25</v>
@@ -6072,22 +6072,22 @@
     </row>
     <row r="25" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J25" t="s">
-        <v>763</v>
+        <v>758</v>
       </c>
     </row>
     <row r="26" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J26" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
     </row>
     <row r="27" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J27" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
     </row>
     <row r="28" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J28" t="s">
-        <v>764</v>
+        <v>759</v>
       </c>
     </row>
     <row r="29" spans="10:21" x14ac:dyDescent="0.25">
@@ -6102,12 +6102,12 @@
     </row>
     <row r="31" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J31" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
     </row>
     <row r="32" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J32" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
     </row>
     <row r="33" spans="10:10" x14ac:dyDescent="0.25">
@@ -6117,12 +6117,12 @@
     </row>
     <row r="34" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J34" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
     </row>
     <row r="35" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J35" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
     </row>
   </sheetData>
@@ -6157,13 +6157,13 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>787</v>
+        <v>782</v>
       </c>
       <c r="J7">
         <v>1</v>
@@ -6177,7 +6177,7 @@
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="F8">
         <v>1</v>
@@ -6197,13 +6197,13 @@
         <v>5</v>
       </c>
       <c r="C9" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="F9">
         <v>3</v>
       </c>
       <c r="G9" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="J9">
         <v>7</v>
@@ -6223,7 +6223,7 @@
         <v>6</v>
       </c>
       <c r="G10" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="J10">
         <v>8</v>
@@ -6237,19 +6237,19 @@
         <v>7</v>
       </c>
       <c r="C11" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="F11">
         <v>7</v>
       </c>
       <c r="G11" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="J11">
         <v>11</v>
       </c>
       <c r="K11" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.25">
@@ -6257,19 +6257,19 @@
         <v>8</v>
       </c>
       <c r="C12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="F12">
         <v>8</v>
       </c>
       <c r="G12" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="J12">
         <v>11</v>
       </c>
       <c r="K12" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.25">
@@ -6277,7 +6277,7 @@
         <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="F13">
         <v>12</v>
@@ -6289,7 +6289,7 @@
         <v>13</v>
       </c>
       <c r="K13" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="14" spans="2:11" x14ac:dyDescent="0.25">
@@ -6303,13 +6303,13 @@
         <v>16</v>
       </c>
       <c r="G14" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="J14">
         <v>15</v>
       </c>
       <c r="K14" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.25">
@@ -6317,19 +6317,19 @@
         <v>13</v>
       </c>
       <c r="C15" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="F15">
         <v>19</v>
       </c>
       <c r="G15" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="J15">
         <v>18</v>
       </c>
       <c r="K15" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.25">
@@ -6337,7 +6337,7 @@
         <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="F16">
         <v>20</v>
@@ -6349,7 +6349,7 @@
         <v>20</v>
       </c>
       <c r="K16" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
     </row>
     <row r="17" spans="10:11" x14ac:dyDescent="0.25">
@@ -6357,7 +6357,7 @@
         <v>20</v>
       </c>
       <c r="K17" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
     </row>
     <row r="18" spans="10:11" x14ac:dyDescent="0.25">
@@ -6365,27 +6365,27 @@
         <v>25</v>
       </c>
       <c r="K18" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
     </row>
     <row r="27" spans="10:11" x14ac:dyDescent="0.25">
       <c r="K27" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
     </row>
     <row r="28" spans="10:11" x14ac:dyDescent="0.25">
       <c r="K28" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
     </row>
     <row r="29" spans="10:11" x14ac:dyDescent="0.25">
       <c r="K29" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
     </row>
     <row r="30" spans="10:11" x14ac:dyDescent="0.25">
       <c r="K30" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
     </row>
   </sheetData>
@@ -6438,7 +6438,7 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -6462,7 +6462,7 @@
         <v>1</v>
       </c>
       <c r="O7" t="s">
-        <v>499</v>
+        <v>538</v>
       </c>
       <c r="Q7">
         <v>1</v>
@@ -6474,7 +6474,7 @@
         <v>1</v>
       </c>
       <c r="V7" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
     </row>
     <row r="8" spans="2:22" x14ac:dyDescent="0.25">
@@ -6482,7 +6482,7 @@
         <v>3</v>
       </c>
       <c r="C8" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="E8">
         <v>4</v>
@@ -6512,13 +6512,13 @@
         <v>3</v>
       </c>
       <c r="R8" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="U8">
         <v>2</v>
       </c>
       <c r="V8" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
     </row>
     <row r="9" spans="2:22" x14ac:dyDescent="0.25">
@@ -6526,13 +6526,13 @@
         <v>5</v>
       </c>
       <c r="C9" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="E9">
         <v>4</v>
       </c>
       <c r="F9" t="s">
-        <v>593</v>
+        <v>567</v>
       </c>
       <c r="H9">
         <v>4</v>
@@ -6562,7 +6562,7 @@
         <v>2</v>
       </c>
       <c r="V9" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="10" spans="2:22" x14ac:dyDescent="0.25">
@@ -6576,19 +6576,19 @@
         <v>6</v>
       </c>
       <c r="F10" t="s">
-        <v>571</v>
+        <v>592</v>
       </c>
       <c r="H10">
         <v>5</v>
       </c>
       <c r="I10" t="s">
-        <v>526</v>
+        <v>492</v>
       </c>
       <c r="K10">
         <v>8</v>
       </c>
       <c r="L10" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="N10">
         <v>8</v>
@@ -6606,7 +6606,7 @@
         <v>6</v>
       </c>
       <c r="V10" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
     </row>
     <row r="11" spans="2:22" x14ac:dyDescent="0.25">
@@ -6614,19 +6614,19 @@
         <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="E11">
         <v>8</v>
       </c>
       <c r="F11" t="s">
-        <v>586</v>
+        <v>570</v>
       </c>
       <c r="H11">
         <v>7</v>
       </c>
       <c r="I11" t="s">
-        <v>492</v>
+        <v>321</v>
       </c>
       <c r="K11">
         <v>10</v>
@@ -6650,7 +6650,7 @@
         <v>7</v>
       </c>
       <c r="V11" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
     </row>
     <row r="12" spans="2:22" x14ac:dyDescent="0.25">
@@ -6658,19 +6658,19 @@
         <v>10</v>
       </c>
       <c r="C12" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="E12">
         <v>11</v>
       </c>
       <c r="F12" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
       <c r="H12">
         <v>8</v>
       </c>
       <c r="I12" t="s">
-        <v>494</v>
+        <v>526</v>
       </c>
       <c r="K12">
         <v>12</v>
@@ -6694,7 +6694,7 @@
         <v>8</v>
       </c>
       <c r="V12" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="13" spans="2:22" x14ac:dyDescent="0.25">
@@ -6702,43 +6702,43 @@
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="E13">
         <v>14</v>
       </c>
       <c r="F13" t="s">
-        <v>538</v>
+        <v>587</v>
       </c>
       <c r="H13">
         <v>9</v>
       </c>
       <c r="I13" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="K13">
         <v>14</v>
       </c>
       <c r="L13" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="N13">
         <v>14</v>
       </c>
       <c r="O13" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="Q13">
         <v>14</v>
       </c>
       <c r="R13" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="U13">
         <v>9</v>
       </c>
       <c r="V13" t="s">
-        <v>794</v>
+        <v>789</v>
       </c>
     </row>
     <row r="14" spans="2:22" x14ac:dyDescent="0.25">
@@ -6746,7 +6746,7 @@
         <v>14</v>
       </c>
       <c r="C14" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="E14">
         <v>16</v>
@@ -6758,7 +6758,7 @@
         <v>11</v>
       </c>
       <c r="I14" t="s">
-        <v>702</v>
+        <v>494</v>
       </c>
       <c r="K14">
         <v>15</v>
@@ -6782,7 +6782,7 @@
         <v>14</v>
       </c>
       <c r="V14" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
     </row>
     <row r="15" spans="2:22" x14ac:dyDescent="0.25">
@@ -6790,19 +6790,19 @@
         <v>15</v>
       </c>
       <c r="C15" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="E15">
         <v>18</v>
       </c>
       <c r="F15" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="H15">
         <v>16</v>
       </c>
       <c r="I15" t="s">
-        <v>565</v>
+        <v>701</v>
       </c>
       <c r="K15">
         <v>20</v>
@@ -6820,13 +6820,13 @@
         <v>16</v>
       </c>
       <c r="R15" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="U15">
         <v>17</v>
       </c>
       <c r="V15" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
     </row>
     <row r="16" spans="2:22" x14ac:dyDescent="0.25">
@@ -6852,19 +6852,19 @@
         <v>20</v>
       </c>
       <c r="O16" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="Q16">
         <v>20</v>
       </c>
       <c r="R16" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="U16">
         <v>20</v>
       </c>
       <c r="V16" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
     </row>
     <row r="17" spans="11:22" x14ac:dyDescent="0.25">
@@ -6878,7 +6878,7 @@
         <v>23</v>
       </c>
       <c r="O17" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="Q17">
         <v>24</v>
@@ -6890,7 +6890,7 @@
         <v>24</v>
       </c>
       <c r="V17" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
     </row>
     <row r="18" spans="11:22" x14ac:dyDescent="0.25">
@@ -6898,75 +6898,75 @@
         <v>25</v>
       </c>
       <c r="L18" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="N18">
         <v>25</v>
       </c>
       <c r="O18" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="Q18">
         <v>25</v>
       </c>
       <c r="R18" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="U18">
         <v>25</v>
       </c>
       <c r="V18" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="22" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L22" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
     </row>
     <row r="23" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L23" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
     </row>
     <row r="24" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L24" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
     </row>
     <row r="25" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L25" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="26" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L26" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
     </row>
     <row r="27" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L27" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
     </row>
     <row r="28" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L28" t="s">
-        <v>786</v>
+        <v>781</v>
       </c>
     </row>
     <row r="29" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L29" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
     </row>
     <row r="30" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L30" t="s">
-        <v>789</v>
+        <v>784</v>
       </c>
     </row>
     <row r="33" spans="13:13" x14ac:dyDescent="0.25">
       <c r="M33" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
     </row>
   </sheetData>
@@ -7020,7 +7020,7 @@
         <v>1</v>
       </c>
       <c r="I7" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="K7">
         <v>1</v>
@@ -7040,19 +7040,19 @@
         <v>2</v>
       </c>
       <c r="F8" s="39" t="s">
-        <v>751</v>
+        <v>747</v>
       </c>
       <c r="H8">
         <v>2</v>
       </c>
       <c r="I8" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="K8">
         <v>1</v>
       </c>
       <c r="L8" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
@@ -7060,13 +7060,13 @@
         <v>2</v>
       </c>
       <c r="C9" t="s">
-        <v>312</v>
+        <v>812</v>
       </c>
       <c r="E9">
         <v>3</v>
       </c>
       <c r="F9" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="H9">
         <v>5</v>
@@ -7078,15 +7078,15 @@
         <v>3</v>
       </c>
       <c r="L9" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C10" t="s">
-        <v>748</v>
+        <v>312</v>
       </c>
       <c r="E10">
         <v>4</v>
@@ -7098,27 +7098,27 @@
         <v>8</v>
       </c>
       <c r="I10" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="K10">
         <v>4</v>
       </c>
       <c r="L10" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C11" t="s">
-        <v>749</v>
+        <v>810</v>
       </c>
       <c r="E11">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F11" t="s">
-        <v>283</v>
+        <v>809</v>
       </c>
       <c r="H11">
         <v>10</v>
@@ -7130,7 +7130,7 @@
         <v>5</v>
       </c>
       <c r="L11" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
@@ -7141,16 +7141,16 @@
         <v>320</v>
       </c>
       <c r="E12">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F12" t="s">
-        <v>657</v>
+        <v>283</v>
       </c>
       <c r="H12">
         <v>11</v>
       </c>
       <c r="I12" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="K12">
         <v>8</v>
@@ -7164,25 +7164,25 @@
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>750</v>
+        <v>813</v>
       </c>
       <c r="E13">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F13" t="s">
-        <v>354</v>
+        <v>656</v>
       </c>
       <c r="H13">
         <v>14</v>
       </c>
       <c r="I13" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="K13">
         <v>10</v>
       </c>
       <c r="L13" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
@@ -7190,13 +7190,13 @@
         <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>752</v>
+        <v>811</v>
       </c>
       <c r="E14">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F14" t="s">
-        <v>656</v>
+        <v>354</v>
       </c>
       <c r="H14">
         <v>15</v>
@@ -7208,7 +7208,7 @@
         <v>15</v>
       </c>
       <c r="L14" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.25">
@@ -7219,22 +7219,22 @@
         <v>233</v>
       </c>
       <c r="E15">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F15" t="s">
-        <v>237</v>
+        <v>655</v>
       </c>
       <c r="H15">
         <v>17</v>
       </c>
       <c r="I15" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="K15">
         <v>18</v>
       </c>
       <c r="L15" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
@@ -7242,28 +7242,34 @@
         <v>15</v>
       </c>
       <c r="C16" s="39" t="s">
-        <v>756</v>
+        <v>751</v>
       </c>
       <c r="E16">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F16" t="s">
-        <v>662</v>
+        <v>237</v>
       </c>
       <c r="H16">
         <v>20</v>
       </c>
       <c r="I16" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="K16">
         <v>20</v>
       </c>
       <c r="L16" t="s">
-        <v>793</v>
-      </c>
-    </row>
-    <row r="17" spans="8:12" x14ac:dyDescent="0.25">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="17" spans="5:12" x14ac:dyDescent="0.25">
+      <c r="E17">
+        <v>20</v>
+      </c>
+      <c r="F17" t="s">
+        <v>661</v>
+      </c>
       <c r="H17">
         <v>23</v>
       </c>
@@ -7274,15 +7280,15 @@
         <v>21</v>
       </c>
       <c r="L17" t="s">
-        <v>666</v>
-      </c>
-    </row>
-    <row r="18" spans="8:12" x14ac:dyDescent="0.25">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="18" spans="5:12" x14ac:dyDescent="0.25">
       <c r="H18">
         <v>25</v>
       </c>
       <c r="I18" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="K18">
         <v>25</v>
@@ -7291,27 +7297,27 @@
         <v>544</v>
       </c>
     </row>
-    <row r="22" spans="8:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="5:12" x14ac:dyDescent="0.25">
       <c r="I22" t="s">
         <v>547</v>
       </c>
     </row>
-    <row r="23" spans="8:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="5:12" x14ac:dyDescent="0.25">
       <c r="I23" t="s">
         <v>548</v>
       </c>
     </row>
-    <row r="24" spans="8:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="5:12" x14ac:dyDescent="0.25">
       <c r="I24" t="s">
-        <v>661</v>
-      </c>
-    </row>
-    <row r="25" spans="8:12" x14ac:dyDescent="0.25">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="25" spans="5:12" x14ac:dyDescent="0.25">
       <c r="I25" t="s">
         <v>550</v>
       </c>
     </row>
-    <row r="26" spans="8:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="5:12" x14ac:dyDescent="0.25">
       <c r="I26" t="s">
         <v>551</v>
       </c>
@@ -8684,10 +8690,10 @@
     <row r="7" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B8" s="35" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="C8" s="36" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="H8" t="s">
         <v>12</v>
@@ -8867,7 +8873,7 @@
         <v>248</v>
       </c>
       <c r="M17" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.25">
@@ -9121,7 +9127,7 @@
         <v>63</v>
       </c>
       <c r="I32" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="L32" t="s">
         <v>51</v>
@@ -9135,13 +9141,13 @@
         <v>512</v>
       </c>
       <c r="I33" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="L33" t="s">
         <v>54</v>
       </c>
       <c r="M33" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="34" spans="8:13" x14ac:dyDescent="0.25">
@@ -9149,7 +9155,7 @@
         <v>64</v>
       </c>
       <c r="I34" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="L34" t="s">
         <v>55</v>
@@ -9163,13 +9169,13 @@
         <v>59</v>
       </c>
       <c r="I35" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="L35" t="s">
         <v>532</v>
       </c>
       <c r="M35" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="36" spans="8:13" x14ac:dyDescent="0.25">
@@ -9177,7 +9183,7 @@
         <v>58</v>
       </c>
       <c r="M36" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
     </row>
     <row r="37" spans="8:13" x14ac:dyDescent="0.25">
@@ -9185,7 +9191,7 @@
         <v>61</v>
       </c>
       <c r="M37" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
     </row>
   </sheetData>
@@ -9203,7 +9209,7 @@
   <sheetData>
     <row r="5" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
     </row>
     <row r="6" spans="2:2" x14ac:dyDescent="0.25">
@@ -9360,13 +9366,13 @@
         <v>2</v>
       </c>
       <c r="L8" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="N8">
         <v>2</v>
       </c>
       <c r="O8" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="Q8">
         <v>2</v>
@@ -9378,7 +9384,7 @@
         <v>2</v>
       </c>
       <c r="U8" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="9" spans="2:21" x14ac:dyDescent="0.25">
@@ -9474,19 +9480,19 @@
         <v>8</v>
       </c>
       <c r="C11" s="37" t="s">
-        <v>776</v>
+        <v>771</v>
       </c>
       <c r="E11">
         <v>8</v>
       </c>
       <c r="F11" s="37" t="s">
-        <v>777</v>
+        <v>772</v>
       </c>
       <c r="H11">
         <v>8</v>
       </c>
       <c r="I11" s="37" t="s">
-        <v>778</v>
+        <v>773</v>
       </c>
       <c r="K11">
         <v>10</v>
@@ -9524,7 +9530,7 @@
         <v>10</v>
       </c>
       <c r="F12" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="H12">
         <v>10</v>
@@ -9580,25 +9586,25 @@
         <v>14</v>
       </c>
       <c r="L13" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="N13">
         <v>14</v>
       </c>
       <c r="O13" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="Q13">
         <v>14</v>
       </c>
       <c r="R13" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="T13">
         <v>14</v>
       </c>
       <c r="U13" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
     </row>
     <row r="14" spans="2:21" x14ac:dyDescent="0.25">
@@ -9612,13 +9618,13 @@
         <v>15</v>
       </c>
       <c r="F14" s="39" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="H14">
         <v>15</v>
       </c>
       <c r="I14" s="39" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="K14">
         <v>15</v>
@@ -9706,25 +9712,25 @@
         <v>20</v>
       </c>
       <c r="L16" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="N16">
         <v>20</v>
       </c>
       <c r="O16" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="Q16">
         <v>20</v>
       </c>
       <c r="R16" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="T16">
         <v>20</v>
       </c>
       <c r="U16" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
     </row>
     <row r="17" spans="9:21" x14ac:dyDescent="0.25">
@@ -9781,42 +9787,42 @@
     </row>
     <row r="22" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I22" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
     </row>
     <row r="23" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I23" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="24" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I24" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
     </row>
     <row r="25" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I25" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
     </row>
     <row r="26" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I26" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
     </row>
     <row r="27" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I27" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
     </row>
     <row r="28" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I28" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
     </row>
     <row r="29" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I29" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
     </row>
     <row r="36" spans="11:11" x14ac:dyDescent="0.25">
@@ -9907,7 +9913,7 @@
         <v>3</v>
       </c>
       <c r="I8" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="K8">
         <v>3</v>
@@ -9939,13 +9945,13 @@
         <v>5</v>
       </c>
       <c r="I9" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="K9">
         <v>5</v>
       </c>
       <c r="L9" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="N9">
         <v>5</v>
@@ -9971,13 +9977,13 @@
         <v>8</v>
       </c>
       <c r="I10" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="K10">
         <v>8</v>
       </c>
       <c r="L10" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="N10">
         <v>6</v>
@@ -10061,25 +10067,25 @@
         <v>14</v>
       </c>
       <c r="F13" s="39" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="H13">
         <v>14</v>
       </c>
       <c r="I13" t="s">
-        <v>795</v>
+        <v>790</v>
       </c>
       <c r="K13">
         <v>14</v>
       </c>
       <c r="L13" t="s">
-        <v>795</v>
+        <v>790</v>
       </c>
       <c r="N13">
         <v>14</v>
       </c>
       <c r="O13" t="s">
-        <v>796</v>
+        <v>791</v>
       </c>
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.25">
@@ -10111,7 +10117,7 @@
         <v>15</v>
       </c>
       <c r="O14" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.25">
@@ -10157,19 +10163,19 @@
         <v>20</v>
       </c>
       <c r="I16" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="K16">
         <v>20</v>
       </c>
       <c r="L16" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="N16">
         <v>21</v>
       </c>
       <c r="O16" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
     </row>
     <row r="17" spans="8:15" x14ac:dyDescent="0.25">
@@ -10214,27 +10220,27 @@
     </row>
     <row r="22" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I22" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="23" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I23" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
     </row>
     <row r="24" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I24" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
     </row>
     <row r="25" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I25" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="26" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I26" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
     </row>
   </sheetData>
@@ -10342,7 +10348,7 @@
         <v>4</v>
       </c>
       <c r="C9" t="s">
-        <v>779</v>
+        <v>774</v>
       </c>
       <c r="E9">
         <v>4</v>
@@ -10380,7 +10386,7 @@
         <v>4</v>
       </c>
       <c r="F10" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="H10">
         <v>8</v>
@@ -10392,7 +10398,7 @@
         <v>7</v>
       </c>
       <c r="L10" t="s">
-        <v>781</v>
+        <v>776</v>
       </c>
       <c r="N10">
         <v>5</v>
@@ -10444,7 +10450,7 @@
         <v>8</v>
       </c>
       <c r="F12" t="s">
-        <v>780</v>
+        <v>775</v>
       </c>
       <c r="H12">
         <v>12</v>
@@ -10456,7 +10462,7 @@
         <v>10</v>
       </c>
       <c r="L12" t="s">
-        <v>775</v>
+        <v>770</v>
       </c>
       <c r="N12">
         <v>10</v>
@@ -10502,7 +10508,7 @@
         <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="E14">
         <v>14</v>
@@ -10520,7 +10526,7 @@
         <v>15</v>
       </c>
       <c r="L14" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="N14">
         <v>17</v>
@@ -10546,7 +10552,7 @@
         <v>16</v>
       </c>
       <c r="I15" t="s">
-        <v>774</v>
+        <v>769</v>
       </c>
       <c r="K15">
         <v>16</v>
@@ -10584,7 +10590,7 @@
         <v>17</v>
       </c>
       <c r="L16" t="s">
-        <v>768</v>
+        <v>763</v>
       </c>
       <c r="N16">
         <v>21</v>
@@ -10630,7 +10636,7 @@
         <v>25</v>
       </c>
       <c r="O18" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
   </sheetData>
@@ -10779,7 +10785,7 @@
         <v>10</v>
       </c>
       <c r="F11" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="H11">
         <v>10</v>
@@ -10791,7 +10797,7 @@
         <v>7</v>
       </c>
       <c r="L11" t="s">
-        <v>785</v>
+        <v>780</v>
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
@@ -10825,13 +10831,13 @@
         <v>10</v>
       </c>
       <c r="C13" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="E13">
         <v>14</v>
       </c>
       <c r="F13" s="39" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="H13">
         <v>14</v>
@@ -10863,7 +10869,7 @@
         <v>15</v>
       </c>
       <c r="I14" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="K14">
         <v>16</v>
@@ -10889,13 +10895,13 @@
         <v>16</v>
       </c>
       <c r="I15" t="s">
-        <v>773</v>
+        <v>768</v>
       </c>
       <c r="K15">
         <v>20</v>
       </c>
       <c r="L15" t="s">
-        <v>771</v>
+        <v>766</v>
       </c>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
@@ -10935,7 +10941,7 @@
         <v>22</v>
       </c>
       <c r="L17" t="s">
-        <v>782</v>
+        <v>777</v>
       </c>
     </row>
     <row r="18" spans="8:12" x14ac:dyDescent="0.25">
@@ -10949,7 +10955,7 @@
         <v>25</v>
       </c>
       <c r="L18" t="s">
-        <v>772</v>
+        <v>767</v>
       </c>
     </row>
   </sheetData>
@@ -11172,7 +11178,7 @@
         <v>8</v>
       </c>
       <c r="U10" t="s">
-        <v>753</v>
+        <v>748</v>
       </c>
     </row>
     <row r="11" spans="2:21" x14ac:dyDescent="0.25">
@@ -11204,19 +11210,19 @@
         <v>9</v>
       </c>
       <c r="O11" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="Q11">
         <v>9</v>
       </c>
       <c r="R11" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="T11">
         <v>9</v>
       </c>
       <c r="U11" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="12" spans="2:21" x14ac:dyDescent="0.25">
@@ -11292,19 +11298,19 @@
         <v>14</v>
       </c>
       <c r="O13" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="Q13">
         <v>14</v>
       </c>
       <c r="R13" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="T13">
         <v>14</v>
       </c>
       <c r="U13" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
     </row>
     <row r="14" spans="2:21" x14ac:dyDescent="0.25">
@@ -11348,7 +11354,7 @@
         <v>15</v>
       </c>
       <c r="U14" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
     </row>
     <row r="15" spans="2:21" x14ac:dyDescent="0.25">
@@ -11380,19 +11386,19 @@
         <v>17</v>
       </c>
       <c r="O15" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="Q15">
         <v>17</v>
       </c>
       <c r="R15" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="T15">
         <v>17</v>
       </c>
       <c r="U15" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
     </row>
     <row r="16" spans="2:21" x14ac:dyDescent="0.25">
@@ -11424,7 +11430,7 @@
         <v>21</v>
       </c>
       <c r="O16" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="Q16">
         <v>21</v>
@@ -11444,19 +11450,19 @@
         <v>22</v>
       </c>
       <c r="O17" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="Q17">
         <v>22</v>
       </c>
       <c r="R17" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="T17">
         <v>22</v>
       </c>
       <c r="U17" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
     </row>
     <row r="18" spans="9:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
retoques armas, algun ataque que faltaba y primeras lineas
</commit_message>
<xml_diff>
--- a/arquetiposZ.xlsx
+++ b/arquetiposZ.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sergius\Desktop\Proyectos\hyperbole\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{850299BE-B260-4CE5-906E-5FC3ABA798CB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBAEA953-57D6-479A-9F45-4FD3DAF60843}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="644" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="644" firstSheet="1" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RESUMEN" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1147" uniqueCount="814">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1146" uniqueCount="813">
   <si>
     <t>daños:</t>
   </si>
@@ -1946,9 +1946,6 @@
   </si>
   <si>
     <t>[hacha 2]</t>
-  </si>
-  <si>
-    <t>[escudo 1]</t>
   </si>
   <si>
     <t>[escudo 2]</t>
@@ -4752,7 +4749,7 @@
         <v>15</v>
       </c>
       <c r="G12" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="J12">
         <v>10</v>
@@ -4834,7 +4831,7 @@
         <v>24</v>
       </c>
       <c r="K17" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
     </row>
     <row r="18" spans="8:11" x14ac:dyDescent="0.25">
@@ -4877,7 +4874,7 @@
     </row>
     <row r="30" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H30" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
     </row>
     <row r="31" spans="8:11" x14ac:dyDescent="0.25">
@@ -4887,7 +4884,7 @@
     </row>
     <row r="32" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H32" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
     </row>
     <row r="33" spans="8:8" x14ac:dyDescent="0.25">
@@ -4949,7 +4946,7 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="H7">
         <v>1</v>
@@ -4967,7 +4964,7 @@
         <v>1</v>
       </c>
       <c r="O7" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="Q7">
         <v>1</v>
@@ -5143,13 +5140,13 @@
         <v>9</v>
       </c>
       <c r="O11" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="Q11">
         <v>10</v>
       </c>
       <c r="R11" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="T11">
         <v>6</v>
@@ -5175,7 +5172,7 @@
         <v>10</v>
       </c>
       <c r="I12" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="K12">
         <v>12</v>
@@ -5187,7 +5184,7 @@
         <v>10</v>
       </c>
       <c r="O12" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="Q12">
         <v>12</v>
@@ -5219,7 +5216,7 @@
         <v>10</v>
       </c>
       <c r="I13" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="K13">
         <v>14</v>
@@ -5231,7 +5228,7 @@
         <v>11</v>
       </c>
       <c r="O13" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="Q13">
         <v>14</v>
@@ -5243,7 +5240,7 @@
         <v>12</v>
       </c>
       <c r="U13" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="14" spans="2:22" x14ac:dyDescent="0.25">
@@ -5251,7 +5248,7 @@
         <v>13</v>
       </c>
       <c r="C14" s="39" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="E14">
         <v>16</v>
@@ -5269,13 +5266,13 @@
         <v>15</v>
       </c>
       <c r="L14" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="N14">
         <v>12</v>
       </c>
       <c r="O14" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="Q14">
         <v>15</v>
@@ -5301,7 +5298,7 @@
         <v>18</v>
       </c>
       <c r="F15" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="H15">
         <v>16</v>
@@ -5313,7 +5310,7 @@
         <v>16</v>
       </c>
       <c r="L15" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="N15">
         <v>13</v>
@@ -5351,13 +5348,13 @@
         <v>20</v>
       </c>
       <c r="L16" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="N16">
         <v>15</v>
       </c>
       <c r="O16" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="Q16">
         <v>20</v>
@@ -5372,7 +5369,7 @@
         <v>493</v>
       </c>
       <c r="V16" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
     </row>
     <row r="17" spans="9:21" x14ac:dyDescent="0.25">
@@ -5386,7 +5383,7 @@
         <v>20</v>
       </c>
       <c r="O17" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="Q17">
         <v>23</v>
@@ -5398,7 +5395,7 @@
         <v>23</v>
       </c>
       <c r="U17" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
     </row>
     <row r="18" spans="9:21" x14ac:dyDescent="0.25">
@@ -5424,7 +5421,7 @@
         <v>25</v>
       </c>
       <c r="U18" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
     </row>
     <row r="21" spans="9:21" x14ac:dyDescent="0.25">
@@ -5489,7 +5486,7 @@
     </row>
     <row r="33" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I33" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
     </row>
     <row r="34" spans="9:9" x14ac:dyDescent="0.25">
@@ -5509,7 +5506,7 @@
     </row>
     <row r="37" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I37" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
   </sheetData>
@@ -5574,7 +5571,7 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="H7">
         <v>1</v>
@@ -5586,7 +5583,7 @@
         <v>1</v>
       </c>
       <c r="L7" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="N7">
         <v>1</v>
@@ -5598,13 +5595,13 @@
         <v>1</v>
       </c>
       <c r="R7" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="T7">
         <v>1</v>
       </c>
       <c r="U7" s="39" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="8" spans="2:21" x14ac:dyDescent="0.25">
@@ -5630,13 +5627,13 @@
         <v>1</v>
       </c>
       <c r="L8" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="N8">
         <v>1</v>
       </c>
       <c r="O8" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="Q8">
         <v>3</v>
@@ -5648,7 +5645,7 @@
         <v>1</v>
       </c>
       <c r="U8" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
     </row>
     <row r="9" spans="2:21" x14ac:dyDescent="0.25">
@@ -5656,7 +5653,7 @@
         <v>4</v>
       </c>
       <c r="C9" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -5686,13 +5683,13 @@
         <v>7</v>
       </c>
       <c r="R9" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="T9">
         <v>1</v>
       </c>
       <c r="U9" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
     </row>
     <row r="10" spans="2:21" x14ac:dyDescent="0.25">
@@ -5700,31 +5697,31 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="E10">
         <v>5</v>
       </c>
       <c r="F10" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="H10">
         <v>7</v>
       </c>
       <c r="I10" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="K10">
         <v>5</v>
       </c>
       <c r="L10" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="N10">
         <v>5</v>
       </c>
       <c r="O10" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="Q10">
         <v>10</v>
@@ -5744,13 +5741,13 @@
         <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E11">
         <v>10</v>
       </c>
       <c r="F11" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="H11">
         <v>10</v>
@@ -5774,7 +5771,7 @@
         <v>11</v>
       </c>
       <c r="R11" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="T11">
         <v>7</v>
@@ -5794,19 +5791,19 @@
         <v>12</v>
       </c>
       <c r="F12" s="39" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="H12">
         <v>15</v>
       </c>
       <c r="I12" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="K12">
         <v>11</v>
       </c>
       <c r="L12" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="N12">
         <v>12</v>
@@ -5818,7 +5815,7 @@
         <v>12</v>
       </c>
       <c r="R12" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="T12">
         <v>10</v>
@@ -5850,7 +5847,7 @@
         <v>14</v>
       </c>
       <c r="L13" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="N13">
         <v>12</v>
@@ -5862,7 +5859,7 @@
         <v>12</v>
       </c>
       <c r="R13" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="T13">
         <v>11</v>
@@ -5894,7 +5891,7 @@
         <v>16</v>
       </c>
       <c r="L14" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="N14">
         <v>15</v>
@@ -5932,13 +5929,13 @@
         <v>20</v>
       </c>
       <c r="I15" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="K15">
         <v>18</v>
       </c>
       <c r="L15" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="N15">
         <v>18</v>
@@ -5956,7 +5953,7 @@
         <v>15</v>
       </c>
       <c r="U15" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
     </row>
     <row r="16" spans="2:21" x14ac:dyDescent="0.25">
@@ -5964,25 +5961,25 @@
         <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="E16">
         <v>20</v>
       </c>
       <c r="F16" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="H16">
         <v>20</v>
       </c>
       <c r="I16" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="K16">
         <v>21</v>
       </c>
       <c r="L16" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="N16">
         <v>20</v>
@@ -6000,7 +5997,7 @@
         <v>19</v>
       </c>
       <c r="U16" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
     </row>
     <row r="17" spans="10:21" x14ac:dyDescent="0.25">
@@ -6008,7 +6005,7 @@
         <v>22</v>
       </c>
       <c r="L17" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="N17">
         <v>20</v>
@@ -6034,7 +6031,7 @@
         <v>25</v>
       </c>
       <c r="L18" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="N18">
         <v>25</v>
@@ -6072,22 +6069,22 @@
     </row>
     <row r="25" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J25" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
     </row>
     <row r="26" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J26" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
     </row>
     <row r="27" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J27" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
     </row>
     <row r="28" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J28" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
     </row>
     <row r="29" spans="10:21" x14ac:dyDescent="0.25">
@@ -6102,12 +6099,12 @@
     </row>
     <row r="31" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J31" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
     </row>
     <row r="32" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J32" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
     </row>
     <row r="33" spans="10:10" x14ac:dyDescent="0.25">
@@ -6117,12 +6114,12 @@
     </row>
     <row r="34" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J34" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
     <row r="35" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J35" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
     </row>
   </sheetData>
@@ -6163,7 +6160,7 @@
         <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>782</v>
+        <v>635</v>
       </c>
       <c r="J7">
         <v>1</v>
@@ -6183,7 +6180,7 @@
         <v>1</v>
       </c>
       <c r="G8" t="s">
-        <v>348</v>
+        <v>634</v>
       </c>
       <c r="J8">
         <v>5</v>
@@ -6197,13 +6194,13 @@
         <v>5</v>
       </c>
       <c r="C9" t="s">
-        <v>633</v>
+        <v>480</v>
       </c>
       <c r="F9">
         <v>3</v>
       </c>
       <c r="G9" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="J9">
         <v>7</v>
@@ -6217,7 +6214,7 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>346</v>
+        <v>633</v>
       </c>
       <c r="F10">
         <v>6</v>
@@ -6229,7 +6226,7 @@
         <v>8</v>
       </c>
       <c r="K10" t="s">
-        <v>355</v>
+        <v>485</v>
       </c>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.25">
@@ -6237,7 +6234,7 @@
         <v>7</v>
       </c>
       <c r="C11" t="s">
-        <v>626</v>
+        <v>285</v>
       </c>
       <c r="F11">
         <v>7</v>
@@ -6249,7 +6246,7 @@
         <v>11</v>
       </c>
       <c r="K11" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.25">
@@ -6257,19 +6254,19 @@
         <v>8</v>
       </c>
       <c r="C12" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="F12">
         <v>8</v>
       </c>
       <c r="G12" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="J12">
         <v>11</v>
       </c>
       <c r="K12" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.25">
@@ -6277,19 +6274,19 @@
         <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>634</v>
+        <v>627</v>
       </c>
       <c r="F13">
         <v>12</v>
       </c>
       <c r="G13" t="s">
-        <v>353</v>
+        <v>641</v>
       </c>
       <c r="J13">
         <v>13</v>
       </c>
       <c r="K13" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
     </row>
     <row r="14" spans="2:11" x14ac:dyDescent="0.25">
@@ -6297,7 +6294,7 @@
         <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>347</v>
+        <v>479</v>
       </c>
       <c r="F14">
         <v>16</v>
@@ -6309,12 +6306,12 @@
         <v>15</v>
       </c>
       <c r="K14" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B15">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C15" t="s">
         <v>635</v>
@@ -6323,22 +6320,16 @@
         <v>19</v>
       </c>
       <c r="G15" t="s">
-        <v>643</v>
+        <v>782</v>
       </c>
       <c r="J15">
         <v>18</v>
       </c>
       <c r="K15" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B16">
-        <v>15</v>
-      </c>
-      <c r="C16" t="s">
-        <v>636</v>
-      </c>
       <c r="F16">
         <v>20</v>
       </c>
@@ -6385,7 +6376,7 @@
     </row>
     <row r="30" spans="10:11" x14ac:dyDescent="0.25">
       <c r="K30" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
     </row>
   </sheetData>
@@ -6474,7 +6465,7 @@
         <v>1</v>
       </c>
       <c r="V7" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
     </row>
     <row r="8" spans="2:22" x14ac:dyDescent="0.25">
@@ -6512,13 +6503,13 @@
         <v>3</v>
       </c>
       <c r="R8" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="U8">
         <v>2</v>
       </c>
       <c r="V8" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
     <row r="9" spans="2:22" x14ac:dyDescent="0.25">
@@ -6526,7 +6517,7 @@
         <v>5</v>
       </c>
       <c r="C9" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="E9">
         <v>4</v>
@@ -6562,7 +6553,7 @@
         <v>2</v>
       </c>
       <c r="V9" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
     </row>
     <row r="10" spans="2:22" x14ac:dyDescent="0.25">
@@ -6606,7 +6597,7 @@
         <v>6</v>
       </c>
       <c r="V10" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
     </row>
     <row r="11" spans="2:22" x14ac:dyDescent="0.25">
@@ -6650,7 +6641,7 @@
         <v>7</v>
       </c>
       <c r="V11" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
     </row>
     <row r="12" spans="2:22" x14ac:dyDescent="0.25">
@@ -6658,7 +6649,7 @@
         <v>10</v>
       </c>
       <c r="C12" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="E12">
         <v>11</v>
@@ -6694,7 +6685,7 @@
         <v>8</v>
       </c>
       <c r="V12" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="13" spans="2:22" x14ac:dyDescent="0.25">
@@ -6714,7 +6705,7 @@
         <v>9</v>
       </c>
       <c r="I13" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="K13">
         <v>14</v>
@@ -6732,13 +6723,13 @@
         <v>14</v>
       </c>
       <c r="R13" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="U13">
         <v>9</v>
       </c>
       <c r="V13" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
     </row>
     <row r="14" spans="2:22" x14ac:dyDescent="0.25">
@@ -6746,7 +6737,7 @@
         <v>14</v>
       </c>
       <c r="C14" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="E14">
         <v>16</v>
@@ -6782,7 +6773,7 @@
         <v>14</v>
       </c>
       <c r="V14" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
     </row>
     <row r="15" spans="2:22" x14ac:dyDescent="0.25">
@@ -6796,13 +6787,13 @@
         <v>18</v>
       </c>
       <c r="F15" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="H15">
         <v>16</v>
       </c>
       <c r="I15" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="K15">
         <v>20</v>
@@ -6820,7 +6811,7 @@
         <v>16</v>
       </c>
       <c r="R15" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="U15">
         <v>17</v>
@@ -6864,7 +6855,7 @@
         <v>20</v>
       </c>
       <c r="V16" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="17" spans="11:22" x14ac:dyDescent="0.25">
@@ -6890,7 +6881,7 @@
         <v>24</v>
       </c>
       <c r="V17" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
     </row>
     <row r="18" spans="11:22" x14ac:dyDescent="0.25">
@@ -6904,7 +6895,7 @@
         <v>25</v>
       </c>
       <c r="O18" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="Q18">
         <v>25</v>
@@ -6916,22 +6907,22 @@
         <v>25</v>
       </c>
       <c r="V18" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
     </row>
     <row r="22" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L22" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
     </row>
     <row r="23" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L23" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
     </row>
     <row r="24" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L24" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
     </row>
     <row r="25" spans="11:22" x14ac:dyDescent="0.25">
@@ -6951,7 +6942,7 @@
     </row>
     <row r="28" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L28" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
     </row>
     <row r="29" spans="11:22" x14ac:dyDescent="0.25">
@@ -6961,12 +6952,12 @@
     </row>
     <row r="30" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L30" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
     </row>
     <row r="33" spans="13:13" x14ac:dyDescent="0.25">
       <c r="M33" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
     </row>
   </sheetData>
@@ -7040,13 +7031,13 @@
         <v>2</v>
       </c>
       <c r="F8" s="39" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="H8">
         <v>2</v>
       </c>
       <c r="I8" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="K8">
         <v>1</v>
@@ -7060,13 +7051,13 @@
         <v>2</v>
       </c>
       <c r="C9" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="E9">
         <v>3</v>
       </c>
       <c r="F9" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="H9">
         <v>5</v>
@@ -7078,7 +7069,7 @@
         <v>3</v>
       </c>
       <c r="L9" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
@@ -7098,13 +7089,13 @@
         <v>8</v>
       </c>
       <c r="I10" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="K10">
         <v>4</v>
       </c>
       <c r="L10" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
@@ -7112,13 +7103,13 @@
         <v>4</v>
       </c>
       <c r="C11" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="E11">
         <v>8</v>
       </c>
       <c r="F11" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="H11">
         <v>10</v>
@@ -7130,7 +7121,7 @@
         <v>5</v>
       </c>
       <c r="L11" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
@@ -7150,7 +7141,7 @@
         <v>11</v>
       </c>
       <c r="I12" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="K12">
         <v>8</v>
@@ -7164,19 +7155,19 @@
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="E13">
         <v>12</v>
       </c>
       <c r="F13" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="H13">
         <v>14</v>
       </c>
       <c r="I13" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="K13">
         <v>10</v>
@@ -7190,7 +7181,7 @@
         <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="E14">
         <v>13</v>
@@ -7208,7 +7199,7 @@
         <v>15</v>
       </c>
       <c r="L14" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.25">
@@ -7222,19 +7213,19 @@
         <v>16</v>
       </c>
       <c r="F15" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="H15">
         <v>17</v>
       </c>
       <c r="I15" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="K15">
         <v>18</v>
       </c>
       <c r="L15" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
@@ -7242,7 +7233,7 @@
         <v>15</v>
       </c>
       <c r="C16" s="39" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="E16">
         <v>17</v>
@@ -7260,7 +7251,7 @@
         <v>20</v>
       </c>
       <c r="L16" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
     </row>
     <row r="17" spans="5:12" x14ac:dyDescent="0.25">
@@ -7268,7 +7259,7 @@
         <v>20</v>
       </c>
       <c r="F17" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="H17">
         <v>23</v>
@@ -7280,7 +7271,7 @@
         <v>21</v>
       </c>
       <c r="L17" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
     </row>
     <row r="18" spans="5:12" x14ac:dyDescent="0.25">
@@ -7309,7 +7300,7 @@
     </row>
     <row r="24" spans="5:12" x14ac:dyDescent="0.25">
       <c r="I24" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
     </row>
     <row r="25" spans="5:12" x14ac:dyDescent="0.25">
@@ -8690,10 +8681,10 @@
     <row r="7" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B8" s="35" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="C8" s="36" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="H8" t="s">
         <v>12</v>
@@ -8873,7 +8864,7 @@
         <v>248</v>
       </c>
       <c r="M17" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.25">
@@ -9209,7 +9200,7 @@
   <sheetData>
     <row r="5" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
     </row>
     <row r="6" spans="2:2" x14ac:dyDescent="0.25">
@@ -9480,19 +9471,19 @@
         <v>8</v>
       </c>
       <c r="C11" s="37" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="E11">
         <v>8</v>
       </c>
       <c r="F11" s="37" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="H11">
         <v>8</v>
       </c>
       <c r="I11" s="37" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="K11">
         <v>10</v>
@@ -9530,7 +9521,7 @@
         <v>10</v>
       </c>
       <c r="F12" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="H12">
         <v>10</v>
@@ -9586,25 +9577,25 @@
         <v>14</v>
       </c>
       <c r="L13" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="N13">
         <v>14</v>
       </c>
       <c r="O13" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="Q13">
         <v>14</v>
       </c>
       <c r="R13" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="T13">
         <v>14</v>
       </c>
       <c r="U13" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
     </row>
     <row r="14" spans="2:21" x14ac:dyDescent="0.25">
@@ -9618,13 +9609,13 @@
         <v>15</v>
       </c>
       <c r="F14" s="39" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="H14">
         <v>15</v>
       </c>
       <c r="I14" s="39" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="K14">
         <v>15</v>
@@ -9977,13 +9968,13 @@
         <v>8</v>
       </c>
       <c r="I10" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="K10">
         <v>8</v>
       </c>
       <c r="L10" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="N10">
         <v>6</v>
@@ -10067,25 +10058,25 @@
         <v>14</v>
       </c>
       <c r="F13" s="39" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="H13">
         <v>14</v>
       </c>
       <c r="I13" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="K13">
         <v>14</v>
       </c>
       <c r="L13" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="N13">
         <v>14</v>
       </c>
       <c r="O13" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.25">
@@ -10117,7 +10108,7 @@
         <v>15</v>
       </c>
       <c r="O14" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.25">
@@ -10220,22 +10211,22 @@
     </row>
     <row r="22" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I22" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="23" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I23" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="24" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I24" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
     </row>
     <row r="25" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I25" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="26" spans="8:15" x14ac:dyDescent="0.25">
@@ -10348,7 +10339,7 @@
         <v>4</v>
       </c>
       <c r="C9" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="E9">
         <v>4</v>
@@ -10386,7 +10377,7 @@
         <v>4</v>
       </c>
       <c r="F10" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="H10">
         <v>8</v>
@@ -10398,7 +10389,7 @@
         <v>7</v>
       </c>
       <c r="L10" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="N10">
         <v>5</v>
@@ -10450,7 +10441,7 @@
         <v>8</v>
       </c>
       <c r="F12" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="H12">
         <v>12</v>
@@ -10462,7 +10453,7 @@
         <v>10</v>
       </c>
       <c r="L12" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="N12">
         <v>10</v>
@@ -10508,7 +10499,7 @@
         <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="E14">
         <v>14</v>
@@ -10526,7 +10517,7 @@
         <v>15</v>
       </c>
       <c r="L14" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="N14">
         <v>17</v>
@@ -10552,7 +10543,7 @@
         <v>16</v>
       </c>
       <c r="I15" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="K15">
         <v>16</v>
@@ -10590,7 +10581,7 @@
         <v>17</v>
       </c>
       <c r="L16" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="N16">
         <v>21</v>
@@ -10636,7 +10627,7 @@
         <v>25</v>
       </c>
       <c r="O18" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
   </sheetData>
@@ -10785,7 +10776,7 @@
         <v>10</v>
       </c>
       <c r="F11" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="H11">
         <v>10</v>
@@ -10797,7 +10788,7 @@
         <v>7</v>
       </c>
       <c r="L11" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
@@ -10831,13 +10822,13 @@
         <v>10</v>
       </c>
       <c r="C13" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="E13">
         <v>14</v>
       </c>
       <c r="F13" s="39" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="H13">
         <v>14</v>
@@ -10869,7 +10860,7 @@
         <v>15</v>
       </c>
       <c r="I14" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="K14">
         <v>16</v>
@@ -10895,13 +10886,13 @@
         <v>16</v>
       </c>
       <c r="I15" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="K15">
         <v>20</v>
       </c>
       <c r="L15" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
@@ -10941,7 +10932,7 @@
         <v>22</v>
       </c>
       <c r="L17" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
     </row>
     <row r="18" spans="8:12" x14ac:dyDescent="0.25">
@@ -10955,7 +10946,7 @@
         <v>25</v>
       </c>
       <c r="L18" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
     </row>
   </sheetData>
@@ -11178,7 +11169,7 @@
         <v>8</v>
       </c>
       <c r="U10" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
     </row>
     <row r="11" spans="2:21" x14ac:dyDescent="0.25">
@@ -11210,19 +11201,19 @@
         <v>9</v>
       </c>
       <c r="O11" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="Q11">
         <v>9</v>
       </c>
       <c r="R11" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="T11">
         <v>9</v>
       </c>
       <c r="U11" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
     </row>
     <row r="12" spans="2:21" x14ac:dyDescent="0.25">
@@ -11298,19 +11289,19 @@
         <v>14</v>
       </c>
       <c r="O13" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="Q13">
         <v>14</v>
       </c>
       <c r="R13" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="T13">
         <v>14</v>
       </c>
       <c r="U13" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
     </row>
     <row r="14" spans="2:21" x14ac:dyDescent="0.25">
@@ -11354,7 +11345,7 @@
         <v>15</v>
       </c>
       <c r="U14" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
     </row>
     <row r="15" spans="2:21" x14ac:dyDescent="0.25">
@@ -11386,19 +11377,19 @@
         <v>17</v>
       </c>
       <c r="O15" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="Q15">
         <v>17</v>
       </c>
       <c r="R15" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="T15">
         <v>17</v>
       </c>
       <c r="U15" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
     </row>
     <row r="16" spans="2:21" x14ac:dyDescent="0.25">
@@ -11430,7 +11421,7 @@
         <v>21</v>
       </c>
       <c r="O16" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="Q16">
         <v>21</v>
@@ -11450,19 +11441,19 @@
         <v>22</v>
       </c>
       <c r="O17" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="Q17">
         <v>22</v>
       </c>
       <c r="R17" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="T17">
         <v>22</v>
       </c>
       <c r="U17" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
     </row>
     <row r="18" spans="9:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
todas las lineas terminadas
</commit_message>
<xml_diff>
--- a/arquetiposZ.xlsx
+++ b/arquetiposZ.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sergius\Desktop\Proyectos\hyperbole\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBAEA953-57D6-479A-9F45-4FD3DAF60843}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ACE246F-6AF6-4693-8851-3E79DEA21016}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="644" firstSheet="1" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="644" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RESUMEN" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1146" uniqueCount="813">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1145" uniqueCount="813">
   <si>
     <t>daños:</t>
   </si>
@@ -1531,9 +1531,6 @@
     <t>masukunda</t>
   </si>
   <si>
-    <t>agydyne</t>
-  </si>
-  <si>
     <t>magic counter</t>
   </si>
   <si>
@@ -2483,6 +2480,9 @@
   </si>
   <si>
     <t>resistir paralisis/cong</t>
+  </si>
+  <si>
+    <t>romper res fisicos</t>
   </si>
 </sst>
 </file>
@@ -4222,7 +4222,7 @@
         <v>43</v>
       </c>
       <c r="L26" s="5" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="M26" s="5"/>
       <c r="N26" s="5"/>
@@ -4367,7 +4367,7 @@
         <v>54</v>
       </c>
       <c r="L31" s="5" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="M31" s="5"/>
       <c r="N31" s="5"/>
@@ -4394,7 +4394,7 @@
         <v>55</v>
       </c>
       <c r="L32" s="5" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="M32" s="5"/>
       <c r="N32" s="5"/>
@@ -4417,13 +4417,13 @@
       <c r="H33" s="5"/>
       <c r="I33" s="1"/>
       <c r="J33" s="5" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="K33" s="5" t="s">
         <v>66</v>
       </c>
       <c r="L33" s="5" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="M33" s="5"/>
       <c r="N33" s="5"/>
@@ -4454,7 +4454,7 @@
         <v>58</v>
       </c>
       <c r="L34" s="5" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="M34" s="5"/>
       <c r="N34" s="5"/>
@@ -4740,7 +4740,7 @@
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B12">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C12" t="s">
         <v>360</v>
@@ -4749,7 +4749,7 @@
         <v>15</v>
       </c>
       <c r="G12" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="J12">
         <v>10</v>
@@ -4831,7 +4831,7 @@
         <v>24</v>
       </c>
       <c r="K17" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
     </row>
     <row r="18" spans="8:11" x14ac:dyDescent="0.25">
@@ -4874,7 +4874,7 @@
     </row>
     <row r="30" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H30" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="31" spans="8:11" x14ac:dyDescent="0.25">
@@ -4884,7 +4884,7 @@
     </row>
     <row r="32" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H32" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="33" spans="8:8" x14ac:dyDescent="0.25">
@@ -4946,31 +4946,31 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="H7">
         <v>1</v>
       </c>
       <c r="I7" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="K7">
         <v>1</v>
       </c>
       <c r="L7" t="s">
+        <v>637</v>
+      </c>
+      <c r="N7">
+        <v>1</v>
+      </c>
+      <c r="O7" t="s">
         <v>464</v>
       </c>
-      <c r="N7">
-        <v>1</v>
-      </c>
-      <c r="O7" t="s">
-        <v>638</v>
-      </c>
       <c r="Q7">
         <v>1</v>
       </c>
       <c r="R7" t="s">
-        <v>485</v>
+        <v>497</v>
       </c>
       <c r="T7">
         <v>1</v>
@@ -5058,7 +5058,7 @@
         <v>6</v>
       </c>
       <c r="R9" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="T9">
         <v>3</v>
@@ -5102,7 +5102,7 @@
         <v>8</v>
       </c>
       <c r="R10" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
       <c r="T10">
         <v>3</v>
@@ -5140,13 +5140,13 @@
         <v>9</v>
       </c>
       <c r="O11" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="Q11">
         <v>10</v>
       </c>
       <c r="R11" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="T11">
         <v>6</v>
@@ -5172,7 +5172,7 @@
         <v>10</v>
       </c>
       <c r="I12" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="K12">
         <v>12</v>
@@ -5184,13 +5184,13 @@
         <v>10</v>
       </c>
       <c r="O12" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="Q12">
         <v>12</v>
       </c>
       <c r="R12" t="s">
-        <v>506</v>
+        <v>488</v>
       </c>
       <c r="T12">
         <v>9</v>
@@ -5216,7 +5216,7 @@
         <v>10</v>
       </c>
       <c r="I13" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="K13">
         <v>14</v>
@@ -5228,19 +5228,19 @@
         <v>11</v>
       </c>
       <c r="O13" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="Q13">
         <v>14</v>
       </c>
       <c r="R13" t="s">
-        <v>488</v>
+        <v>495</v>
       </c>
       <c r="T13">
         <v>12</v>
       </c>
       <c r="U13" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="14" spans="2:22" x14ac:dyDescent="0.25">
@@ -5248,7 +5248,7 @@
         <v>13</v>
       </c>
       <c r="C14" s="39" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="E14">
         <v>16</v>
@@ -5266,19 +5266,19 @@
         <v>15</v>
       </c>
       <c r="L14" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="N14">
         <v>12</v>
       </c>
       <c r="O14" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="Q14">
         <v>15</v>
       </c>
       <c r="R14" t="s">
-        <v>495</v>
+        <v>81</v>
       </c>
       <c r="T14">
         <v>15</v>
@@ -5298,7 +5298,7 @@
         <v>18</v>
       </c>
       <c r="F15" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="H15">
         <v>16</v>
@@ -5310,7 +5310,7 @@
         <v>16</v>
       </c>
       <c r="L15" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="N15">
         <v>13</v>
@@ -5322,13 +5322,13 @@
         <v>16</v>
       </c>
       <c r="R15" t="s">
-        <v>496</v>
+        <v>506</v>
       </c>
       <c r="T15">
         <v>17</v>
       </c>
       <c r="U15" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="16" spans="2:22" x14ac:dyDescent="0.25">
@@ -5342,25 +5342,25 @@
         <v>20</v>
       </c>
       <c r="I16" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="K16">
         <v>20</v>
       </c>
       <c r="L16" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="N16">
         <v>15</v>
       </c>
       <c r="O16" t="s">
-        <v>728</v>
+        <v>812</v>
       </c>
       <c r="Q16">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="R16" t="s">
-        <v>507</v>
+        <v>727</v>
       </c>
       <c r="T16">
         <v>19</v>
@@ -5369,7 +5369,7 @@
         <v>493</v>
       </c>
       <c r="V16" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
     </row>
     <row r="17" spans="9:21" x14ac:dyDescent="0.25">
@@ -5383,19 +5383,19 @@
         <v>20</v>
       </c>
       <c r="O17" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="Q17">
         <v>23</v>
       </c>
       <c r="R17" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="T17">
         <v>23</v>
       </c>
       <c r="U17" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
     </row>
     <row r="18" spans="9:21" x14ac:dyDescent="0.25">
@@ -5415,13 +5415,13 @@
         <v>25</v>
       </c>
       <c r="R18" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="T18">
         <v>25</v>
       </c>
       <c r="U18" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
     </row>
     <row r="21" spans="9:21" x14ac:dyDescent="0.25">
@@ -5486,12 +5486,12 @@
     </row>
     <row r="33" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I33" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
     </row>
     <row r="34" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I34" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="35" spans="9:9" x14ac:dyDescent="0.25">
@@ -5501,12 +5501,12 @@
     </row>
     <row r="36" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I36" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
     </row>
     <row r="37" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I37" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
     </row>
   </sheetData>
@@ -5571,7 +5571,7 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="H7">
         <v>1</v>
@@ -5583,7 +5583,7 @@
         <v>1</v>
       </c>
       <c r="L7" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="N7">
         <v>1</v>
@@ -5595,13 +5595,13 @@
         <v>1</v>
       </c>
       <c r="R7" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="T7">
         <v>1</v>
       </c>
       <c r="U7" s="39" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
     </row>
     <row r="8" spans="2:21" x14ac:dyDescent="0.25">
@@ -5627,13 +5627,13 @@
         <v>1</v>
       </c>
       <c r="L8" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="N8">
         <v>1</v>
       </c>
       <c r="O8" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="Q8">
         <v>3</v>
@@ -5645,7 +5645,7 @@
         <v>1</v>
       </c>
       <c r="U8" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
     </row>
     <row r="9" spans="2:21" x14ac:dyDescent="0.25">
@@ -5653,7 +5653,7 @@
         <v>4</v>
       </c>
       <c r="C9" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -5671,7 +5671,7 @@
         <v>1</v>
       </c>
       <c r="L9" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="N9">
         <v>1</v>
@@ -5683,13 +5683,13 @@
         <v>7</v>
       </c>
       <c r="R9" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="T9">
         <v>1</v>
       </c>
       <c r="U9" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
     </row>
     <row r="10" spans="2:21" x14ac:dyDescent="0.25">
@@ -5697,31 +5697,31 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="E10">
         <v>5</v>
       </c>
       <c r="F10" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="H10">
         <v>7</v>
       </c>
       <c r="I10" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="K10">
         <v>5</v>
       </c>
       <c r="L10" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="N10">
         <v>5</v>
       </c>
       <c r="O10" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="Q10">
         <v>10</v>
@@ -5741,13 +5741,13 @@
         <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="E11">
         <v>10</v>
       </c>
       <c r="F11" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="H11">
         <v>10</v>
@@ -5759,7 +5759,7 @@
         <v>9</v>
       </c>
       <c r="L11" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="N11">
         <v>10</v>
@@ -5771,7 +5771,7 @@
         <v>11</v>
       </c>
       <c r="R11" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="T11">
         <v>7</v>
@@ -5791,19 +5791,19 @@
         <v>12</v>
       </c>
       <c r="F12" s="39" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="H12">
         <v>15</v>
       </c>
       <c r="I12" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="K12">
         <v>11</v>
       </c>
       <c r="L12" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="N12">
         <v>12</v>
@@ -5815,7 +5815,7 @@
         <v>12</v>
       </c>
       <c r="R12" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="T12">
         <v>10</v>
@@ -5835,7 +5835,7 @@
         <v>17</v>
       </c>
       <c r="F13" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="H13">
         <v>15</v>
@@ -5847,7 +5847,7 @@
         <v>14</v>
       </c>
       <c r="L13" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="N13">
         <v>12</v>
@@ -5859,7 +5859,7 @@
         <v>12</v>
       </c>
       <c r="R13" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="T13">
         <v>11</v>
@@ -5873,7 +5873,7 @@
         <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="E14">
         <v>18</v>
@@ -5891,13 +5891,13 @@
         <v>16</v>
       </c>
       <c r="L14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="N14">
         <v>15</v>
       </c>
       <c r="O14" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="Q14">
         <v>15</v>
@@ -5917,25 +5917,25 @@
         <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="E15">
         <v>19</v>
       </c>
       <c r="F15" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="H15">
         <v>20</v>
       </c>
       <c r="I15" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="K15">
         <v>18</v>
       </c>
       <c r="L15" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="N15">
         <v>18</v>
@@ -5953,7 +5953,7 @@
         <v>15</v>
       </c>
       <c r="U15" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
     </row>
     <row r="16" spans="2:21" x14ac:dyDescent="0.25">
@@ -5961,25 +5961,25 @@
         <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="E16">
         <v>20</v>
       </c>
       <c r="F16" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="H16">
         <v>20</v>
       </c>
       <c r="I16" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="K16">
         <v>21</v>
       </c>
       <c r="L16" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="N16">
         <v>20</v>
@@ -5997,7 +5997,7 @@
         <v>19</v>
       </c>
       <c r="U16" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
     </row>
     <row r="17" spans="10:21" x14ac:dyDescent="0.25">
@@ -6005,7 +6005,7 @@
         <v>22</v>
       </c>
       <c r="L17" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="N17">
         <v>20</v>
@@ -6031,7 +6031,7 @@
         <v>25</v>
       </c>
       <c r="L18" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="N18">
         <v>25</v>
@@ -6069,22 +6069,22 @@
     </row>
     <row r="25" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J25" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
     </row>
     <row r="26" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J26" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
     </row>
     <row r="27" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J27" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
     </row>
     <row r="28" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J28" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
     </row>
     <row r="29" spans="10:21" x14ac:dyDescent="0.25">
@@ -6099,27 +6099,27 @@
     </row>
     <row r="31" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J31" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
     </row>
     <row r="32" spans="10:21" x14ac:dyDescent="0.25">
       <c r="J32" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
     </row>
     <row r="33" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J33" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
     </row>
     <row r="34" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J34" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
     </row>
     <row r="35" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J35" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
   </sheetData>
@@ -6154,19 +6154,19 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="J7">
         <v>1</v>
       </c>
       <c r="K7" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.25">
@@ -6174,13 +6174,13 @@
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="F8">
         <v>1</v>
       </c>
       <c r="G8" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="J8">
         <v>5</v>
@@ -6200,13 +6200,13 @@
         <v>3</v>
       </c>
       <c r="G9" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="J9">
         <v>7</v>
       </c>
       <c r="K9" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.25">
@@ -6214,13 +6214,13 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="F10">
         <v>6</v>
       </c>
       <c r="G10" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="J10">
         <v>8</v>
@@ -6240,13 +6240,13 @@
         <v>7</v>
       </c>
       <c r="G11" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="J11">
         <v>11</v>
       </c>
       <c r="K11" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.25">
@@ -6254,19 +6254,19 @@
         <v>8</v>
       </c>
       <c r="C12" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="F12">
         <v>8</v>
       </c>
       <c r="G12" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="J12">
         <v>11</v>
       </c>
       <c r="K12" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.25">
@@ -6274,19 +6274,19 @@
         <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="F13">
         <v>12</v>
       </c>
       <c r="G13" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="J13">
         <v>13</v>
       </c>
       <c r="K13" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
     </row>
     <row r="14" spans="2:11" x14ac:dyDescent="0.25">
@@ -6300,13 +6300,13 @@
         <v>16</v>
       </c>
       <c r="G14" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="J14">
         <v>15</v>
       </c>
       <c r="K14" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.25">
@@ -6314,19 +6314,19 @@
         <v>15</v>
       </c>
       <c r="C15" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="F15">
         <v>19</v>
       </c>
       <c r="G15" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="J15">
         <v>18</v>
       </c>
       <c r="K15" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.25">
@@ -6334,13 +6334,13 @@
         <v>20</v>
       </c>
       <c r="G16" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="J16">
         <v>20</v>
       </c>
       <c r="K16" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
     </row>
     <row r="17" spans="10:11" x14ac:dyDescent="0.25">
@@ -6348,7 +6348,7 @@
         <v>20</v>
       </c>
       <c r="K17" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
     </row>
     <row r="18" spans="10:11" x14ac:dyDescent="0.25">
@@ -6356,27 +6356,27 @@
         <v>25</v>
       </c>
       <c r="K18" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
     </row>
     <row r="27" spans="10:11" x14ac:dyDescent="0.25">
       <c r="K27" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
     </row>
     <row r="28" spans="10:11" x14ac:dyDescent="0.25">
       <c r="K28" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
     </row>
     <row r="29" spans="10:11" x14ac:dyDescent="0.25">
       <c r="K29" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
     </row>
     <row r="30" spans="10:11" x14ac:dyDescent="0.25">
       <c r="K30" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
   </sheetData>
@@ -6409,7 +6409,7 @@
         <v>63</v>
       </c>
       <c r="I6" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="L6" t="s">
         <v>54</v>
@@ -6418,7 +6418,7 @@
         <v>55</v>
       </c>
       <c r="R6" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="V6" t="s">
         <v>66</v>
@@ -6429,7 +6429,7 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -6441,31 +6441,31 @@
         <v>1</v>
       </c>
       <c r="I7" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="K7">
         <v>1</v>
       </c>
       <c r="L7" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="N7">
         <v>1</v>
       </c>
       <c r="O7" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="Q7">
         <v>1</v>
       </c>
       <c r="R7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="U7">
         <v>1</v>
       </c>
       <c r="V7" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
     </row>
     <row r="8" spans="2:22" x14ac:dyDescent="0.25">
@@ -6473,7 +6473,7 @@
         <v>3</v>
       </c>
       <c r="C8" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="E8">
         <v>4</v>
@@ -6485,13 +6485,13 @@
         <v>1</v>
       </c>
       <c r="I8" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="K8">
         <v>1</v>
       </c>
       <c r="L8" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="N8">
         <v>1</v>
@@ -6503,13 +6503,13 @@
         <v>3</v>
       </c>
       <c r="R8" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="U8">
         <v>2</v>
       </c>
       <c r="V8" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
     </row>
     <row r="9" spans="2:22" x14ac:dyDescent="0.25">
@@ -6517,13 +6517,13 @@
         <v>5</v>
       </c>
       <c r="C9" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="E9">
         <v>4</v>
       </c>
       <c r="F9" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="H9">
         <v>4</v>
@@ -6547,13 +6547,13 @@
         <v>5</v>
       </c>
       <c r="R9" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="U9">
         <v>2</v>
       </c>
       <c r="V9" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
     </row>
     <row r="10" spans="2:22" x14ac:dyDescent="0.25">
@@ -6561,13 +6561,13 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="E10">
         <v>6</v>
       </c>
       <c r="F10" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="H10">
         <v>5</v>
@@ -6579,13 +6579,13 @@
         <v>8</v>
       </c>
       <c r="L10" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="N10">
         <v>8</v>
       </c>
       <c r="O10" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="Q10">
         <v>8</v>
@@ -6597,7 +6597,7 @@
         <v>6</v>
       </c>
       <c r="V10" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
     </row>
     <row r="11" spans="2:22" x14ac:dyDescent="0.25">
@@ -6605,13 +6605,13 @@
         <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="E11">
         <v>8</v>
       </c>
       <c r="F11" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="H11">
         <v>7</v>
@@ -6635,13 +6635,13 @@
         <v>10</v>
       </c>
       <c r="R11" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="U11">
         <v>7</v>
       </c>
       <c r="V11" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
     </row>
     <row r="12" spans="2:22" x14ac:dyDescent="0.25">
@@ -6649,43 +6649,43 @@
         <v>10</v>
       </c>
       <c r="C12" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="E12">
         <v>11</v>
       </c>
       <c r="F12" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="H12">
         <v>8</v>
       </c>
       <c r="I12" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="K12">
         <v>12</v>
       </c>
       <c r="L12" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="N12">
         <v>12</v>
       </c>
       <c r="O12" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="Q12">
         <v>12</v>
       </c>
       <c r="R12" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="U12">
         <v>8</v>
       </c>
       <c r="V12" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
     </row>
     <row r="13" spans="2:22" x14ac:dyDescent="0.25">
@@ -6693,43 +6693,43 @@
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="E13">
         <v>14</v>
       </c>
       <c r="F13" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="H13">
         <v>9</v>
       </c>
       <c r="I13" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="K13">
         <v>14</v>
       </c>
       <c r="L13" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="N13">
         <v>14</v>
       </c>
       <c r="O13" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="Q13">
         <v>14</v>
       </c>
       <c r="R13" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="U13">
         <v>9</v>
       </c>
       <c r="V13" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
     </row>
     <row r="14" spans="2:22" x14ac:dyDescent="0.25">
@@ -6737,7 +6737,7 @@
         <v>14</v>
       </c>
       <c r="C14" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="E14">
         <v>16</v>
@@ -6767,13 +6767,13 @@
         <v>15</v>
       </c>
       <c r="R14" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="U14">
         <v>14</v>
       </c>
       <c r="V14" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
     </row>
     <row r="15" spans="2:22" x14ac:dyDescent="0.25">
@@ -6781,43 +6781,43 @@
         <v>15</v>
       </c>
       <c r="C15" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="E15">
         <v>18</v>
       </c>
       <c r="F15" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="H15">
         <v>16</v>
       </c>
       <c r="I15" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="K15">
         <v>20</v>
       </c>
       <c r="L15" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="N15">
         <v>16</v>
       </c>
       <c r="O15" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="Q15">
         <v>16</v>
       </c>
       <c r="R15" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="U15">
         <v>17</v>
       </c>
       <c r="V15" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
     </row>
     <row r="16" spans="2:22" x14ac:dyDescent="0.25">
@@ -6825,37 +6825,37 @@
         <v>20</v>
       </c>
       <c r="F16" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="H16">
         <v>20</v>
       </c>
       <c r="I16" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="K16">
         <v>20</v>
       </c>
       <c r="L16" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="N16">
         <v>20</v>
       </c>
       <c r="O16" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="Q16">
         <v>20</v>
       </c>
       <c r="R16" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="U16">
         <v>20</v>
       </c>
       <c r="V16" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="17" spans="11:22" x14ac:dyDescent="0.25">
@@ -6863,25 +6863,25 @@
         <v>24</v>
       </c>
       <c r="L17" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="N17">
         <v>23</v>
       </c>
       <c r="O17" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="Q17">
         <v>24</v>
       </c>
       <c r="R17" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="U17">
         <v>24</v>
       </c>
       <c r="V17" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
     </row>
     <row r="18" spans="11:22" x14ac:dyDescent="0.25">
@@ -6889,75 +6889,75 @@
         <v>25</v>
       </c>
       <c r="L18" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="N18">
         <v>25</v>
       </c>
       <c r="O18" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="Q18">
         <v>25</v>
       </c>
       <c r="R18" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="U18">
         <v>25</v>
       </c>
       <c r="V18" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
     </row>
     <row r="22" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L22" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
     </row>
     <row r="23" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L23" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="24" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L24" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
     </row>
     <row r="25" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L25" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="26" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L26" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
     </row>
     <row r="27" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L27" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
     </row>
     <row r="28" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L28" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
     <row r="29" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L29" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
     </row>
     <row r="30" spans="11:22" x14ac:dyDescent="0.25">
       <c r="L30" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
     </row>
     <row r="33" spans="13:13" x14ac:dyDescent="0.25">
       <c r="M33" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
     </row>
   </sheetData>
@@ -6999,25 +6999,25 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E7">
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="H7">
         <v>1</v>
       </c>
       <c r="I7" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="K7">
         <v>1</v>
       </c>
       <c r="L7" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
@@ -7025,25 +7025,25 @@
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>272</v>
+        <v>631</v>
       </c>
       <c r="E8">
         <v>2</v>
       </c>
       <c r="F8" s="39" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="H8">
         <v>2</v>
       </c>
       <c r="I8" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="K8">
         <v>1</v>
       </c>
       <c r="L8" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
@@ -7051,13 +7051,13 @@
         <v>2</v>
       </c>
       <c r="C9" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="E9">
         <v>3</v>
       </c>
       <c r="F9" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="H9">
         <v>5</v>
@@ -7069,7 +7069,7 @@
         <v>3</v>
       </c>
       <c r="L9" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
@@ -7077,25 +7077,25 @@
         <v>3</v>
       </c>
       <c r="C10" t="s">
-        <v>312</v>
+        <v>632</v>
       </c>
       <c r="E10">
         <v>4</v>
       </c>
       <c r="F10" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="H10">
         <v>8</v>
       </c>
       <c r="I10" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="K10">
         <v>4</v>
       </c>
       <c r="L10" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
@@ -7103,13 +7103,13 @@
         <v>4</v>
       </c>
       <c r="C11" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="E11">
         <v>8</v>
       </c>
       <c r="F11" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="H11">
         <v>10</v>
@@ -7121,7 +7121,7 @@
         <v>5</v>
       </c>
       <c r="L11" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
@@ -7129,25 +7129,25 @@
         <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="E12">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F12" t="s">
-        <v>283</v>
+        <v>654</v>
       </c>
       <c r="H12">
         <v>11</v>
       </c>
       <c r="I12" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="K12">
         <v>8</v>
       </c>
       <c r="L12" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
@@ -7155,25 +7155,25 @@
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="E13">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F13" t="s">
-        <v>655</v>
+        <v>321</v>
       </c>
       <c r="H13">
         <v>14</v>
       </c>
       <c r="I13" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="K13">
         <v>10</v>
       </c>
       <c r="L13" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
@@ -7181,13 +7181,13 @@
         <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="E14">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F14" t="s">
-        <v>354</v>
+        <v>653</v>
       </c>
       <c r="H14">
         <v>15</v>
@@ -7199,7 +7199,7 @@
         <v>15</v>
       </c>
       <c r="L14" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.25">
@@ -7210,22 +7210,22 @@
         <v>233</v>
       </c>
       <c r="E15">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F15" t="s">
-        <v>654</v>
+        <v>237</v>
       </c>
       <c r="H15">
         <v>17</v>
       </c>
       <c r="I15" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="K15">
         <v>18</v>
       </c>
       <c r="L15" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
@@ -7233,84 +7233,78 @@
         <v>15</v>
       </c>
       <c r="C16" s="39" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="E16">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F16" t="s">
-        <v>237</v>
+        <v>659</v>
       </c>
       <c r="H16">
         <v>20</v>
       </c>
       <c r="I16" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="K16">
         <v>20</v>
       </c>
       <c r="L16" t="s">
-        <v>787</v>
-      </c>
-    </row>
-    <row r="17" spans="5:12" x14ac:dyDescent="0.25">
-      <c r="E17">
-        <v>20</v>
-      </c>
-      <c r="F17" t="s">
-        <v>660</v>
-      </c>
+        <v>786</v>
+      </c>
+    </row>
+    <row r="17" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H17">
         <v>23</v>
       </c>
       <c r="I17" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="K17">
         <v>21</v>
       </c>
       <c r="L17" t="s">
-        <v>664</v>
-      </c>
-    </row>
-    <row r="18" spans="5:12" x14ac:dyDescent="0.25">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="18" spans="8:12" x14ac:dyDescent="0.25">
       <c r="H18">
         <v>25</v>
       </c>
       <c r="I18" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="K18">
         <v>25</v>
       </c>
       <c r="L18" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="22" spans="5:12" x14ac:dyDescent="0.25">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="22" spans="8:12" x14ac:dyDescent="0.25">
       <c r="I22" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="23" spans="8:12" x14ac:dyDescent="0.25">
+      <c r="I23" t="s">
         <v>547</v>
       </c>
     </row>
-    <row r="23" spans="5:12" x14ac:dyDescent="0.25">
-      <c r="I23" t="s">
-        <v>548</v>
-      </c>
-    </row>
-    <row r="24" spans="5:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="8:12" x14ac:dyDescent="0.25">
       <c r="I24" t="s">
-        <v>659</v>
-      </c>
-    </row>
-    <row r="25" spans="5:12" x14ac:dyDescent="0.25">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="25" spans="8:12" x14ac:dyDescent="0.25">
       <c r="I25" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="26" spans="8:12" x14ac:dyDescent="0.25">
+      <c r="I26" t="s">
         <v>550</v>
-      </c>
-    </row>
-    <row r="26" spans="5:12" x14ac:dyDescent="0.25">
-      <c r="I26" t="s">
-        <v>551</v>
       </c>
     </row>
   </sheetData>
@@ -8681,10 +8675,10 @@
     <row r="7" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B8" s="35" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="C8" s="36" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="H8" t="s">
         <v>12</v>
@@ -8864,7 +8858,7 @@
         <v>248</v>
       </c>
       <c r="M17" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.25">
@@ -9118,7 +9112,7 @@
         <v>63</v>
       </c>
       <c r="I32" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="L32" t="s">
         <v>51</v>
@@ -9129,16 +9123,16 @@
     </row>
     <row r="33" spans="8:13" x14ac:dyDescent="0.25">
       <c r="H33" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="I33" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="L33" t="s">
         <v>54</v>
       </c>
       <c r="M33" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="34" spans="8:13" x14ac:dyDescent="0.25">
@@ -9146,7 +9140,7 @@
         <v>64</v>
       </c>
       <c r="I34" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="L34" t="s">
         <v>55</v>
@@ -9160,13 +9154,13 @@
         <v>59</v>
       </c>
       <c r="I35" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="L35" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="M35" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
     </row>
     <row r="36" spans="8:13" x14ac:dyDescent="0.25">
@@ -9174,7 +9168,7 @@
         <v>58</v>
       </c>
       <c r="M36" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
     </row>
     <row r="37" spans="8:13" x14ac:dyDescent="0.25">
@@ -9182,7 +9176,7 @@
         <v>61</v>
       </c>
       <c r="M37" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
   </sheetData>
@@ -9200,7 +9194,7 @@
   <sheetData>
     <row r="5" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="6" spans="2:2" x14ac:dyDescent="0.25">
@@ -9210,7 +9204,7 @@
     </row>
     <row r="8" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
     </row>
     <row r="9" spans="2:2" x14ac:dyDescent="0.25">
@@ -9240,7 +9234,7 @@
     </row>
     <row r="16" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
     </row>
   </sheetData>
@@ -9357,13 +9351,13 @@
         <v>2</v>
       </c>
       <c r="L8" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="N8">
         <v>2</v>
       </c>
       <c r="O8" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="Q8">
         <v>2</v>
@@ -9375,7 +9369,7 @@
         <v>2</v>
       </c>
       <c r="U8" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
     </row>
     <row r="9" spans="2:21" x14ac:dyDescent="0.25">
@@ -9471,19 +9465,19 @@
         <v>8</v>
       </c>
       <c r="C11" s="37" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="E11">
         <v>8</v>
       </c>
       <c r="F11" s="37" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="H11">
         <v>8</v>
       </c>
       <c r="I11" s="37" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="K11">
         <v>10</v>
@@ -9521,7 +9515,7 @@
         <v>10</v>
       </c>
       <c r="F12" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="H12">
         <v>10</v>
@@ -9577,25 +9571,25 @@
         <v>14</v>
       </c>
       <c r="L13" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="N13">
         <v>14</v>
       </c>
       <c r="O13" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="Q13">
         <v>14</v>
       </c>
       <c r="R13" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="T13">
         <v>14</v>
       </c>
       <c r="U13" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="14" spans="2:21" x14ac:dyDescent="0.25">
@@ -9609,13 +9603,13 @@
         <v>15</v>
       </c>
       <c r="F14" s="39" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="H14">
         <v>15</v>
       </c>
       <c r="I14" s="39" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="K14">
         <v>15</v>
@@ -9703,25 +9697,25 @@
         <v>20</v>
       </c>
       <c r="L16" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="N16">
         <v>20</v>
       </c>
       <c r="O16" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="Q16">
         <v>20</v>
       </c>
       <c r="R16" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="T16">
         <v>20</v>
       </c>
       <c r="U16" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
     </row>
     <row r="17" spans="9:21" x14ac:dyDescent="0.25">
@@ -9778,42 +9772,42 @@
     </row>
     <row r="22" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I22" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
     </row>
     <row r="23" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I23" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
     </row>
     <row r="24" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I24" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
     </row>
     <row r="25" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I25" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="26" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I26" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
     </row>
     <row r="27" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I27" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
     </row>
     <row r="28" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I28" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="29" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I29" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
     </row>
     <row r="36" spans="11:11" x14ac:dyDescent="0.25">
@@ -9904,7 +9898,7 @@
         <v>3</v>
       </c>
       <c r="I8" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="K8">
         <v>3</v>
@@ -9936,13 +9930,13 @@
         <v>5</v>
       </c>
       <c r="I9" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="K9">
         <v>5</v>
       </c>
       <c r="L9" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="N9">
         <v>5</v>
@@ -9968,13 +9962,13 @@
         <v>8</v>
       </c>
       <c r="I10" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="K10">
         <v>8</v>
       </c>
       <c r="L10" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="N10">
         <v>6</v>
@@ -10058,25 +10052,25 @@
         <v>14</v>
       </c>
       <c r="F13" s="39" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="H13">
         <v>14</v>
       </c>
       <c r="I13" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="K13">
         <v>14</v>
       </c>
       <c r="L13" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="N13">
         <v>14</v>
       </c>
       <c r="O13" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.25">
@@ -10108,7 +10102,7 @@
         <v>15</v>
       </c>
       <c r="O14" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.25">
@@ -10154,19 +10148,19 @@
         <v>20</v>
       </c>
       <c r="I16" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="K16">
         <v>20</v>
       </c>
       <c r="L16" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="N16">
         <v>21</v>
       </c>
       <c r="O16" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
     </row>
     <row r="17" spans="8:15" x14ac:dyDescent="0.25">
@@ -10194,13 +10188,13 @@
         <v>25</v>
       </c>
       <c r="I18" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="K18">
         <v>25</v>
       </c>
       <c r="L18" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="N18">
         <v>25</v>
@@ -10211,27 +10205,27 @@
     </row>
     <row r="22" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I22" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="23" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I23" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="24" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I24" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="25" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I25" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="26" spans="8:15" x14ac:dyDescent="0.25">
       <c r="I26" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
     </row>
   </sheetData>
@@ -10339,7 +10333,7 @@
         <v>4</v>
       </c>
       <c r="C9" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="E9">
         <v>4</v>
@@ -10377,7 +10371,7 @@
         <v>4</v>
       </c>
       <c r="F10" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="H10">
         <v>8</v>
@@ -10389,7 +10383,7 @@
         <v>7</v>
       </c>
       <c r="L10" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="N10">
         <v>5</v>
@@ -10441,7 +10435,7 @@
         <v>8</v>
       </c>
       <c r="F12" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="H12">
         <v>12</v>
@@ -10453,7 +10447,7 @@
         <v>10</v>
       </c>
       <c r="L12" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="N12">
         <v>10</v>
@@ -10473,7 +10467,7 @@
         <v>11</v>
       </c>
       <c r="F13" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="H13">
         <v>14</v>
@@ -10499,7 +10493,7 @@
         <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="E14">
         <v>14</v>
@@ -10517,7 +10511,7 @@
         <v>15</v>
       </c>
       <c r="L14" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="N14">
         <v>17</v>
@@ -10543,7 +10537,7 @@
         <v>16</v>
       </c>
       <c r="I15" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="K15">
         <v>16</v>
@@ -10581,7 +10575,7 @@
         <v>17</v>
       </c>
       <c r="L16" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="N16">
         <v>21</v>
@@ -10627,7 +10621,7 @@
         <v>25</v>
       </c>
       <c r="O18" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
   </sheetData>
@@ -10684,7 +10678,7 @@
         <v>1</v>
       </c>
       <c r="L7" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
@@ -10736,7 +10730,7 @@
         <v>5</v>
       </c>
       <c r="L9" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
@@ -10776,7 +10770,7 @@
         <v>10</v>
       </c>
       <c r="F11" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="H11">
         <v>10</v>
@@ -10788,7 +10782,7 @@
         <v>7</v>
       </c>
       <c r="L11" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
@@ -10814,7 +10808,7 @@
         <v>9</v>
       </c>
       <c r="L12" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
@@ -10822,13 +10816,13 @@
         <v>10</v>
       </c>
       <c r="C13" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="E13">
         <v>14</v>
       </c>
       <c r="F13" s="39" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="H13">
         <v>14</v>
@@ -10840,7 +10834,7 @@
         <v>11</v>
       </c>
       <c r="L13" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
@@ -10860,7 +10854,7 @@
         <v>15</v>
       </c>
       <c r="I14" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="K14">
         <v>16</v>
@@ -10886,13 +10880,13 @@
         <v>16</v>
       </c>
       <c r="I15" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="K15">
         <v>20</v>
       </c>
       <c r="L15" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
@@ -10932,7 +10926,7 @@
         <v>22</v>
       </c>
       <c r="L17" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
     </row>
     <row r="18" spans="8:12" x14ac:dyDescent="0.25">
@@ -10946,7 +10940,7 @@
         <v>25</v>
       </c>
       <c r="L18" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
   </sheetData>
@@ -11169,12 +11163,12 @@
         <v>8</v>
       </c>
       <c r="U10" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
     </row>
     <row r="11" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B11">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C11" t="s">
         <v>317</v>
@@ -11201,19 +11195,19 @@
         <v>9</v>
       </c>
       <c r="O11" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="Q11">
         <v>9</v>
       </c>
       <c r="R11" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="T11">
         <v>9</v>
       </c>
       <c r="U11" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
     </row>
     <row r="12" spans="2:21" x14ac:dyDescent="0.25">
@@ -11289,19 +11283,19 @@
         <v>14</v>
       </c>
       <c r="O13" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="Q13">
         <v>14</v>
       </c>
       <c r="R13" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="T13">
         <v>14</v>
       </c>
       <c r="U13" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
     </row>
     <row r="14" spans="2:21" x14ac:dyDescent="0.25">
@@ -11345,7 +11339,7 @@
         <v>15</v>
       </c>
       <c r="U14" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="15" spans="2:21" x14ac:dyDescent="0.25">
@@ -11377,19 +11371,19 @@
         <v>17</v>
       </c>
       <c r="O15" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="Q15">
         <v>17</v>
       </c>
       <c r="R15" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="T15">
         <v>17</v>
       </c>
       <c r="U15" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="16" spans="2:21" x14ac:dyDescent="0.25">
@@ -11421,7 +11415,7 @@
         <v>21</v>
       </c>
       <c r="O16" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="Q16">
         <v>21</v>
@@ -11441,19 +11435,19 @@
         <v>22</v>
       </c>
       <c r="O17" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="Q17">
         <v>22</v>
       </c>
       <c r="R17" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="T17">
         <v>22</v>
       </c>
       <c r="U17" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="18" spans="9:21" x14ac:dyDescent="0.25">
@@ -11508,7 +11502,7 @@
     </row>
     <row r="30" spans="9:21" x14ac:dyDescent="0.25">
       <c r="I30" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
hp mp y ruta lista para exportar
</commit_message>
<xml_diff>
--- a/arquetiposZ.xlsx
+++ b/arquetiposZ.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sergius\Desktop\Proyectos\hyperbole\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ACE246F-6AF6-4693-8851-3E79DEA21016}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84D255F0-A026-454D-9E30-3ACD96D9B4BA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="644" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="644" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RESUMEN" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1145" uniqueCount="813">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1212" uniqueCount="818">
   <si>
     <t>daños:</t>
   </si>
@@ -2483,6 +2483,21 @@
   </si>
   <si>
     <t>romper res fisicos</t>
+  </si>
+  <si>
+    <t>HP</t>
+  </si>
+  <si>
+    <t>MP</t>
+  </si>
+  <si>
+    <t>r2 -&gt; 750 a 900</t>
+  </si>
+  <si>
+    <t>r3 -&gt; 1300 a 1500</t>
+  </si>
+  <si>
+    <t>r1 -&gt; 330 a 350</t>
   </si>
 </sst>
 </file>
@@ -2512,7 +2527,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="38">
+  <borders count="43">
     <border>
       <left/>
       <right/>
@@ -2718,40 +2733,10 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="dotted">
         <color indexed="64"/>
       </left>
       <right style="dotted">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="dotted">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="dotted">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
         <color indexed="64"/>
       </right>
       <top style="thin">
@@ -2781,37 +2766,7 @@
       <left style="dotted">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="dotted">
-        <color indexed="64"/>
-      </top>
-      <bottom style="dotted">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="dotted">
-        <color indexed="64"/>
-      </left>
       <right style="dotted">
-        <color indexed="64"/>
-      </right>
-      <top style="dotted">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="dotted">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
         <color indexed="64"/>
       </right>
       <top style="dotted">
@@ -2969,11 +2924,146 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="dotted">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dotted">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="dotted">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="dotted">
+        <color indexed="64"/>
+      </top>
+      <bottom style="dotted">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dotted">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="dotted">
+        <color indexed="64"/>
+      </top>
+      <bottom style="dotted">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="dotted">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dotted">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="dotted">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
@@ -3007,18 +3097,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3068,6 +3154,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3572,29 +3672,29 @@
     </row>
     <row r="4" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B4" s="12"/>
-      <c r="C4" s="49" t="s">
+      <c r="C4" s="45" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="51"/>
+      <c r="D4" s="47"/>
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
       <c r="G4" s="5"/>
       <c r="H4" s="5"/>
-      <c r="I4" s="49" t="s">
+      <c r="I4" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="J4" s="50"/>
-      <c r="K4" s="50"/>
-      <c r="L4" s="49" t="s">
+      <c r="J4" s="46"/>
+      <c r="K4" s="46"/>
+      <c r="L4" s="45" t="s">
         <v>374</v>
       </c>
-      <c r="M4" s="50"/>
-      <c r="N4" s="50"/>
-      <c r="O4" s="50"/>
-      <c r="P4" s="50"/>
-      <c r="Q4" s="50"/>
-      <c r="R4" s="50"/>
-      <c r="S4" s="51"/>
+      <c r="M4" s="46"/>
+      <c r="N4" s="46"/>
+      <c r="O4" s="46"/>
+      <c r="P4" s="46"/>
+      <c r="Q4" s="46"/>
+      <c r="R4" s="46"/>
+      <c r="S4" s="47"/>
       <c r="T4" s="13"/>
     </row>
     <row r="5" spans="2:20" x14ac:dyDescent="0.25">
@@ -3620,7 +3720,7 @@
     </row>
     <row r="6" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B6" s="12"/>
-      <c r="C6" s="52" t="s">
+      <c r="C6" s="48" t="s">
         <v>362</v>
       </c>
       <c r="D6" s="2" t="s">
@@ -3653,7 +3753,7 @@
     </row>
     <row r="7" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B7" s="12"/>
-      <c r="C7" s="52"/>
+      <c r="C7" s="48"/>
       <c r="D7" s="2" t="s">
         <v>2</v>
       </c>
@@ -3680,7 +3780,7 @@
     </row>
     <row r="8" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B8" s="12"/>
-      <c r="C8" s="52"/>
+      <c r="C8" s="48"/>
       <c r="D8" s="2" t="s">
         <v>3</v>
       </c>
@@ -3734,7 +3834,7 @@
     </row>
     <row r="10" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B10" s="12"/>
-      <c r="C10" s="53" t="s">
+      <c r="C10" s="49" t="s">
         <v>363</v>
       </c>
       <c r="D10" s="2" t="s">
@@ -3767,7 +3867,7 @@
     </row>
     <row r="11" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B11" s="12"/>
-      <c r="C11" s="52"/>
+      <c r="C11" s="48"/>
       <c r="D11" s="2" t="s">
         <v>5</v>
       </c>
@@ -3794,7 +3894,7 @@
     </row>
     <row r="12" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B12" s="12"/>
-      <c r="C12" s="52"/>
+      <c r="C12" s="48"/>
       <c r="D12" s="2" t="s">
         <v>6</v>
       </c>
@@ -3821,7 +3921,7 @@
     </row>
     <row r="13" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B13" s="12"/>
-      <c r="C13" s="52"/>
+      <c r="C13" s="48"/>
       <c r="D13" s="2" t="s">
         <v>7</v>
       </c>
@@ -3885,7 +3985,7 @@
     </row>
     <row r="15" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B15" s="12"/>
-      <c r="C15" s="53" t="s">
+      <c r="C15" s="49" t="s">
         <v>364</v>
       </c>
       <c r="D15" s="2" t="s">
@@ -3920,7 +4020,7 @@
     </row>
     <row r="16" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B16" s="12"/>
-      <c r="C16" s="52"/>
+      <c r="C16" s="48"/>
       <c r="D16" s="2" t="s">
         <v>8</v>
       </c>
@@ -3951,7 +4051,7 @@
     </row>
     <row r="17" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B17" s="12"/>
-      <c r="C17" s="52"/>
+      <c r="C17" s="48"/>
       <c r="D17" s="2" t="s">
         <v>9</v>
       </c>
@@ -3978,7 +4078,7 @@
     </row>
     <row r="18" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B18" s="12"/>
-      <c r="C18" s="52"/>
+      <c r="C18" s="48"/>
       <c r="D18" s="2" t="s">
         <v>10</v>
       </c>
@@ -4036,10 +4136,10 @@
     </row>
     <row r="20" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="12"/>
-      <c r="C20" s="43" t="s">
+      <c r="C20" s="39" t="s">
         <v>367</v>
       </c>
-      <c r="D20" s="45"/>
+      <c r="D20" s="41"/>
       <c r="E20" s="5"/>
       <c r="F20" s="5"/>
       <c r="G20" s="5"/>
@@ -4123,11 +4223,11 @@
     </row>
     <row r="23" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B23" s="12"/>
-      <c r="C23" s="49" t="s">
+      <c r="C23" s="45" t="s">
         <v>361</v>
       </c>
-      <c r="D23" s="50"/>
-      <c r="E23" s="51"/>
+      <c r="D23" s="46"/>
+      <c r="E23" s="47"/>
       <c r="F23" s="5"/>
       <c r="G23" s="5"/>
       <c r="H23" s="5"/>
@@ -4492,11 +4592,11 @@
     </row>
     <row r="36" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B36" s="12"/>
-      <c r="C36" s="40" t="s">
+      <c r="C36" s="36" t="s">
         <v>368</v>
       </c>
-      <c r="D36" s="41"/>
-      <c r="E36" s="42"/>
+      <c r="D36" s="37"/>
+      <c r="E36" s="38"/>
       <c r="F36" s="5"/>
       <c r="G36" s="5"/>
       <c r="H36" s="5"/>
@@ -4515,9 +4615,9 @@
     </row>
     <row r="37" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B37" s="12"/>
-      <c r="C37" s="43"/>
-      <c r="D37" s="44"/>
-      <c r="E37" s="45"/>
+      <c r="C37" s="39"/>
+      <c r="D37" s="40"/>
+      <c r="E37" s="41"/>
       <c r="F37" s="5"/>
       <c r="G37" s="5"/>
       <c r="H37" s="5"/>
@@ -4536,9 +4636,9 @@
     </row>
     <row r="38" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B38" s="12"/>
-      <c r="C38" s="43"/>
-      <c r="D38" s="44"/>
-      <c r="E38" s="45"/>
+      <c r="C38" s="39"/>
+      <c r="D38" s="40"/>
+      <c r="E38" s="41"/>
       <c r="F38" s="5"/>
       <c r="G38" s="5"/>
       <c r="H38" s="5"/>
@@ -4557,25 +4657,25 @@
     </row>
     <row r="39" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B39" s="12"/>
-      <c r="C39" s="46"/>
-      <c r="D39" s="47"/>
-      <c r="E39" s="48"/>
+      <c r="C39" s="42"/>
+      <c r="D39" s="43"/>
+      <c r="E39" s="44"/>
       <c r="F39" s="5"/>
-      <c r="G39" s="49" t="s">
+      <c r="G39" s="45" t="s">
         <v>375</v>
       </c>
-      <c r="H39" s="50"/>
-      <c r="I39" s="50"/>
-      <c r="J39" s="50"/>
-      <c r="K39" s="50"/>
-      <c r="L39" s="50"/>
-      <c r="M39" s="50"/>
-      <c r="N39" s="50"/>
-      <c r="O39" s="50"/>
-      <c r="P39" s="50"/>
-      <c r="Q39" s="50"/>
-      <c r="R39" s="50"/>
-      <c r="S39" s="51"/>
+      <c r="H39" s="46"/>
+      <c r="I39" s="46"/>
+      <c r="J39" s="46"/>
+      <c r="K39" s="46"/>
+      <c r="L39" s="46"/>
+      <c r="M39" s="46"/>
+      <c r="N39" s="46"/>
+      <c r="O39" s="46"/>
+      <c r="P39" s="46"/>
+      <c r="Q39" s="46"/>
+      <c r="R39" s="46"/>
+      <c r="S39" s="47"/>
       <c r="T39" s="13"/>
     </row>
     <row r="40" spans="2:20" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4722,7 +4822,7 @@
       <c r="B11">
         <v>7</v>
       </c>
-      <c r="C11" s="39" t="s">
+      <c r="C11" s="35" t="s">
         <v>394</v>
       </c>
       <c r="F11">
@@ -5247,7 +5347,7 @@
       <c r="B14">
         <v>13</v>
       </c>
-      <c r="C14" s="39" t="s">
+      <c r="C14" s="35" t="s">
         <v>747</v>
       </c>
       <c r="E14">
@@ -5600,7 +5700,7 @@
       <c r="T7">
         <v>1</v>
       </c>
-      <c r="U7" s="39" t="s">
+      <c r="U7" s="35" t="s">
         <v>760</v>
       </c>
     </row>
@@ -5790,7 +5890,7 @@
       <c r="E12">
         <v>12</v>
       </c>
-      <c r="F12" s="39" t="s">
+      <c r="F12" s="35" t="s">
         <v>748</v>
       </c>
       <c r="H12">
@@ -7030,7 +7130,7 @@
       <c r="E8">
         <v>2</v>
       </c>
-      <c r="F8" s="39" t="s">
+      <c r="F8" s="35" t="s">
         <v>745</v>
       </c>
       <c r="H8">
@@ -7232,7 +7332,7 @@
       <c r="B16">
         <v>15</v>
       </c>
-      <c r="C16" s="39" t="s">
+      <c r="C16" s="35" t="s">
         <v>749</v>
       </c>
       <c r="E16">
@@ -7314,1345 +7414,1974 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17742D48-5777-4272-A622-CC37012FB88C}">
-  <dimension ref="C4:T38"/>
+  <dimension ref="C3:AA38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="13" customWidth="1"/>
     <col min="4" max="11" width="6.7109375" customWidth="1"/>
     <col min="12" max="12" width="16.140625" customWidth="1"/>
     <col min="13" max="20" width="6.7109375" customWidth="1"/>
+    <col min="22" max="22" width="13.42578125" customWidth="1"/>
+    <col min="23" max="23" width="8" customWidth="1"/>
+    <col min="24" max="24" width="8.140625" customWidth="1"/>
+    <col min="25" max="25" width="15.85546875" customWidth="1"/>
+    <col min="26" max="26" width="7.42578125" customWidth="1"/>
+    <col min="27" max="27" width="7.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C4" s="17" t="s">
+    <row r="3" spans="3:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C4" s="50" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="D4" s="51" t="s">
         <v>417</v>
       </c>
-      <c r="E4" s="17" t="s">
+      <c r="E4" s="51" t="s">
         <v>418</v>
       </c>
-      <c r="F4" s="17" t="s">
+      <c r="F4" s="51" t="s">
         <v>419</v>
       </c>
-      <c r="G4" s="17" t="s">
+      <c r="G4" s="51" t="s">
         <v>422</v>
       </c>
-      <c r="H4" s="17" t="s">
+      <c r="H4" s="51" t="s">
         <v>420</v>
       </c>
-      <c r="I4" s="17" t="s">
+      <c r="I4" s="51" t="s">
         <v>421</v>
       </c>
-      <c r="J4" s="17" t="s">
+      <c r="J4" s="51" t="s">
         <v>423</v>
       </c>
-      <c r="K4" s="17" t="s">
+      <c r="K4" s="51" t="s">
         <v>424</v>
       </c>
-      <c r="L4" s="17" t="s">
+      <c r="L4" s="51" t="s">
         <v>11</v>
       </c>
-      <c r="M4" s="17" t="s">
+      <c r="M4" s="51" t="s">
         <v>417</v>
       </c>
-      <c r="N4" s="17" t="s">
+      <c r="N4" s="51" t="s">
         <v>418</v>
       </c>
-      <c r="O4" s="17" t="s">
+      <c r="O4" s="51" t="s">
         <v>419</v>
       </c>
-      <c r="P4" s="17" t="s">
+      <c r="P4" s="51" t="s">
         <v>422</v>
       </c>
-      <c r="Q4" s="17" t="s">
+      <c r="Q4" s="51" t="s">
         <v>420</v>
       </c>
-      <c r="R4" s="17" t="s">
+      <c r="R4" s="51" t="s">
         <v>421</v>
       </c>
-      <c r="S4" s="17" t="s">
+      <c r="S4" s="51" t="s">
         <v>423</v>
       </c>
-      <c r="T4" s="17" t="s">
+      <c r="T4" s="52" t="s">
         <v>424</v>
       </c>
-    </row>
-    <row r="5" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C5" s="24" t="s">
+      <c r="V4" s="50" t="s">
+        <v>11</v>
+      </c>
+      <c r="W4" s="51" t="s">
+        <v>813</v>
+      </c>
+      <c r="X4" s="51" t="s">
+        <v>814</v>
+      </c>
+      <c r="Y4" s="51" t="s">
+        <v>11</v>
+      </c>
+      <c r="Z4" s="51" t="s">
+        <v>813</v>
+      </c>
+      <c r="AA4" s="52" t="s">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="5" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C5" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="27"/>
-      <c r="E5" s="18">
+      <c r="D5" s="23"/>
+      <c r="E5" s="17">
         <v>2</v>
       </c>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="18">
-        <v>1</v>
-      </c>
-      <c r="I5" s="18"/>
-      <c r="J5" s="18"/>
-      <c r="K5" s="18">
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="17">
+        <v>1</v>
+      </c>
+      <c r="I5" s="17"/>
+      <c r="J5" s="17"/>
+      <c r="K5" s="17">
         <v>2</v>
       </c>
-      <c r="L5" s="24" t="s">
+      <c r="L5" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="M5" s="27"/>
-      <c r="N5" s="18">
+      <c r="M5" s="23"/>
+      <c r="N5" s="17">
         <v>8</v>
       </c>
-      <c r="O5" s="18">
+      <c r="O5" s="17">
         <v>2</v>
       </c>
-      <c r="P5" s="18"/>
-      <c r="Q5" s="18">
+      <c r="P5" s="17"/>
+      <c r="Q5" s="17">
         <v>3</v>
       </c>
-      <c r="R5" s="18">
+      <c r="R5" s="17">
         <v>4</v>
       </c>
-      <c r="S5" s="18"/>
-      <c r="T5" s="19">
+      <c r="S5" s="17"/>
+      <c r="T5" s="54">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C6" s="25" t="s">
+      <c r="V5" s="53" t="s">
+        <v>12</v>
+      </c>
+      <c r="W5" s="23">
+        <v>132</v>
+      </c>
+      <c r="X5" s="59">
+        <f>350-W5*1.2</f>
+        <v>191.6</v>
+      </c>
+      <c r="Y5" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z5" s="23">
+        <v>467</v>
+      </c>
+      <c r="AA5" s="61">
+        <f>1500-Z5*1.2</f>
+        <v>939.6</v>
+      </c>
+    </row>
+    <row r="6" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C6" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="28"/>
-      <c r="E6" s="20">
+      <c r="D6" s="24"/>
+      <c r="E6" s="18">
         <v>5</v>
       </c>
-      <c r="F6" s="20">
-        <v>1</v>
-      </c>
-      <c r="G6" s="20"/>
-      <c r="H6" s="20">
+      <c r="F6" s="18">
+        <v>1</v>
+      </c>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18">
         <v>2</v>
       </c>
-      <c r="I6" s="20">
-        <v>1</v>
-      </c>
-      <c r="J6" s="20"/>
-      <c r="K6" s="20">
+      <c r="I6" s="18">
+        <v>1</v>
+      </c>
+      <c r="J6" s="18"/>
+      <c r="K6" s="18">
         <v>2</v>
       </c>
-      <c r="L6" s="25" t="s">
+      <c r="L6" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="M6" s="28"/>
-      <c r="N6" s="20">
+      <c r="M6" s="24"/>
+      <c r="N6" s="18">
         <v>8</v>
       </c>
-      <c r="O6" s="20">
+      <c r="O6" s="18">
         <v>5</v>
       </c>
-      <c r="P6" s="20"/>
-      <c r="Q6" s="20">
+      <c r="P6" s="18"/>
+      <c r="Q6" s="18">
         <v>4</v>
       </c>
-      <c r="R6" s="20">
+      <c r="R6" s="18">
         <v>2</v>
       </c>
-      <c r="S6" s="20"/>
-      <c r="T6" s="21">
+      <c r="S6" s="18"/>
+      <c r="T6" s="56">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C7" s="25" t="s">
+      <c r="V6" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="W6" s="24">
+        <v>314</v>
+      </c>
+      <c r="X6" s="60">
+        <f>850-W6*1.2</f>
+        <v>473.2</v>
+      </c>
+      <c r="Y6" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="Z6" s="24">
+        <v>483</v>
+      </c>
+      <c r="AA6" s="63">
+        <f t="shared" ref="AA6:AA33" si="0">1500-Z6*1.2</f>
+        <v>920.4</v>
+      </c>
+    </row>
+    <row r="7" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C7" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="28">
-        <v>1</v>
-      </c>
-      <c r="E7" s="20">
+      <c r="D7" s="24">
+        <v>1</v>
+      </c>
+      <c r="E7" s="18">
         <v>4</v>
       </c>
-      <c r="F7" s="20"/>
-      <c r="G7" s="20">
-        <v>1</v>
-      </c>
-      <c r="H7" s="20">
+      <c r="F7" s="18"/>
+      <c r="G7" s="18">
+        <v>1</v>
+      </c>
+      <c r="H7" s="18">
         <v>2</v>
       </c>
-      <c r="I7" s="20"/>
-      <c r="J7" s="20"/>
-      <c r="K7" s="20">
+      <c r="I7" s="18"/>
+      <c r="J7" s="18"/>
+      <c r="K7" s="18">
         <v>3</v>
       </c>
-      <c r="L7" s="25" t="s">
+      <c r="L7" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="M7" s="28">
+      <c r="M7" s="24">
         <v>3</v>
       </c>
-      <c r="N7" s="20">
+      <c r="N7" s="18">
         <v>8</v>
       </c>
-      <c r="O7" s="20"/>
-      <c r="P7" s="20">
+      <c r="O7" s="18"/>
+      <c r="P7" s="18">
         <v>2</v>
       </c>
-      <c r="Q7" s="20">
+      <c r="Q7" s="18">
         <v>4</v>
       </c>
-      <c r="R7" s="20"/>
-      <c r="S7" s="20"/>
-      <c r="T7" s="21">
+      <c r="R7" s="18"/>
+      <c r="S7" s="18"/>
+      <c r="T7" s="56">
         <v>5</v>
       </c>
-    </row>
-    <row r="8" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C8" s="25" t="s">
+      <c r="V7" s="55" t="s">
+        <v>22</v>
+      </c>
+      <c r="W7">
+        <v>321</v>
+      </c>
+      <c r="X7" s="60">
+        <f>850-W7*1.2</f>
+        <v>464.8</v>
+      </c>
+      <c r="Y7" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z7" s="24">
+        <v>500</v>
+      </c>
+      <c r="AA7" s="63">
+        <f t="shared" si="0"/>
+        <v>900</v>
+      </c>
+    </row>
+    <row r="8" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C8" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="28"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20">
+      <c r="D8" s="24"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18">
         <v>2</v>
       </c>
-      <c r="G8" s="20"/>
-      <c r="H8" s="20"/>
-      <c r="I8" s="20">
+      <c r="G8" s="18"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="18">
         <v>2</v>
       </c>
-      <c r="J8" s="20"/>
-      <c r="K8" s="20">
-        <v>1</v>
-      </c>
-      <c r="L8" s="25" t="s">
+      <c r="J8" s="18"/>
+      <c r="K8" s="18">
+        <v>1</v>
+      </c>
+      <c r="L8" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="M8" s="28">
-        <v>1</v>
-      </c>
-      <c r="N8" s="20">
+      <c r="M8" s="24">
+        <v>1</v>
+      </c>
+      <c r="N8" s="18">
         <v>8</v>
       </c>
-      <c r="O8" s="20"/>
-      <c r="P8" s="20">
-        <v>1</v>
-      </c>
-      <c r="Q8" s="20">
+      <c r="O8" s="18"/>
+      <c r="P8" s="18">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="18">
         <v>3</v>
       </c>
-      <c r="R8" s="20">
+      <c r="R8" s="18">
         <v>3</v>
       </c>
-      <c r="S8" s="20"/>
-      <c r="T8" s="21">
+      <c r="S8" s="18"/>
+      <c r="T8" s="56">
         <v>6</v>
       </c>
-    </row>
-    <row r="9" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C9" s="25" t="s">
+      <c r="V8" s="55" t="s">
+        <v>13</v>
+      </c>
+      <c r="W8" s="24">
+        <v>139</v>
+      </c>
+      <c r="X8" s="60">
+        <f>350-W8*1.2</f>
+        <v>183.20000000000002</v>
+      </c>
+      <c r="Y8" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="Z8" s="24">
+        <v>496</v>
+      </c>
+      <c r="AA8" s="63">
+        <f t="shared" si="0"/>
+        <v>904.80000000000007</v>
+      </c>
+    </row>
+    <row r="9" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C9" s="55" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="28"/>
-      <c r="E9" s="20">
+      <c r="D9" s="24"/>
+      <c r="E9" s="18">
         <v>2</v>
       </c>
-      <c r="F9" s="20">
+      <c r="F9" s="18">
         <v>5</v>
       </c>
-      <c r="G9" s="20"/>
-      <c r="H9" s="20"/>
-      <c r="I9" s="20">
+      <c r="G9" s="18"/>
+      <c r="H9" s="18"/>
+      <c r="I9" s="18">
         <v>3</v>
       </c>
-      <c r="J9" s="20"/>
-      <c r="K9" s="20">
-        <v>1</v>
-      </c>
-      <c r="L9" s="25" t="s">
+      <c r="J9" s="18"/>
+      <c r="K9" s="18">
+        <v>1</v>
+      </c>
+      <c r="L9" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="M9" s="28"/>
-      <c r="N9" s="20">
+      <c r="M9" s="24"/>
+      <c r="N9" s="18">
         <v>4</v>
       </c>
-      <c r="O9" s="20">
+      <c r="O9" s="18">
         <v>8</v>
       </c>
-      <c r="P9" s="20"/>
-      <c r="Q9" s="20">
-        <v>1</v>
-      </c>
-      <c r="R9" s="20">
+      <c r="P9" s="18"/>
+      <c r="Q9" s="18">
+        <v>1</v>
+      </c>
+      <c r="R9" s="18">
         <v>6</v>
       </c>
-      <c r="S9" s="20"/>
-      <c r="T9" s="21">
+      <c r="S9" s="18"/>
+      <c r="T9" s="56">
         <v>3</v>
       </c>
-    </row>
-    <row r="10" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C10" s="25" t="s">
+      <c r="V9" s="55" t="s">
+        <v>15</v>
+      </c>
+      <c r="W9" s="24">
+        <v>333</v>
+      </c>
+      <c r="X9" s="60">
+        <f t="shared" ref="X8:X31" si="1">850-W9*1.2</f>
+        <v>450.40000000000003</v>
+      </c>
+      <c r="Y9" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="Z9" s="24">
+        <v>516</v>
+      </c>
+      <c r="AA9" s="63">
+        <f t="shared" si="0"/>
+        <v>880.80000000000007</v>
+      </c>
+    </row>
+    <row r="10" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C10" s="55" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="28"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20">
+      <c r="D10" s="24"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18">
         <v>2</v>
       </c>
-      <c r="G10" s="20"/>
-      <c r="H10" s="20"/>
-      <c r="I10" s="20">
-        <v>1</v>
-      </c>
-      <c r="J10" s="20"/>
-      <c r="K10" s="20">
+      <c r="G10" s="18"/>
+      <c r="H10" s="18"/>
+      <c r="I10" s="18">
+        <v>1</v>
+      </c>
+      <c r="J10" s="18"/>
+      <c r="K10" s="18">
         <v>2</v>
       </c>
-      <c r="L10" s="25" t="s">
+      <c r="L10" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="M10" s="28"/>
-      <c r="N10" s="20">
+      <c r="M10" s="24"/>
+      <c r="N10" s="18">
         <v>2</v>
       </c>
-      <c r="O10" s="20">
+      <c r="O10" s="18">
         <v>8</v>
       </c>
-      <c r="P10" s="20"/>
-      <c r="Q10" s="20"/>
-      <c r="R10" s="20">
+      <c r="P10" s="18"/>
+      <c r="Q10" s="18"/>
+      <c r="R10" s="18">
         <v>7</v>
       </c>
-      <c r="S10" s="20"/>
-      <c r="T10" s="21">
+      <c r="S10" s="18"/>
+      <c r="T10" s="56">
         <v>5</v>
       </c>
-    </row>
-    <row r="11" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C11" s="25" t="s">
+      <c r="V10" s="55" t="s">
+        <v>25</v>
+      </c>
+      <c r="W10" s="24">
+        <v>150</v>
+      </c>
+      <c r="X10" s="60">
+        <f>350-W10*1.2</f>
+        <v>170</v>
+      </c>
+      <c r="Y10" s="21" t="s">
+        <v>21</v>
+      </c>
+      <c r="Z10" s="24">
+        <v>508</v>
+      </c>
+      <c r="AA10" s="63">
+        <f t="shared" si="0"/>
+        <v>890.4</v>
+      </c>
+    </row>
+    <row r="11" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C11" s="55" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="28"/>
-      <c r="E11" s="20">
-        <v>1</v>
-      </c>
-      <c r="F11" s="20">
+      <c r="D11" s="24"/>
+      <c r="E11" s="18">
+        <v>1</v>
+      </c>
+      <c r="F11" s="18">
         <v>5</v>
       </c>
-      <c r="G11" s="20">
-        <v>1</v>
-      </c>
-      <c r="H11" s="20">
-        <v>1</v>
-      </c>
-      <c r="I11" s="20">
-        <v>1</v>
-      </c>
-      <c r="J11" s="20"/>
-      <c r="K11" s="20">
+      <c r="G11" s="18">
+        <v>1</v>
+      </c>
+      <c r="H11" s="18">
+        <v>1</v>
+      </c>
+      <c r="I11" s="18">
+        <v>1</v>
+      </c>
+      <c r="J11" s="18"/>
+      <c r="K11" s="18">
         <v>2</v>
       </c>
-      <c r="L11" s="25" t="s">
+      <c r="L11" s="21" t="s">
         <v>425</v>
       </c>
-      <c r="M11" s="28"/>
-      <c r="N11" s="20">
+      <c r="M11" s="24"/>
+      <c r="N11" s="18">
         <v>6</v>
       </c>
-      <c r="O11" s="20">
+      <c r="O11" s="18">
         <v>6</v>
       </c>
-      <c r="P11" s="20"/>
-      <c r="Q11" s="20"/>
-      <c r="R11" s="20">
+      <c r="P11" s="18"/>
+      <c r="Q11" s="18"/>
+      <c r="R11" s="18">
         <v>6</v>
       </c>
-      <c r="S11" s="20"/>
-      <c r="T11" s="21">
+      <c r="S11" s="18"/>
+      <c r="T11" s="56">
         <v>4</v>
       </c>
-    </row>
-    <row r="12" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C12" s="25" t="s">
+      <c r="V11" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="W11" s="24">
+        <v>346</v>
+      </c>
+      <c r="X11" s="60">
+        <f t="shared" si="1"/>
+        <v>434.8</v>
+      </c>
+      <c r="Y11" s="21" t="s">
+        <v>425</v>
+      </c>
+      <c r="Z11" s="24">
+        <v>461</v>
+      </c>
+      <c r="AA11" s="63">
+        <f t="shared" si="0"/>
+        <v>946.80000000000007</v>
+      </c>
+    </row>
+    <row r="12" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C12" s="55" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="28">
-        <v>1</v>
-      </c>
-      <c r="E12" s="20"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="20">
-        <v>1</v>
-      </c>
-      <c r="H12" s="20"/>
-      <c r="I12" s="20"/>
-      <c r="J12" s="20">
+      <c r="D12" s="24">
+        <v>1</v>
+      </c>
+      <c r="E12" s="18"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="18">
+        <v>1</v>
+      </c>
+      <c r="H12" s="18"/>
+      <c r="I12" s="18"/>
+      <c r="J12" s="18">
         <v>2</v>
       </c>
-      <c r="K12" s="20">
-        <v>1</v>
-      </c>
-      <c r="L12" s="25" t="s">
+      <c r="K12" s="18">
+        <v>1</v>
+      </c>
+      <c r="L12" s="21" t="s">
         <v>248</v>
       </c>
-      <c r="M12" s="28"/>
-      <c r="N12" s="20">
+      <c r="M12" s="24"/>
+      <c r="N12" s="18">
         <v>4</v>
       </c>
-      <c r="O12" s="20">
+      <c r="O12" s="18">
         <v>7</v>
       </c>
-      <c r="P12" s="20">
-        <v>1</v>
-      </c>
-      <c r="Q12" s="20">
+      <c r="P12" s="18">
+        <v>1</v>
+      </c>
+      <c r="Q12" s="18">
         <v>2</v>
       </c>
-      <c r="R12" s="20">
+      <c r="R12" s="18">
         <v>2</v>
       </c>
-      <c r="S12" s="20"/>
-      <c r="T12" s="21">
+      <c r="S12" s="18"/>
+      <c r="T12" s="56">
         <v>6</v>
       </c>
-    </row>
-    <row r="13" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C13" s="25" t="s">
+      <c r="V12" s="55" t="s">
+        <v>28</v>
+      </c>
+      <c r="W12" s="24">
+        <v>181</v>
+      </c>
+      <c r="X12" s="60">
+        <f>350-W12*1.2</f>
+        <v>132.80000000000001</v>
+      </c>
+      <c r="Y12" s="21" t="s">
+        <v>248</v>
+      </c>
+      <c r="Z12" s="24">
+        <v>521</v>
+      </c>
+      <c r="AA12" s="63">
+        <f t="shared" si="0"/>
+        <v>874.80000000000007</v>
+      </c>
+    </row>
+    <row r="13" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C13" s="55" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="28">
+      <c r="D13" s="24">
         <v>2</v>
       </c>
-      <c r="E13" s="20"/>
-      <c r="F13" s="20">
+      <c r="E13" s="18"/>
+      <c r="F13" s="18">
         <v>3</v>
       </c>
-      <c r="G13" s="20"/>
-      <c r="H13" s="20"/>
-      <c r="I13" s="20"/>
-      <c r="J13" s="20">
+      <c r="G13" s="18"/>
+      <c r="H13" s="18"/>
+      <c r="I13" s="18"/>
+      <c r="J13" s="18">
         <v>5</v>
       </c>
-      <c r="K13" s="20">
-        <v>1</v>
-      </c>
-      <c r="L13" s="25" t="s">
+      <c r="K13" s="18">
+        <v>1</v>
+      </c>
+      <c r="L13" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="M13" s="28"/>
-      <c r="N13" s="20">
+      <c r="M13" s="24"/>
+      <c r="N13" s="18">
         <v>4</v>
       </c>
-      <c r="O13" s="20">
+      <c r="O13" s="18">
         <v>8</v>
       </c>
-      <c r="P13" s="20">
-        <v>1</v>
-      </c>
-      <c r="Q13" s="20">
-        <v>1</v>
-      </c>
-      <c r="R13" s="20">
-        <v>1</v>
-      </c>
-      <c r="S13" s="20"/>
-      <c r="T13" s="21">
+      <c r="P13" s="18">
+        <v>1</v>
+      </c>
+      <c r="Q13" s="18">
+        <v>1</v>
+      </c>
+      <c r="R13" s="18">
+        <v>1</v>
+      </c>
+      <c r="S13" s="18"/>
+      <c r="T13" s="56">
         <v>7</v>
       </c>
-    </row>
-    <row r="14" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C14" s="25" t="s">
+      <c r="V13" s="55" t="s">
+        <v>29</v>
+      </c>
+      <c r="W13" s="24">
+        <v>422</v>
+      </c>
+      <c r="X13" s="60">
+        <f t="shared" si="1"/>
+        <v>343.6</v>
+      </c>
+      <c r="Y13" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="Z13" s="24">
+        <v>542</v>
+      </c>
+      <c r="AA13" s="63">
+        <f t="shared" si="0"/>
+        <v>849.6</v>
+      </c>
+    </row>
+    <row r="14" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C14" s="55" t="s">
         <v>35</v>
       </c>
-      <c r="D14" s="28">
+      <c r="D14" s="24">
         <v>2</v>
       </c>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="20">
-        <v>1</v>
-      </c>
-      <c r="H14" s="20">
-        <v>1</v>
-      </c>
-      <c r="I14" s="20"/>
-      <c r="J14" s="20">
-        <v>1</v>
-      </c>
-      <c r="K14" s="20"/>
-      <c r="L14" s="25" t="s">
+      <c r="E14" s="18"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="18">
+        <v>1</v>
+      </c>
+      <c r="H14" s="18">
+        <v>1</v>
+      </c>
+      <c r="I14" s="18"/>
+      <c r="J14" s="18">
+        <v>1</v>
+      </c>
+      <c r="K14" s="18"/>
+      <c r="L14" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="M14" s="28"/>
-      <c r="N14" s="20">
+      <c r="M14" s="24"/>
+      <c r="N14" s="18">
         <v>3</v>
       </c>
-      <c r="O14" s="20">
+      <c r="O14" s="18">
         <v>7</v>
       </c>
-      <c r="P14" s="20">
+      <c r="P14" s="18">
         <v>2</v>
       </c>
-      <c r="Q14" s="20">
+      <c r="Q14" s="18">
         <v>7</v>
       </c>
-      <c r="R14" s="20">
+      <c r="R14" s="18">
         <v>2</v>
       </c>
-      <c r="S14" s="20"/>
-      <c r="T14" s="21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C15" s="25" t="s">
+      <c r="S14" s="18"/>
+      <c r="T14" s="56">
+        <v>1</v>
+      </c>
+      <c r="V14" s="55" t="s">
+        <v>35</v>
+      </c>
+      <c r="W14" s="24">
+        <v>236</v>
+      </c>
+      <c r="X14" s="60">
+        <f>350-W14*1.2</f>
+        <v>66.800000000000011</v>
+      </c>
+      <c r="Y14" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z14" s="24">
+        <v>555</v>
+      </c>
+      <c r="AA14" s="63">
+        <f t="shared" si="0"/>
+        <v>834</v>
+      </c>
+    </row>
+    <row r="15" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C15" s="55" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="28">
+      <c r="D15" s="24">
         <v>5</v>
       </c>
-      <c r="E15" s="20"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="20">
-        <v>1</v>
-      </c>
-      <c r="H15" s="20">
-        <v>1</v>
-      </c>
-      <c r="I15" s="20"/>
-      <c r="J15" s="20">
+      <c r="E15" s="18"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="18">
+        <v>1</v>
+      </c>
+      <c r="H15" s="18">
+        <v>1</v>
+      </c>
+      <c r="I15" s="18"/>
+      <c r="J15" s="18">
         <v>4</v>
       </c>
-      <c r="K15" s="20"/>
-      <c r="L15" s="25" t="s">
+      <c r="K15" s="18"/>
+      <c r="L15" s="21" t="s">
         <v>249</v>
       </c>
-      <c r="M15" s="28">
+      <c r="M15" s="24">
         <v>3</v>
       </c>
-      <c r="N15" s="20">
+      <c r="N15" s="18">
         <v>3</v>
       </c>
-      <c r="O15" s="20">
+      <c r="O15" s="18">
         <v>8</v>
       </c>
-      <c r="P15" s="20"/>
-      <c r="Q15" s="20"/>
-      <c r="R15" s="20"/>
-      <c r="S15" s="20">
+      <c r="P15" s="18"/>
+      <c r="Q15" s="18"/>
+      <c r="R15" s="18"/>
+      <c r="S15" s="18">
         <v>6</v>
       </c>
-      <c r="T15" s="21">
+      <c r="T15" s="56">
         <v>2</v>
       </c>
-    </row>
-    <row r="16" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C16" s="25" t="s">
+      <c r="V15" s="55" t="s">
+        <v>32</v>
+      </c>
+      <c r="W15" s="24">
+        <v>458</v>
+      </c>
+      <c r="X15" s="60">
+        <f t="shared" si="1"/>
+        <v>300.39999999999998</v>
+      </c>
+      <c r="Y15" s="21" t="s">
+        <v>249</v>
+      </c>
+      <c r="Z15" s="24">
+        <v>549</v>
+      </c>
+      <c r="AA15" s="63">
+        <f t="shared" si="0"/>
+        <v>841.2</v>
+      </c>
+    </row>
+    <row r="16" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C16" s="55" t="s">
         <v>56</v>
       </c>
-      <c r="D16" s="28">
+      <c r="D16" s="24">
         <v>5</v>
       </c>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="20">
+      <c r="E16" s="18"/>
+      <c r="F16" s="18"/>
+      <c r="G16" s="18">
         <v>3</v>
       </c>
-      <c r="H16" s="20">
-        <v>1</v>
-      </c>
-      <c r="I16" s="20">
-        <v>1</v>
-      </c>
-      <c r="J16" s="20">
-        <v>1</v>
-      </c>
-      <c r="K16" s="20"/>
-      <c r="L16" s="25" t="s">
+      <c r="H16" s="18">
+        <v>1</v>
+      </c>
+      <c r="I16" s="18">
+        <v>1</v>
+      </c>
+      <c r="J16" s="18">
+        <v>1</v>
+      </c>
+      <c r="K16" s="18"/>
+      <c r="L16" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="M16" s="28">
+      <c r="M16" s="24">
         <v>6</v>
       </c>
-      <c r="N16" s="20"/>
-      <c r="O16" s="20">
+      <c r="N16" s="18"/>
+      <c r="O16" s="18">
         <v>3</v>
       </c>
-      <c r="P16" s="20"/>
-      <c r="Q16" s="20"/>
-      <c r="R16" s="20"/>
-      <c r="S16" s="20">
+      <c r="P16" s="18"/>
+      <c r="Q16" s="18"/>
+      <c r="R16" s="18"/>
+      <c r="S16" s="18">
         <v>8</v>
       </c>
-      <c r="T16" s="21">
+      <c r="T16" s="56">
         <v>5</v>
       </c>
-    </row>
-    <row r="17" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C17" s="25" t="s">
+      <c r="V16" s="55" t="s">
+        <v>56</v>
+      </c>
+      <c r="W16" s="24">
+        <v>499</v>
+      </c>
+      <c r="X16" s="60">
+        <f t="shared" si="1"/>
+        <v>251.20000000000005</v>
+      </c>
+      <c r="Y16" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="Z16" s="24">
+        <v>766</v>
+      </c>
+      <c r="AA16" s="63">
+        <f t="shared" si="0"/>
+        <v>580.80000000000007</v>
+      </c>
+    </row>
+    <row r="17" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C17" s="55" t="s">
         <v>36</v>
       </c>
-      <c r="D17" s="28">
+      <c r="D17" s="24">
         <v>4</v>
       </c>
-      <c r="E17" s="20">
-        <v>1</v>
-      </c>
-      <c r="F17" s="20">
-        <v>1</v>
-      </c>
-      <c r="G17" s="20">
-        <v>1</v>
-      </c>
-      <c r="H17" s="20">
-        <v>1</v>
-      </c>
-      <c r="I17" s="20">
-        <v>1</v>
-      </c>
-      <c r="J17" s="20">
-        <v>1</v>
-      </c>
-      <c r="K17" s="20">
-        <v>1</v>
-      </c>
-      <c r="L17" s="25" t="s">
+      <c r="E17" s="18">
+        <v>1</v>
+      </c>
+      <c r="F17" s="18">
+        <v>1</v>
+      </c>
+      <c r="G17" s="18">
+        <v>1</v>
+      </c>
+      <c r="H17" s="18">
+        <v>1</v>
+      </c>
+      <c r="I17" s="18">
+        <v>1</v>
+      </c>
+      <c r="J17" s="18">
+        <v>1</v>
+      </c>
+      <c r="K17" s="18">
+        <v>1</v>
+      </c>
+      <c r="L17" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="M17" s="28">
+      <c r="M17" s="24">
         <v>8</v>
       </c>
-      <c r="N17" s="20"/>
-      <c r="O17" s="20"/>
-      <c r="P17" s="20">
+      <c r="N17" s="18"/>
+      <c r="O17" s="18"/>
+      <c r="P17" s="18">
         <v>5</v>
       </c>
-      <c r="Q17" s="20">
+      <c r="Q17" s="18">
         <v>2</v>
       </c>
-      <c r="R17" s="20"/>
-      <c r="S17" s="20">
+      <c r="R17" s="18"/>
+      <c r="S17" s="18">
         <v>7</v>
       </c>
-      <c r="T17" s="21"/>
-    </row>
-    <row r="18" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C18" s="25" t="s">
+      <c r="T17" s="56"/>
+      <c r="V17" s="55" t="s">
+        <v>36</v>
+      </c>
+      <c r="W17" s="24">
+        <v>415</v>
+      </c>
+      <c r="X17" s="60">
+        <f t="shared" si="1"/>
+        <v>352</v>
+      </c>
+      <c r="Y17" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z17" s="24">
+        <v>857</v>
+      </c>
+      <c r="AA17" s="63">
+        <f t="shared" si="0"/>
+        <v>471.60000000000014</v>
+      </c>
+    </row>
+    <row r="18" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C18" s="55" t="s">
         <v>33</v>
       </c>
-      <c r="D18" s="28">
+      <c r="D18" s="24">
         <v>2</v>
       </c>
-      <c r="E18" s="20"/>
-      <c r="F18" s="20"/>
-      <c r="G18" s="20">
-        <v>1</v>
-      </c>
-      <c r="H18" s="20"/>
-      <c r="I18" s="20">
-        <v>1</v>
-      </c>
-      <c r="J18" s="20">
-        <v>1</v>
-      </c>
-      <c r="K18" s="20"/>
-      <c r="L18" s="25" t="s">
+      <c r="E18" s="18"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="18">
+        <v>1</v>
+      </c>
+      <c r="H18" s="18"/>
+      <c r="I18" s="18">
+        <v>1</v>
+      </c>
+      <c r="J18" s="18">
+        <v>1</v>
+      </c>
+      <c r="K18" s="18"/>
+      <c r="L18" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="M18" s="28">
+      <c r="M18" s="24">
         <v>8</v>
       </c>
-      <c r="N18" s="20"/>
-      <c r="O18" s="20"/>
-      <c r="P18" s="20">
+      <c r="N18" s="18"/>
+      <c r="O18" s="18"/>
+      <c r="P18" s="18">
         <v>6</v>
       </c>
-      <c r="Q18" s="20">
+      <c r="Q18" s="18">
         <v>5</v>
       </c>
-      <c r="R18" s="20">
+      <c r="R18" s="18">
         <v>2</v>
       </c>
-      <c r="S18" s="20">
-        <v>1</v>
-      </c>
-      <c r="T18" s="21"/>
-    </row>
-    <row r="19" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C19" s="25" t="s">
+      <c r="S18" s="18">
+        <v>1</v>
+      </c>
+      <c r="T18" s="56"/>
+      <c r="V18" s="55" t="s">
+        <v>33</v>
+      </c>
+      <c r="W18" s="24">
+        <v>252</v>
+      </c>
+      <c r="X18" s="60">
+        <f>350-W18*1.2</f>
+        <v>47.600000000000023</v>
+      </c>
+      <c r="Y18" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="Z18" s="24">
+        <v>915</v>
+      </c>
+      <c r="AA18" s="63">
+        <f t="shared" si="0"/>
+        <v>402</v>
+      </c>
+    </row>
+    <row r="19" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C19" s="55" t="s">
         <v>62</v>
       </c>
-      <c r="D19" s="28">
+      <c r="D19" s="24">
         <v>4</v>
       </c>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20">
-        <v>1</v>
-      </c>
-      <c r="G19" s="20">
+      <c r="E19" s="18"/>
+      <c r="F19" s="18">
+        <v>1</v>
+      </c>
+      <c r="G19" s="18">
         <v>2</v>
       </c>
-      <c r="H19" s="20"/>
-      <c r="I19" s="20">
+      <c r="H19" s="18"/>
+      <c r="I19" s="18">
         <v>2</v>
       </c>
-      <c r="J19" s="20">
+      <c r="J19" s="18">
         <v>2</v>
       </c>
-      <c r="K19" s="20"/>
-      <c r="L19" s="25" t="s">
+      <c r="K19" s="18"/>
+      <c r="L19" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="M19" s="28">
+      <c r="M19" s="24">
         <v>8</v>
       </c>
-      <c r="N19" s="20">
+      <c r="N19" s="18">
         <v>3</v>
       </c>
-      <c r="O19" s="20">
-        <v>1</v>
-      </c>
-      <c r="P19" s="20">
-        <v>1</v>
-      </c>
-      <c r="Q19" s="20">
-        <v>1</v>
-      </c>
-      <c r="R19" s="20">
+      <c r="O19" s="18">
+        <v>1</v>
+      </c>
+      <c r="P19" s="18">
+        <v>1</v>
+      </c>
+      <c r="Q19" s="18">
+        <v>1</v>
+      </c>
+      <c r="R19" s="18">
         <v>2</v>
       </c>
-      <c r="S19" s="20">
-        <v>1</v>
-      </c>
-      <c r="T19" s="21">
+      <c r="S19" s="18">
+        <v>1</v>
+      </c>
+      <c r="T19" s="56">
         <v>5</v>
       </c>
-    </row>
-    <row r="20" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C20" s="25" t="s">
+      <c r="V19" s="55" t="s">
+        <v>62</v>
+      </c>
+      <c r="W19" s="24">
+        <v>555</v>
+      </c>
+      <c r="X19" s="60">
+        <f t="shared" si="1"/>
+        <v>184</v>
+      </c>
+      <c r="Y19" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="Z19" s="24">
+        <v>820</v>
+      </c>
+      <c r="AA19" s="63">
+        <f t="shared" si="0"/>
+        <v>516</v>
+      </c>
+    </row>
+    <row r="20" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C20" s="55" t="s">
         <v>38</v>
       </c>
-      <c r="D20" s="28">
-        <v>1</v>
-      </c>
-      <c r="E20" s="20">
-        <v>1</v>
-      </c>
-      <c r="F20" s="20">
-        <v>1</v>
-      </c>
-      <c r="G20" s="20">
+      <c r="D20" s="24">
+        <v>1</v>
+      </c>
+      <c r="E20" s="18">
+        <v>1</v>
+      </c>
+      <c r="F20" s="18">
+        <v>1</v>
+      </c>
+      <c r="G20" s="18">
         <v>2</v>
       </c>
-      <c r="H20" s="20"/>
-      <c r="I20" s="20"/>
-      <c r="J20" s="20"/>
-      <c r="K20" s="20"/>
-      <c r="L20" s="25" t="s">
+      <c r="H20" s="18"/>
+      <c r="I20" s="18"/>
+      <c r="J20" s="18"/>
+      <c r="K20" s="18"/>
+      <c r="L20" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="M20" s="28">
+      <c r="M20" s="24">
         <v>8</v>
       </c>
-      <c r="N20" s="20"/>
-      <c r="O20" s="20">
-        <v>1</v>
-      </c>
-      <c r="P20" s="20">
+      <c r="N20" s="18"/>
+      <c r="O20" s="18">
+        <v>1</v>
+      </c>
+      <c r="P20" s="18">
         <v>3</v>
       </c>
-      <c r="Q20" s="20"/>
-      <c r="R20" s="20">
+      <c r="Q20" s="18"/>
+      <c r="R20" s="18">
         <v>5</v>
       </c>
-      <c r="S20" s="20">
+      <c r="S20" s="18">
         <v>5</v>
       </c>
-      <c r="T20" s="21"/>
-    </row>
-    <row r="21" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C21" s="25" t="s">
+      <c r="T20" s="56"/>
+      <c r="V20" s="55" t="s">
+        <v>38</v>
+      </c>
+      <c r="W20" s="24">
+        <v>225</v>
+      </c>
+      <c r="X20" s="60">
+        <f>350-W20*1.2</f>
+        <v>80</v>
+      </c>
+      <c r="Y20" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z20" s="24">
+        <v>990</v>
+      </c>
+      <c r="AA20" s="63">
+        <f t="shared" si="0"/>
+        <v>312</v>
+      </c>
+    </row>
+    <row r="21" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C21" s="55" t="s">
         <v>39</v>
       </c>
-      <c r="D21" s="28">
+      <c r="D21" s="24">
         <v>2</v>
       </c>
-      <c r="E21" s="20">
-        <v>1</v>
-      </c>
-      <c r="F21" s="20">
+      <c r="E21" s="18">
+        <v>1</v>
+      </c>
+      <c r="F21" s="18">
         <v>2</v>
       </c>
-      <c r="G21" s="20">
+      <c r="G21" s="18">
         <v>4</v>
       </c>
-      <c r="H21" s="20">
-        <v>1</v>
-      </c>
-      <c r="I21" s="20">
-        <v>1</v>
-      </c>
-      <c r="J21" s="20"/>
-      <c r="K21" s="20"/>
-      <c r="L21" s="25" t="s">
+      <c r="H21" s="18">
+        <v>1</v>
+      </c>
+      <c r="I21" s="18">
+        <v>1</v>
+      </c>
+      <c r="J21" s="18"/>
+      <c r="K21" s="18"/>
+      <c r="L21" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="M21" s="28">
+      <c r="M21" s="24">
         <v>3</v>
       </c>
-      <c r="N21" s="20">
-        <v>1</v>
-      </c>
-      <c r="O21" s="20">
+      <c r="N21" s="18">
+        <v>1</v>
+      </c>
+      <c r="O21" s="18">
         <v>2</v>
       </c>
-      <c r="P21" s="20">
+      <c r="P21" s="18">
         <v>8</v>
       </c>
-      <c r="Q21" s="20">
+      <c r="Q21" s="18">
         <v>4</v>
       </c>
-      <c r="R21" s="20">
+      <c r="R21" s="18">
         <v>4</v>
       </c>
-      <c r="S21" s="20"/>
-      <c r="T21" s="21"/>
-    </row>
-    <row r="22" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C22" s="25" t="s">
+      <c r="S21" s="18"/>
+      <c r="T21" s="56"/>
+      <c r="V21" s="55" t="s">
+        <v>39</v>
+      </c>
+      <c r="W21" s="24">
+        <v>484</v>
+      </c>
+      <c r="X21" s="60">
+        <f t="shared" si="1"/>
+        <v>269.20000000000005</v>
+      </c>
+      <c r="Y21" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="Z21" s="24">
+        <v>943</v>
+      </c>
+      <c r="AA21" s="63">
+        <f t="shared" si="0"/>
+        <v>368.40000000000009</v>
+      </c>
+    </row>
+    <row r="22" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C22" s="55" t="s">
         <v>40</v>
       </c>
-      <c r="D22" s="28">
+      <c r="D22" s="24">
         <v>2</v>
       </c>
-      <c r="E22" s="20">
+      <c r="E22" s="18">
         <v>2</v>
       </c>
-      <c r="F22" s="20">
-        <v>1</v>
-      </c>
-      <c r="G22" s="20">
+      <c r="F22" s="18">
+        <v>1</v>
+      </c>
+      <c r="G22" s="18">
         <v>2</v>
       </c>
-      <c r="H22" s="20"/>
-      <c r="I22" s="20">
+      <c r="H22" s="18"/>
+      <c r="I22" s="18">
         <v>4</v>
       </c>
-      <c r="J22" s="20"/>
-      <c r="K22" s="20"/>
-      <c r="L22" s="25" t="s">
+      <c r="J22" s="18"/>
+      <c r="K22" s="18"/>
+      <c r="L22" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="M22" s="28">
+      <c r="M22" s="24">
         <v>2</v>
       </c>
-      <c r="N22" s="20">
+      <c r="N22" s="18">
         <v>2</v>
       </c>
-      <c r="O22" s="20">
+      <c r="O22" s="18">
         <v>2</v>
       </c>
-      <c r="P22" s="20">
+      <c r="P22" s="18">
         <v>4</v>
       </c>
-      <c r="Q22" s="20">
+      <c r="Q22" s="18">
         <v>8</v>
       </c>
-      <c r="R22" s="20">
+      <c r="R22" s="18">
         <v>4</v>
       </c>
-      <c r="S22" s="20"/>
-      <c r="T22" s="21"/>
-    </row>
-    <row r="23" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C23" s="25" t="s">
+      <c r="S22" s="18"/>
+      <c r="T22" s="56"/>
+      <c r="V22" s="55" t="s">
+        <v>40</v>
+      </c>
+      <c r="W22" s="24">
+        <v>467</v>
+      </c>
+      <c r="X22" s="60">
+        <f t="shared" si="1"/>
+        <v>289.60000000000002</v>
+      </c>
+      <c r="Y22" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="Z22" s="24">
+        <v>901</v>
+      </c>
+      <c r="AA22" s="63">
+        <f t="shared" si="0"/>
+        <v>418.79999999999995</v>
+      </c>
+    </row>
+    <row r="23" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C23" s="55" t="s">
         <v>23</v>
       </c>
-      <c r="D23" s="28"/>
-      <c r="E23" s="20"/>
-      <c r="F23" s="20">
+      <c r="D23" s="24"/>
+      <c r="E23" s="18"/>
+      <c r="F23" s="18">
         <v>2</v>
       </c>
-      <c r="G23" s="20"/>
-      <c r="H23" s="20"/>
-      <c r="I23" s="20">
+      <c r="G23" s="18"/>
+      <c r="H23" s="18"/>
+      <c r="I23" s="18">
         <v>2</v>
       </c>
-      <c r="J23" s="20"/>
-      <c r="K23" s="20">
-        <v>1</v>
-      </c>
-      <c r="L23" s="25" t="s">
+      <c r="J23" s="18"/>
+      <c r="K23" s="18">
+        <v>1</v>
+      </c>
+      <c r="L23" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="M23" s="28">
+      <c r="M23" s="24">
         <v>2</v>
       </c>
-      <c r="N23" s="20">
+      <c r="N23" s="18">
         <v>2</v>
       </c>
-      <c r="O23" s="20">
-        <v>1</v>
-      </c>
-      <c r="P23" s="20">
+      <c r="O23" s="18">
+        <v>1</v>
+      </c>
+      <c r="P23" s="18">
         <v>4</v>
       </c>
-      <c r="Q23" s="20">
+      <c r="Q23" s="18">
         <v>4</v>
       </c>
-      <c r="R23" s="20">
+      <c r="R23" s="18">
         <v>8</v>
       </c>
-      <c r="S23" s="20"/>
-      <c r="T23" s="21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C24" s="25" t="s">
+      <c r="S23" s="18"/>
+      <c r="T23" s="56">
+        <v>1</v>
+      </c>
+      <c r="V23" s="55" t="s">
+        <v>23</v>
+      </c>
+      <c r="W23" s="24">
+        <v>128</v>
+      </c>
+      <c r="X23" s="60">
+        <f>350-W23*1.2</f>
+        <v>196.4</v>
+      </c>
+      <c r="Y23" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z23" s="24">
+        <v>828</v>
+      </c>
+      <c r="AA23" s="63">
+        <f t="shared" si="0"/>
+        <v>506.40000000000009</v>
+      </c>
+    </row>
+    <row r="24" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C24" s="55" t="s">
         <v>42</v>
       </c>
-      <c r="D24" s="28"/>
-      <c r="E24" s="20"/>
-      <c r="F24" s="20">
+      <c r="D24" s="24"/>
+      <c r="E24" s="18"/>
+      <c r="F24" s="18">
         <v>4</v>
       </c>
-      <c r="G24" s="20"/>
-      <c r="H24" s="20"/>
-      <c r="I24" s="20">
+      <c r="G24" s="18"/>
+      <c r="H24" s="18"/>
+      <c r="I24" s="18">
         <v>3</v>
       </c>
-      <c r="J24" s="20"/>
-      <c r="K24" s="20">
+      <c r="J24" s="18"/>
+      <c r="K24" s="18">
         <v>4</v>
       </c>
-      <c r="L24" s="25" t="s">
+      <c r="L24" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="M24" s="28">
+      <c r="M24" s="24">
         <v>3</v>
       </c>
-      <c r="N24" s="20">
+      <c r="N24" s="18">
         <v>4</v>
       </c>
-      <c r="O24" s="20">
+      <c r="O24" s="18">
         <v>3</v>
       </c>
-      <c r="P24" s="20">
+      <c r="P24" s="18">
         <v>7</v>
       </c>
-      <c r="Q24" s="20"/>
-      <c r="R24" s="20">
+      <c r="Q24" s="18"/>
+      <c r="R24" s="18">
         <v>5</v>
       </c>
-      <c r="S24" s="20"/>
-      <c r="T24" s="21"/>
-    </row>
-    <row r="25" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C25" s="25" t="s">
+      <c r="S24" s="18"/>
+      <c r="T24" s="56"/>
+      <c r="V24" s="55" t="s">
+        <v>42</v>
+      </c>
+      <c r="W24" s="24">
+        <v>340</v>
+      </c>
+      <c r="X24" s="60">
+        <f t="shared" si="1"/>
+        <v>442</v>
+      </c>
+      <c r="Y24" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="Z24" s="24">
+        <v>792</v>
+      </c>
+      <c r="AA24" s="63">
+        <f t="shared" si="0"/>
+        <v>549.6</v>
+      </c>
+    </row>
+    <row r="25" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C25" s="55" t="s">
         <v>45</v>
       </c>
-      <c r="D25" s="28"/>
-      <c r="E25" s="20"/>
-      <c r="F25" s="20">
+      <c r="D25" s="24"/>
+      <c r="E25" s="18"/>
+      <c r="F25" s="18">
         <v>4</v>
       </c>
-      <c r="G25" s="20"/>
-      <c r="H25" s="20">
-        <v>1</v>
-      </c>
-      <c r="I25" s="20">
+      <c r="G25" s="18"/>
+      <c r="H25" s="18">
+        <v>1</v>
+      </c>
+      <c r="I25" s="18">
         <v>5</v>
       </c>
-      <c r="J25" s="20"/>
-      <c r="K25" s="20">
-        <v>1</v>
-      </c>
-      <c r="L25" s="25" t="s">
+      <c r="J25" s="18"/>
+      <c r="K25" s="18">
+        <v>1</v>
+      </c>
+      <c r="L25" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="M25" s="28"/>
-      <c r="N25" s="20">
+      <c r="M25" s="24"/>
+      <c r="N25" s="18">
         <v>5</v>
       </c>
-      <c r="O25" s="20">
+      <c r="O25" s="18">
         <v>5</v>
       </c>
-      <c r="P25" s="20"/>
-      <c r="Q25" s="20"/>
-      <c r="R25" s="20">
+      <c r="P25" s="18"/>
+      <c r="Q25" s="18"/>
+      <c r="R25" s="18">
         <v>7</v>
       </c>
-      <c r="S25" s="20">
-        <v>1</v>
-      </c>
-      <c r="T25" s="21">
+      <c r="S25" s="18">
+        <v>1</v>
+      </c>
+      <c r="T25" s="56">
         <v>4</v>
       </c>
-    </row>
-    <row r="26" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C26" s="25" t="s">
+      <c r="V25" s="55" t="s">
+        <v>45</v>
+      </c>
+      <c r="W25" s="24">
+        <v>301</v>
+      </c>
+      <c r="X25" s="60">
+        <f t="shared" si="1"/>
+        <v>488.8</v>
+      </c>
+      <c r="Y25" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="Z25" s="24">
+        <v>444</v>
+      </c>
+      <c r="AA25" s="63">
+        <f t="shared" si="0"/>
+        <v>967.2</v>
+      </c>
+    </row>
+    <row r="26" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C26" s="55" t="s">
         <v>52</v>
       </c>
-      <c r="D26" s="28">
+      <c r="D26" s="24">
         <v>2</v>
       </c>
-      <c r="E26" s="20"/>
-      <c r="F26" s="20"/>
-      <c r="G26" s="20">
+      <c r="E26" s="18"/>
+      <c r="F26" s="18"/>
+      <c r="G26" s="18">
         <v>2</v>
       </c>
-      <c r="H26" s="20">
-        <v>1</v>
-      </c>
-      <c r="I26" s="20"/>
-      <c r="J26" s="20"/>
-      <c r="K26" s="20"/>
-      <c r="L26" s="25" t="s">
+      <c r="H26" s="18">
+        <v>1</v>
+      </c>
+      <c r="I26" s="18"/>
+      <c r="J26" s="18"/>
+      <c r="K26" s="18"/>
+      <c r="L26" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="M26" s="28"/>
-      <c r="N26" s="20"/>
-      <c r="O26" s="20">
+      <c r="M26" s="24"/>
+      <c r="N26" s="18"/>
+      <c r="O26" s="18">
         <v>7</v>
       </c>
-      <c r="P26" s="20"/>
-      <c r="Q26" s="20"/>
-      <c r="R26" s="20">
+      <c r="P26" s="18"/>
+      <c r="Q26" s="18"/>
+      <c r="R26" s="18">
         <v>3</v>
       </c>
-      <c r="S26" s="20"/>
-      <c r="T26" s="21">
+      <c r="S26" s="18"/>
+      <c r="T26" s="56">
         <v>4</v>
       </c>
-    </row>
-    <row r="27" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C27" s="25" t="s">
+      <c r="V26" s="55" t="s">
+        <v>52</v>
+      </c>
+      <c r="W26" s="24">
+        <v>170</v>
+      </c>
+      <c r="X26" s="60">
+        <f>350-W26*1.2</f>
+        <v>146</v>
+      </c>
+      <c r="Y26" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z26" s="24">
+        <v>546</v>
+      </c>
+      <c r="AA26" s="63">
+        <f t="shared" si="0"/>
+        <v>844.80000000000007</v>
+      </c>
+    </row>
+    <row r="27" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C27" s="55" t="s">
         <v>53</v>
       </c>
-      <c r="D27" s="28">
+      <c r="D27" s="24">
         <v>3</v>
       </c>
-      <c r="E27" s="20"/>
-      <c r="F27" s="20"/>
-      <c r="G27" s="20">
+      <c r="E27" s="18"/>
+      <c r="F27" s="18"/>
+      <c r="G27" s="18">
         <v>5</v>
       </c>
-      <c r="H27" s="20">
+      <c r="H27" s="18">
         <v>3</v>
       </c>
-      <c r="I27" s="20"/>
-      <c r="J27" s="20"/>
-      <c r="K27" s="20"/>
-      <c r="L27" s="25" t="s">
+      <c r="I27" s="18"/>
+      <c r="J27" s="18"/>
+      <c r="K27" s="18"/>
+      <c r="L27" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="M27" s="28"/>
-      <c r="N27" s="20"/>
-      <c r="O27" s="20">
+      <c r="M27" s="24"/>
+      <c r="N27" s="18"/>
+      <c r="O27" s="18">
         <v>5</v>
       </c>
-      <c r="P27" s="20">
+      <c r="P27" s="18">
         <v>2</v>
       </c>
-      <c r="Q27" s="20">
-        <v>1</v>
-      </c>
-      <c r="R27" s="20">
+      <c r="Q27" s="18">
+        <v>1</v>
+      </c>
+      <c r="R27" s="18">
         <v>8</v>
       </c>
-      <c r="S27" s="20"/>
-      <c r="T27" s="21">
+      <c r="S27" s="18"/>
+      <c r="T27" s="56">
         <v>6</v>
       </c>
-    </row>
-    <row r="28" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C28" s="25" t="s">
+      <c r="V27" s="55" t="s">
+        <v>53</v>
+      </c>
+      <c r="W27" s="24">
+        <v>404</v>
+      </c>
+      <c r="X27" s="60">
+        <f t="shared" si="1"/>
+        <v>365.20000000000005</v>
+      </c>
+      <c r="Y27" s="21" t="s">
+        <v>46</v>
+      </c>
+      <c r="Z27" s="24">
+        <v>471</v>
+      </c>
+      <c r="AA27" s="63">
+        <f t="shared" si="0"/>
+        <v>934.80000000000007</v>
+      </c>
+    </row>
+    <row r="28" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C28" s="55" t="s">
         <v>60</v>
       </c>
-      <c r="D28" s="28"/>
-      <c r="E28" s="20"/>
-      <c r="F28" s="20"/>
-      <c r="G28" s="20">
-        <v>1</v>
-      </c>
-      <c r="H28" s="20">
-        <v>1</v>
-      </c>
-      <c r="I28" s="20">
-        <v>1</v>
-      </c>
-      <c r="J28" s="20"/>
-      <c r="K28" s="20">
+      <c r="D28" s="24"/>
+      <c r="E28" s="18"/>
+      <c r="F28" s="18"/>
+      <c r="G28" s="18">
+        <v>1</v>
+      </c>
+      <c r="H28" s="18">
+        <v>1</v>
+      </c>
+      <c r="I28" s="18">
+        <v>1</v>
+      </c>
+      <c r="J28" s="18"/>
+      <c r="K28" s="18">
         <v>2</v>
       </c>
-      <c r="L28" s="25" t="s">
+      <c r="L28" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="M28" s="28"/>
-      <c r="N28" s="20"/>
-      <c r="O28" s="20">
+      <c r="M28" s="24"/>
+      <c r="N28" s="18"/>
+      <c r="O28" s="18">
         <v>4</v>
       </c>
-      <c r="P28" s="20"/>
-      <c r="Q28" s="20">
+      <c r="P28" s="18"/>
+      <c r="Q28" s="18">
         <v>7</v>
       </c>
-      <c r="R28" s="20">
+      <c r="R28" s="18">
         <v>8</v>
       </c>
-      <c r="S28" s="20">
+      <c r="S28" s="18">
         <v>2</v>
       </c>
-      <c r="T28" s="21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C29" s="25" t="s">
+      <c r="T28" s="56">
+        <v>1</v>
+      </c>
+      <c r="V28" s="55" t="s">
+        <v>60</v>
+      </c>
+      <c r="W28" s="24">
+        <v>164</v>
+      </c>
+      <c r="X28" s="60">
+        <f>350-W28*1.2</f>
+        <v>153.20000000000002</v>
+      </c>
+      <c r="Y28" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z28" s="24">
+        <v>430</v>
+      </c>
+      <c r="AA28" s="63">
+        <f t="shared" si="0"/>
+        <v>984</v>
+      </c>
+    </row>
+    <row r="29" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C29" s="55" t="s">
         <v>63</v>
       </c>
-      <c r="D29" s="28"/>
-      <c r="E29" s="20"/>
-      <c r="F29" s="20">
+      <c r="D29" s="24"/>
+      <c r="E29" s="18"/>
+      <c r="F29" s="18">
         <v>2</v>
       </c>
-      <c r="G29" s="20">
-        <v>1</v>
-      </c>
-      <c r="H29" s="20">
+      <c r="G29" s="18">
+        <v>1</v>
+      </c>
+      <c r="H29" s="18">
         <v>4</v>
       </c>
-      <c r="I29" s="20">
+      <c r="I29" s="18">
         <v>2</v>
       </c>
-      <c r="J29" s="20"/>
-      <c r="K29" s="20">
+      <c r="J29" s="18"/>
+      <c r="K29" s="18">
         <v>2</v>
       </c>
-      <c r="L29" s="25" t="s">
+      <c r="L29" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="M29" s="28">
+      <c r="M29" s="24">
         <v>5</v>
       </c>
-      <c r="N29" s="20">
+      <c r="N29" s="18">
         <v>3</v>
       </c>
-      <c r="O29" s="20"/>
-      <c r="P29" s="20">
+      <c r="O29" s="18"/>
+      <c r="P29" s="18">
         <v>8</v>
       </c>
-      <c r="Q29" s="20">
+      <c r="Q29" s="18">
         <v>6</v>
       </c>
-      <c r="R29" s="20"/>
-      <c r="S29" s="20"/>
-      <c r="T29" s="21"/>
-    </row>
-    <row r="30" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C30" s="25" t="s">
+      <c r="R29" s="18"/>
+      <c r="S29" s="18"/>
+      <c r="T29" s="56"/>
+      <c r="V29" s="55" t="s">
+        <v>63</v>
+      </c>
+      <c r="W29" s="24">
+        <v>399</v>
+      </c>
+      <c r="X29" s="60">
+        <f t="shared" si="1"/>
+        <v>371.20000000000005</v>
+      </c>
+      <c r="Y29" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="Z29" s="24">
+        <v>808</v>
+      </c>
+      <c r="AA29" s="63">
+        <f t="shared" si="0"/>
+        <v>530.40000000000009</v>
+      </c>
+    </row>
+    <row r="30" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C30" s="55" t="s">
         <v>65</v>
       </c>
-      <c r="D30" s="28"/>
-      <c r="E30" s="20"/>
-      <c r="F30" s="20"/>
-      <c r="G30" s="20">
-        <v>1</v>
-      </c>
-      <c r="H30" s="20">
-        <v>1</v>
-      </c>
-      <c r="I30" s="20">
-        <v>1</v>
-      </c>
-      <c r="J30" s="20">
+      <c r="D30" s="24"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="18"/>
+      <c r="G30" s="18">
+        <v>1</v>
+      </c>
+      <c r="H30" s="18">
+        <v>1</v>
+      </c>
+      <c r="I30" s="18">
+        <v>1</v>
+      </c>
+      <c r="J30" s="18">
         <v>3</v>
       </c>
-      <c r="K30" s="20">
+      <c r="K30" s="18">
         <v>5</v>
       </c>
-      <c r="L30" s="25" t="s">
+      <c r="L30" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="M30" s="28"/>
-      <c r="N30" s="20"/>
-      <c r="O30" s="20">
+      <c r="M30" s="24"/>
+      <c r="N30" s="18"/>
+      <c r="O30" s="18">
         <v>6</v>
       </c>
-      <c r="P30" s="20">
-        <v>1</v>
-      </c>
-      <c r="Q30" s="20">
+      <c r="P30" s="18">
+        <v>1</v>
+      </c>
+      <c r="Q30" s="18">
         <v>4</v>
       </c>
-      <c r="R30" s="20">
+      <c r="R30" s="18">
         <v>6</v>
       </c>
-      <c r="S30" s="20"/>
-      <c r="T30" s="21">
+      <c r="S30" s="18"/>
+      <c r="T30" s="56">
         <v>5</v>
       </c>
-    </row>
-    <row r="31" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C31" s="25" t="s">
+      <c r="V30" s="55" t="s">
+        <v>65</v>
+      </c>
+      <c r="W30" s="24">
+        <v>415</v>
+      </c>
+      <c r="X30" s="60">
+        <f t="shared" si="1"/>
+        <v>352</v>
+      </c>
+      <c r="Y30" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="Z30" s="24">
+        <v>666</v>
+      </c>
+      <c r="AA30" s="63">
+        <f t="shared" si="0"/>
+        <v>700.80000000000007</v>
+      </c>
+    </row>
+    <row r="31" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C31" s="55" t="s">
         <v>64</v>
       </c>
-      <c r="D31" s="28">
-        <v>1</v>
-      </c>
-      <c r="E31" s="20">
-        <v>1</v>
-      </c>
-      <c r="F31" s="20"/>
-      <c r="G31" s="20"/>
-      <c r="H31" s="20">
+      <c r="D31" s="24">
+        <v>1</v>
+      </c>
+      <c r="E31" s="18">
+        <v>1</v>
+      </c>
+      <c r="F31" s="18"/>
+      <c r="G31" s="18"/>
+      <c r="H31" s="18">
         <v>2</v>
       </c>
-      <c r="I31" s="20"/>
-      <c r="J31" s="20">
-        <v>1</v>
-      </c>
-      <c r="K31" s="20"/>
-      <c r="L31" s="25" t="s">
+      <c r="I31" s="18"/>
+      <c r="J31" s="18">
+        <v>1</v>
+      </c>
+      <c r="K31" s="18"/>
+      <c r="L31" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="M31" s="28"/>
-      <c r="N31" s="20"/>
-      <c r="O31" s="20">
+      <c r="M31" s="24"/>
+      <c r="N31" s="18"/>
+      <c r="O31" s="18">
         <v>2</v>
       </c>
-      <c r="P31" s="20">
+      <c r="P31" s="18">
         <v>4</v>
       </c>
-      <c r="Q31" s="20">
+      <c r="Q31" s="18">
         <v>6</v>
       </c>
-      <c r="R31" s="20">
+      <c r="R31" s="18">
         <v>4</v>
       </c>
-      <c r="S31" s="20">
+      <c r="S31" s="18">
         <v>4</v>
       </c>
-      <c r="T31" s="21">
+      <c r="T31" s="56">
         <v>2</v>
       </c>
-    </row>
-    <row r="32" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C32" s="25" t="s">
+      <c r="V31" s="55" t="s">
+        <v>64</v>
+      </c>
+      <c r="W31" s="24">
+        <v>210</v>
+      </c>
+      <c r="X31" s="60">
+        <f>350-W31*1.2</f>
+        <v>98</v>
+      </c>
+      <c r="Y31" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="Z31" s="24">
+        <v>691</v>
+      </c>
+      <c r="AA31" s="63">
+        <f t="shared" si="0"/>
+        <v>670.80000000000007</v>
+      </c>
+    </row>
+    <row r="32" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C32" s="55" t="s">
         <v>59</v>
       </c>
-      <c r="D32" s="28">
+      <c r="D32" s="24">
         <v>2</v>
       </c>
-      <c r="E32" s="20">
+      <c r="E32" s="18">
         <v>2</v>
       </c>
-      <c r="F32" s="20"/>
-      <c r="G32" s="20"/>
-      <c r="H32" s="20">
+      <c r="F32" s="18"/>
+      <c r="G32" s="18"/>
+      <c r="H32" s="18">
         <v>5</v>
       </c>
-      <c r="I32" s="20"/>
-      <c r="J32" s="20">
+      <c r="I32" s="18"/>
+      <c r="J32" s="18">
         <v>2</v>
       </c>
-      <c r="K32" s="20"/>
-      <c r="L32" s="25" t="s">
+      <c r="K32" s="18"/>
+      <c r="L32" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="M32" s="28">
+      <c r="M32" s="24">
         <v>2</v>
       </c>
-      <c r="N32" s="20"/>
-      <c r="O32" s="20"/>
-      <c r="P32" s="20">
+      <c r="N32" s="18"/>
+      <c r="O32" s="18"/>
+      <c r="P32" s="18">
         <v>3</v>
       </c>
-      <c r="Q32" s="20">
+      <c r="Q32" s="18">
         <v>3</v>
       </c>
-      <c r="R32" s="20">
+      <c r="R32" s="18">
         <v>3</v>
       </c>
-      <c r="S32" s="20">
+      <c r="S32" s="18">
         <v>3</v>
       </c>
-      <c r="T32" s="21">
+      <c r="T32" s="56">
         <v>8</v>
       </c>
-    </row>
-    <row r="33" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="L33" s="25" t="s">
+      <c r="V32" s="55" t="s">
+        <v>59</v>
+      </c>
+      <c r="W32" s="24">
+        <v>513</v>
+      </c>
+      <c r="X32" s="60">
+        <f>850-W32*1.2</f>
+        <v>234.39999999999998</v>
+      </c>
+      <c r="Y32" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="Z32" s="24">
+        <v>777</v>
+      </c>
+      <c r="AA32" s="63">
+        <f t="shared" si="0"/>
+        <v>567.6</v>
+      </c>
+    </row>
+    <row r="33" spans="3:27" x14ac:dyDescent="0.25">
+      <c r="C33" s="12"/>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
+      <c r="G33" s="5"/>
+      <c r="H33" s="5"/>
+      <c r="I33" s="5"/>
+      <c r="J33" s="5"/>
+      <c r="K33" s="5"/>
+      <c r="L33" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="M33" s="28">
+      <c r="M33" s="24">
         <v>4</v>
       </c>
-      <c r="N33" s="20">
+      <c r="N33" s="18">
         <v>7</v>
       </c>
-      <c r="O33" s="20"/>
-      <c r="P33" s="20">
-        <v>1</v>
-      </c>
-      <c r="Q33" s="20">
+      <c r="O33" s="18"/>
+      <c r="P33" s="18">
+        <v>1</v>
+      </c>
+      <c r="Q33" s="18">
         <v>8</v>
       </c>
-      <c r="R33" s="20"/>
-      <c r="S33" s="20">
+      <c r="R33" s="18"/>
+      <c r="S33" s="18">
         <v>2</v>
       </c>
-      <c r="T33" s="21"/>
-    </row>
-    <row r="34" spans="3:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C34" s="26"/>
-      <c r="D34" s="30"/>
-      <c r="E34" s="31"/>
-      <c r="F34" s="31"/>
-      <c r="G34" s="31"/>
-      <c r="H34" s="31"/>
-      <c r="I34" s="31"/>
-      <c r="J34" s="31"/>
-      <c r="K34" s="32"/>
-      <c r="L34" s="26" t="s">
+      <c r="T33" s="56"/>
+      <c r="V33" s="12"/>
+      <c r="W33" s="5"/>
+      <c r="X33" s="5"/>
+      <c r="Y33" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z33" s="24">
+        <v>643</v>
+      </c>
+      <c r="AA33" s="63">
+        <f t="shared" si="0"/>
+        <v>728.4</v>
+      </c>
+    </row>
+    <row r="34" spans="3:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C34" s="57"/>
+      <c r="D34" s="26"/>
+      <c r="E34" s="27"/>
+      <c r="F34" s="27"/>
+      <c r="G34" s="27"/>
+      <c r="H34" s="27"/>
+      <c r="I34" s="27"/>
+      <c r="J34" s="27"/>
+      <c r="K34" s="28"/>
+      <c r="L34" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="M34" s="29">
+      <c r="M34" s="25">
         <v>7</v>
       </c>
-      <c r="N34" s="22">
+      <c r="N34" s="19">
         <v>2</v>
       </c>
-      <c r="O34" s="22"/>
-      <c r="P34" s="22">
+      <c r="O34" s="19"/>
+      <c r="P34" s="19">
         <v>3</v>
       </c>
-      <c r="Q34" s="22">
+      <c r="Q34" s="19">
         <v>5</v>
       </c>
-      <c r="R34" s="22"/>
-      <c r="S34" s="22">
+      <c r="R34" s="19"/>
+      <c r="S34" s="19">
         <v>2</v>
       </c>
-      <c r="T34" s="23">
+      <c r="T34" s="58">
         <v>3</v>
       </c>
-    </row>
-    <row r="36" spans="3:20" x14ac:dyDescent="0.25">
+      <c r="V34" s="57"/>
+      <c r="W34" s="26"/>
+      <c r="X34" s="27"/>
+      <c r="Y34" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z34" s="25">
+        <v>689</v>
+      </c>
+      <c r="AA34" s="62">
+        <f>1500-Z34*1.2</f>
+        <v>673.2</v>
+      </c>
+    </row>
+    <row r="36" spans="3:27" x14ac:dyDescent="0.25">
       <c r="C36" t="s">
         <v>427</v>
       </c>
-    </row>
-    <row r="37" spans="3:20" x14ac:dyDescent="0.25">
+      <c r="V36" t="s">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="37" spans="3:27" x14ac:dyDescent="0.25">
       <c r="C37" t="s">
         <v>428</v>
       </c>
-    </row>
-    <row r="38" spans="3:20" x14ac:dyDescent="0.25">
+      <c r="V37" t="s">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="38" spans="3:27" x14ac:dyDescent="0.25">
       <c r="C38" t="s">
         <v>429</v>
+      </c>
+      <c r="V38" t="s">
+        <v>816</v>
       </c>
     </row>
   </sheetData>
@@ -8674,10 +9403,10 @@
   <sheetData>
     <row r="7" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B8" s="35" t="s">
+      <c r="B8" s="31" t="s">
         <v>666</v>
       </c>
-      <c r="C8" s="36" t="s">
+      <c r="C8" s="32" t="s">
         <v>665</v>
       </c>
       <c r="H8" t="s">
@@ -8695,7 +9424,7 @@
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B9" s="12"/>
-      <c r="C9" s="33"/>
+      <c r="C9" s="29"/>
       <c r="H9" t="s">
         <v>14</v>
       </c>
@@ -8713,7 +9442,7 @@
       <c r="B10" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="C10" s="33" t="s">
+      <c r="C10" s="29" t="s">
         <v>123</v>
       </c>
       <c r="H10" t="s">
@@ -8733,7 +9462,7 @@
       <c r="B11" s="12" t="s">
         <v>127</v>
       </c>
-      <c r="C11" s="33" t="s">
+      <c r="C11" s="29" t="s">
         <v>123</v>
       </c>
       <c r="H11" t="s">
@@ -8753,7 +9482,7 @@
       <c r="B12" s="12" t="s">
         <v>140</v>
       </c>
-      <c r="C12" s="33" t="s">
+      <c r="C12" s="29" t="s">
         <v>123</v>
       </c>
       <c r="H12" t="s">
@@ -8771,7 +9500,7 @@
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B13" s="12"/>
-      <c r="C13" s="33"/>
+      <c r="C13" s="29"/>
       <c r="H13" t="s">
         <v>25</v>
       </c>
@@ -8789,7 +9518,7 @@
       <c r="B14" s="12" t="s">
         <v>129</v>
       </c>
-      <c r="C14" s="33" t="s">
+      <c r="C14" s="29" t="s">
         <v>123</v>
       </c>
       <c r="H14" t="s">
@@ -8809,7 +9538,7 @@
       <c r="B15" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="C15" s="33" t="s">
+      <c r="C15" s="29" t="s">
         <v>123</v>
       </c>
       <c r="H15" t="s">
@@ -8829,7 +9558,7 @@
       <c r="B16" s="12" t="s">
         <v>156</v>
       </c>
-      <c r="C16" s="33" t="s">
+      <c r="C16" s="29" t="s">
         <v>123</v>
       </c>
       <c r="H16" t="s">
@@ -8847,7 +9576,7 @@
     </row>
     <row r="17" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B17" s="12"/>
-      <c r="C17" s="33"/>
+      <c r="C17" s="29"/>
       <c r="H17" t="s">
         <v>35</v>
       </c>
@@ -8865,7 +9594,7 @@
       <c r="B18" s="12" t="s">
         <v>128</v>
       </c>
-      <c r="C18" s="33" t="s">
+      <c r="C18" s="29" t="s">
         <v>122</v>
       </c>
       <c r="H18" t="s">
@@ -8885,7 +9614,7 @@
       <c r="B19" s="12" t="s">
         <v>131</v>
       </c>
-      <c r="C19" s="33" t="s">
+      <c r="C19" s="29" t="s">
         <v>122</v>
       </c>
       <c r="H19" t="s">
@@ -8905,7 +9634,7 @@
       <c r="B20" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="C20" s="33" t="s">
+      <c r="C20" s="29" t="s">
         <v>122</v>
       </c>
       <c r="H20" t="s">
@@ -8925,7 +9654,7 @@
       <c r="B21" s="12" t="s">
         <v>134</v>
       </c>
-      <c r="C21" s="33" t="s">
+      <c r="C21" s="29" t="s">
         <v>122</v>
       </c>
       <c r="H21" t="s">
@@ -8943,7 +9672,7 @@
     </row>
     <row r="22" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B22" s="12"/>
-      <c r="C22" s="33"/>
+      <c r="C22" s="29"/>
       <c r="H22" t="s">
         <v>62</v>
       </c>
@@ -8961,7 +9690,7 @@
       <c r="B23" s="12" t="s">
         <v>135</v>
       </c>
-      <c r="C23" s="33" t="s">
+      <c r="C23" s="29" t="s">
         <v>124</v>
       </c>
       <c r="H23" t="s">
@@ -8981,7 +9710,7 @@
       <c r="B24" s="12" t="s">
         <v>136</v>
       </c>
-      <c r="C24" s="33" t="s">
+      <c r="C24" s="29" t="s">
         <v>124</v>
       </c>
       <c r="H24" t="s">
@@ -9001,7 +9730,7 @@
       <c r="B25" s="12" t="s">
         <v>132</v>
       </c>
-      <c r="C25" s="33" t="s">
+      <c r="C25" s="29" t="s">
         <v>124</v>
       </c>
       <c r="H25" t="s">
@@ -9021,7 +9750,7 @@
       <c r="B26" s="14" t="s">
         <v>160</v>
       </c>
-      <c r="C26" s="34" t="s">
+      <c r="C26" s="30" t="s">
         <v>124</v>
       </c>
       <c r="H26" t="s">
@@ -9420,7 +10149,7 @@
       <c r="B10">
         <v>5</v>
       </c>
-      <c r="C10" s="37" t="s">
+      <c r="C10" s="33" t="s">
         <v>70</v>
       </c>
       <c r="E10">
@@ -9464,19 +10193,19 @@
       <c r="B11">
         <v>8</v>
       </c>
-      <c r="C11" s="37" t="s">
+      <c r="C11" s="33" t="s">
         <v>769</v>
       </c>
       <c r="E11">
         <v>8</v>
       </c>
-      <c r="F11" s="37" t="s">
+      <c r="F11" s="33" t="s">
         <v>770</v>
       </c>
       <c r="H11">
         <v>8</v>
       </c>
-      <c r="I11" s="37" t="s">
+      <c r="I11" s="33" t="s">
         <v>771</v>
       </c>
       <c r="K11">
@@ -9602,13 +10331,13 @@
       <c r="E14">
         <v>15</v>
       </c>
-      <c r="F14" s="39" t="s">
+      <c r="F14" s="35" t="s">
         <v>721</v>
       </c>
       <c r="H14">
         <v>15</v>
       </c>
-      <c r="I14" s="39" t="s">
+      <c r="I14" s="35" t="s">
         <v>721</v>
       </c>
       <c r="K14">
@@ -9811,7 +10540,7 @@
       </c>
     </row>
     <row r="36" spans="11:11" x14ac:dyDescent="0.25">
-      <c r="K36" s="38"/>
+      <c r="K36" s="34"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10051,7 +10780,7 @@
       <c r="E13">
         <v>14</v>
       </c>
-      <c r="F13" s="39" t="s">
+      <c r="F13" s="35" t="s">
         <v>720</v>
       </c>
       <c r="H13">
@@ -10821,7 +11550,7 @@
       <c r="E13">
         <v>14</v>
       </c>
-      <c r="F13" s="39" t="s">
+      <c r="F13" s="35" t="s">
         <v>735</v>
       </c>
       <c r="H13">

</xml_diff>